<commit_message>
UI Refactor: Streamline Auth UI and beautify email OTP template
</commit_message>
<xml_diff>
--- a/Project_Tracking.xlsx
+++ b/Project_Tracking.xlsx
@@ -1513,7 +1513,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="39">
+  <cellXfs count="40">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -1587,6 +1587,9 @@
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
@@ -2073,13 +2076,13 @@
     <col min="4" max="4" width="22" customWidth="1"/>
     <col min="5" max="5" width="60" customWidth="1"/>
     <col min="6" max="7" width="14" customWidth="1"/>
-    <col min="8" max="8" width="10" style="33" customWidth="1"/>
+    <col min="8" max="8" width="10" style="34" customWidth="1"/>
     <col min="9" max="9" width="14" customWidth="1"/>
     <col min="10" max="10" width="30" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" ht="40" customHeight="1" spans="1:10">
-      <c r="A1" s="34" t="s">
+      <c r="A1" s="35" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="8"/>
@@ -2088,7 +2091,7 @@
       <c r="E1" s="8"/>
       <c r="F1" s="8"/>
       <c r="G1" s="8"/>
-      <c r="H1" s="35"/>
+      <c r="H1" s="36"/>
       <c r="I1" s="8"/>
       <c r="J1" s="9"/>
     </row>
@@ -2102,7 +2105,7 @@
       <c r="E2" s="8"/>
       <c r="F2" s="8"/>
       <c r="G2" s="8"/>
-      <c r="H2" s="35"/>
+      <c r="H2" s="36"/>
       <c r="I2" s="8"/>
       <c r="J2" s="9"/>
     </row>
@@ -2138,26 +2141,26 @@
         <v>11</v>
       </c>
     </row>
-    <row r="4" s="32" customFormat="1" ht="28" customHeight="1" spans="1:10">
+    <row r="4" s="33" customFormat="1" ht="28" customHeight="1" spans="1:10">
       <c r="A4" s="26" t="s">
         <v>12</v>
       </c>
-      <c r="H4" s="36"/>
+      <c r="H4" s="37"/>
     </row>
     <row r="5" ht="45" customHeight="1" spans="1:10">
-      <c r="A5" s="37">
+      <c r="A5" s="38">
         <v>1</v>
       </c>
-      <c r="B5" s="37" t="s">
+      <c r="B5" s="38" t="s">
         <v>13</v>
       </c>
-      <c r="C5" s="37" t="s">
+      <c r="C5" s="38" t="s">
         <v>14</v>
       </c>
-      <c r="D5" s="37" t="s">
+      <c r="D5" s="38" t="s">
         <v>15</v>
       </c>
-      <c r="E5" s="37" t="s">
+      <c r="E5" s="38" t="s">
         <v>16</v>
       </c>
       <c r="F5" s="5" t="s">
@@ -2166,7 +2169,7 @@
       <c r="G5" s="5" t="s">
         <v>18</v>
       </c>
-      <c r="H5" s="38" t="s">
+      <c r="H5" s="39" t="s">
         <v>19</v>
       </c>
       <c r="I5" s="24"/>
@@ -2175,19 +2178,19 @@
       </c>
     </row>
     <row r="6" ht="45" customHeight="1" spans="1:10">
-      <c r="A6" s="37">
+      <c r="A6" s="38">
         <v>2</v>
       </c>
-      <c r="B6" s="37" t="s">
+      <c r="B6" s="38" t="s">
         <v>21</v>
       </c>
-      <c r="C6" s="37" t="s">
+      <c r="C6" s="38" t="s">
         <v>22</v>
       </c>
-      <c r="D6" s="37" t="s">
+      <c r="D6" s="38" t="s">
         <v>23</v>
       </c>
-      <c r="E6" s="37" t="s">
+      <c r="E6" s="38" t="s">
         <v>24</v>
       </c>
       <c r="F6" s="5" t="s">
@@ -2196,7 +2199,7 @@
       <c r="G6" s="5" t="s">
         <v>18</v>
       </c>
-      <c r="H6" s="38" t="s">
+      <c r="H6" s="39" t="s">
         <v>19</v>
       </c>
       <c r="I6" s="24"/>
@@ -2205,19 +2208,19 @@
       </c>
     </row>
     <row r="7" ht="45" customHeight="1" spans="1:10">
-      <c r="A7" s="37">
+      <c r="A7" s="38">
         <v>3</v>
       </c>
-      <c r="B7" s="37" t="s">
+      <c r="B7" s="38" t="s">
         <v>25</v>
       </c>
-      <c r="C7" s="37" t="s">
+      <c r="C7" s="38" t="s">
         <v>26</v>
       </c>
-      <c r="D7" s="37" t="s">
+      <c r="D7" s="38" t="s">
         <v>15</v>
       </c>
-      <c r="E7" s="37" t="s">
+      <c r="E7" s="38" t="s">
         <v>27</v>
       </c>
       <c r="F7" s="5" t="s">
@@ -2226,7 +2229,7 @@
       <c r="G7" s="5" t="s">
         <v>18</v>
       </c>
-      <c r="H7" s="38" t="s">
+      <c r="H7" s="39" t="s">
         <v>19</v>
       </c>
       <c r="I7" s="24"/>
@@ -2235,19 +2238,19 @@
       </c>
     </row>
     <row r="8" ht="45" customHeight="1" spans="1:10">
-      <c r="A8" s="37">
+      <c r="A8" s="38">
         <v>4</v>
       </c>
-      <c r="B8" s="37" t="s">
+      <c r="B8" s="38" t="s">
         <v>28</v>
       </c>
-      <c r="C8" s="37" t="s">
+      <c r="C8" s="38" t="s">
         <v>29</v>
       </c>
-      <c r="D8" s="37" t="s">
+      <c r="D8" s="38" t="s">
         <v>15</v>
       </c>
-      <c r="E8" s="37" t="s">
+      <c r="E8" s="38" t="s">
         <v>30</v>
       </c>
       <c r="F8" s="5" t="s">
@@ -2256,7 +2259,7 @@
       <c r="G8" s="5" t="s">
         <v>18</v>
       </c>
-      <c r="H8" s="38" t="s">
+      <c r="H8" s="39" t="s">
         <v>19</v>
       </c>
       <c r="I8" s="24"/>
@@ -2265,19 +2268,19 @@
       </c>
     </row>
     <row r="9" ht="45" customHeight="1" spans="1:10">
-      <c r="A9" s="37">
+      <c r="A9" s="38">
         <v>5</v>
       </c>
-      <c r="B9" s="37" t="s">
+      <c r="B9" s="38" t="s">
         <v>31</v>
       </c>
-      <c r="C9" s="37" t="s">
+      <c r="C9" s="38" t="s">
         <v>32</v>
       </c>
-      <c r="D9" s="37" t="s">
+      <c r="D9" s="38" t="s">
         <v>15</v>
       </c>
-      <c r="E9" s="37" t="s">
+      <c r="E9" s="38" t="s">
         <v>33</v>
       </c>
       <c r="F9" s="5" t="s">
@@ -2286,7 +2289,7 @@
       <c r="G9" s="5" t="s">
         <v>18</v>
       </c>
-      <c r="H9" s="38" t="s">
+      <c r="H9" s="39" t="s">
         <v>19</v>
       </c>
       <c r="I9" s="24"/>
@@ -2330,7 +2333,7 @@
       <c r="G11" s="5" t="s">
         <v>38</v>
       </c>
-      <c r="H11" s="38" t="s">
+      <c r="H11" s="39" t="s">
         <v>19</v>
       </c>
       <c r="I11" s="5" t="s">
@@ -2362,7 +2365,7 @@
       <c r="G12" s="5" t="s">
         <v>38</v>
       </c>
-      <c r="H12" s="38" t="s">
+      <c r="H12" s="39" t="s">
         <v>19</v>
       </c>
       <c r="I12" s="5" t="s">
@@ -2394,7 +2397,7 @@
       <c r="G13" s="5" t="s">
         <v>38</v>
       </c>
-      <c r="H13" s="38" t="s">
+      <c r="H13" s="39" t="s">
         <v>19</v>
       </c>
       <c r="I13" s="5" t="s">
@@ -2426,7 +2429,7 @@
       <c r="G14" s="5" t="s">
         <v>38</v>
       </c>
-      <c r="H14" s="38" t="s">
+      <c r="H14" s="39" t="s">
         <v>19</v>
       </c>
       <c r="I14" s="5" t="s">
@@ -2458,7 +2461,7 @@
       <c r="G15" s="5" t="s">
         <v>38</v>
       </c>
-      <c r="H15" s="38" t="s">
+      <c r="H15" s="39" t="s">
         <v>19</v>
       </c>
       <c r="I15" s="5" t="s">
@@ -2490,7 +2493,7 @@
       <c r="G16" s="5" t="s">
         <v>38</v>
       </c>
-      <c r="H16" s="38" t="s">
+      <c r="H16" s="39" t="s">
         <v>19</v>
       </c>
       <c r="I16" s="5" t="s">
@@ -2522,7 +2525,7 @@
       <c r="G17" s="5" t="s">
         <v>38</v>
       </c>
-      <c r="H17" s="38" t="s">
+      <c r="H17" s="39" t="s">
         <v>19</v>
       </c>
       <c r="I17" s="5" t="s">
@@ -2554,7 +2557,7 @@
       <c r="G18" s="5" t="s">
         <v>38</v>
       </c>
-      <c r="H18" s="38" t="s">
+      <c r="H18" s="39" t="s">
         <v>19</v>
       </c>
       <c r="I18" s="5" t="s">
@@ -2586,7 +2589,7 @@
       <c r="G19" s="5" t="s">
         <v>38</v>
       </c>
-      <c r="H19" s="38" t="s">
+      <c r="H19" s="39" t="s">
         <v>64</v>
       </c>
       <c r="I19" s="5" t="s">
@@ -2618,7 +2621,7 @@
       <c r="G20" s="5" t="s">
         <v>38</v>
       </c>
-      <c r="H20" s="38" t="s">
+      <c r="H20" s="39" t="s">
         <v>64</v>
       </c>
       <c r="I20" s="5" t="s">
@@ -2650,7 +2653,7 @@
       <c r="G21" s="5" t="s">
         <v>38</v>
       </c>
-      <c r="H21" s="38" t="s">
+      <c r="H21" s="39" t="s">
         <v>64</v>
       </c>
       <c r="I21" s="5" t="s">
@@ -2660,7 +2663,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="22" s="32" customFormat="1" ht="28" customHeight="1" spans="1:10">
+    <row r="22" s="33" customFormat="1" ht="28" customHeight="1" spans="1:10">
       <c r="A22" s="6">
         <v>17</v>
       </c>
@@ -2682,7 +2685,7 @@
       <c r="G22" s="5" t="s">
         <v>38</v>
       </c>
-      <c r="H22" s="38" t="s">
+      <c r="H22" s="39" t="s">
         <v>64</v>
       </c>
       <c r="I22" s="24" t="s">
@@ -2714,7 +2717,7 @@
       <c r="G23" s="5" t="s">
         <v>38</v>
       </c>
-      <c r="H23" s="38" t="s">
+      <c r="H23" s="39" t="s">
         <v>64</v>
       </c>
       <c r="I23" s="5" t="s">
@@ -2746,7 +2749,7 @@
       <c r="G24" s="5" t="s">
         <v>38</v>
       </c>
-      <c r="H24" s="38" t="s">
+      <c r="H24" s="39" t="s">
         <v>64</v>
       </c>
       <c r="I24" s="5" t="s">
@@ -2778,7 +2781,7 @@
       <c r="G25" s="5" t="s">
         <v>38</v>
       </c>
-      <c r="H25" s="38" t="s">
+      <c r="H25" s="39" t="s">
         <v>64</v>
       </c>
       <c r="I25" s="5" t="s">
@@ -2810,7 +2813,7 @@
       <c r="G26" s="5" t="s">
         <v>38</v>
       </c>
-      <c r="H26" s="38" t="s">
+      <c r="H26" s="39" t="s">
         <v>84</v>
       </c>
       <c r="I26" s="5" t="s">
@@ -2842,7 +2845,7 @@
       <c r="G27" s="5" t="s">
         <v>38</v>
       </c>
-      <c r="H27" s="38" t="s">
+      <c r="H27" s="39" t="s">
         <v>84</v>
       </c>
       <c r="I27" s="5" t="s">
@@ -2888,7 +2891,7 @@
       <c r="G29" s="5" t="s">
         <v>38</v>
       </c>
-      <c r="H29" s="38" t="s">
+      <c r="H29" s="39" t="s">
         <v>64</v>
       </c>
       <c r="I29" s="5" t="s">
@@ -2920,7 +2923,7 @@
       <c r="G30" s="5" t="s">
         <v>38</v>
       </c>
-      <c r="H30" s="38" t="s">
+      <c r="H30" s="39" t="s">
         <v>64</v>
       </c>
       <c r="I30" s="5" t="s">
@@ -2952,7 +2955,7 @@
       <c r="G31" s="5" t="s">
         <v>38</v>
       </c>
-      <c r="H31" s="38" t="s">
+      <c r="H31" s="39" t="s">
         <v>64</v>
       </c>
       <c r="I31" s="5" t="s">
@@ -2984,7 +2987,7 @@
       <c r="G32" s="5" t="s">
         <v>38</v>
       </c>
-      <c r="H32" s="38" t="s">
+      <c r="H32" s="39" t="s">
         <v>64</v>
       </c>
       <c r="I32" s="5" t="s">
@@ -3016,7 +3019,7 @@
       <c r="G33" s="5" t="s">
         <v>38</v>
       </c>
-      <c r="H33" s="38" t="s">
+      <c r="H33" s="39" t="s">
         <v>64</v>
       </c>
       <c r="I33" s="5" t="s">
@@ -3026,20 +3029,20 @@
         <v>20</v>
       </c>
     </row>
-    <row r="34" s="32" customFormat="1" ht="38" customHeight="1" spans="1:10">
+    <row r="34" s="33" customFormat="1" ht="38" customHeight="1" spans="1:10">
       <c r="A34" s="5">
         <v>28</v>
       </c>
       <c r="B34" s="5" t="s">
         <v>103</v>
       </c>
-      <c r="C34" s="37" t="s">
+      <c r="C34" s="38" t="s">
         <v>104</v>
       </c>
-      <c r="D34" s="37" t="s">
+      <c r="D34" s="38" t="s">
         <v>91</v>
       </c>
-      <c r="E34" s="37" t="s">
+      <c r="E34" s="38" t="s">
         <v>105</v>
       </c>
       <c r="F34" s="5" t="s">
@@ -3048,7 +3051,7 @@
       <c r="G34" s="5" t="s">
         <v>38</v>
       </c>
-      <c r="H34" s="38" t="s">
+      <c r="H34" s="39" t="s">
         <v>64</v>
       </c>
       <c r="I34" s="24" t="s">
@@ -3080,7 +3083,7 @@
       <c r="G35" s="5" t="s">
         <v>38</v>
       </c>
-      <c r="H35" s="38" t="s">
+      <c r="H35" s="39" t="s">
         <v>64</v>
       </c>
       <c r="I35" s="5" t="s">
@@ -3112,7 +3115,7 @@
       <c r="G36" s="5" t="s">
         <v>38</v>
       </c>
-      <c r="H36" s="38" t="s">
+      <c r="H36" s="39" t="s">
         <v>64</v>
       </c>
       <c r="I36" s="5" t="s">
@@ -3144,7 +3147,7 @@
       <c r="G37" s="5" t="s">
         <v>38</v>
       </c>
-      <c r="H37" s="38" t="s">
+      <c r="H37" s="39" t="s">
         <v>64</v>
       </c>
       <c r="I37" s="5" t="s">
@@ -3176,7 +3179,7 @@
       <c r="G38" s="5" t="s">
         <v>38</v>
       </c>
-      <c r="H38" s="38" t="s">
+      <c r="H38" s="39" t="s">
         <v>64</v>
       </c>
       <c r="I38" s="5" t="s">
@@ -3208,7 +3211,7 @@
       <c r="G39" s="5" t="s">
         <v>38</v>
       </c>
-      <c r="H39" s="38" t="s">
+      <c r="H39" s="39" t="s">
         <v>64</v>
       </c>
       <c r="I39" s="5" t="s">
@@ -3232,7 +3235,7 @@
       <c r="I40" s="22"/>
       <c r="J40" s="23"/>
     </row>
-    <row r="41" s="32" customFormat="1" ht="46" customHeight="1" spans="1:10">
+    <row r="41" s="33" customFormat="1" ht="46" customHeight="1" spans="1:10">
       <c r="A41" s="6">
         <v>34</v>
       </c>
@@ -3254,7 +3257,7 @@
       <c r="G41" s="5" t="s">
         <v>38</v>
       </c>
-      <c r="H41" s="38" t="s">
+      <c r="H41" s="39" t="s">
         <v>64</v>
       </c>
       <c r="I41" s="24" t="s">
@@ -3286,7 +3289,7 @@
       <c r="G42" s="5" t="s">
         <v>38</v>
       </c>
-      <c r="H42" s="38" t="s">
+      <c r="H42" s="39" t="s">
         <v>64</v>
       </c>
       <c r="I42" s="5" t="s">
@@ -3318,7 +3321,7 @@
       <c r="G43" s="5" t="s">
         <v>38</v>
       </c>
-      <c r="H43" s="38" t="s">
+      <c r="H43" s="39" t="s">
         <v>64</v>
       </c>
       <c r="I43" s="5" t="s">
@@ -3350,7 +3353,7 @@
       <c r="G44" s="5" t="s">
         <v>38</v>
       </c>
-      <c r="H44" s="38" t="s">
+      <c r="H44" s="39" t="s">
         <v>64</v>
       </c>
       <c r="I44" s="5" t="s">
@@ -3382,7 +3385,7 @@
       <c r="G45" s="5" t="s">
         <v>38</v>
       </c>
-      <c r="H45" s="38" t="s">
+      <c r="H45" s="39" t="s">
         <v>64</v>
       </c>
       <c r="I45" s="5" t="s">
@@ -3428,7 +3431,7 @@
       <c r="G47" s="5" t="s">
         <v>38</v>
       </c>
-      <c r="H47" s="38" t="s">
+      <c r="H47" s="39" t="s">
         <v>64</v>
       </c>
       <c r="I47" s="5" t="s">
@@ -3460,7 +3463,7 @@
       <c r="G48" s="5" t="s">
         <v>38</v>
       </c>
-      <c r="H48" s="38" t="s">
+      <c r="H48" s="39" t="s">
         <v>64</v>
       </c>
       <c r="I48" s="5" t="s">
@@ -3492,7 +3495,7 @@
       <c r="G49" s="5" t="s">
         <v>38</v>
       </c>
-      <c r="H49" s="38" t="s">
+      <c r="H49" s="39" t="s">
         <v>64</v>
       </c>
       <c r="I49" s="5" t="s">
@@ -3502,20 +3505,20 @@
         <v>20</v>
       </c>
     </row>
-    <row r="50" s="32" customFormat="1" ht="28" customHeight="1" spans="1:10">
+    <row r="50" s="33" customFormat="1" ht="28" customHeight="1" spans="1:10">
       <c r="A50" s="5">
         <v>42</v>
       </c>
-      <c r="B50" s="37" t="s">
+      <c r="B50" s="38" t="s">
         <v>147</v>
       </c>
-      <c r="C50" s="37" t="s">
+      <c r="C50" s="38" t="s">
         <v>148</v>
       </c>
-      <c r="D50" s="37" t="s">
+      <c r="D50" s="38" t="s">
         <v>139</v>
       </c>
-      <c r="E50" s="37" t="s">
+      <c r="E50" s="38" t="s">
         <v>149</v>
       </c>
       <c r="F50" s="5" t="s">
@@ -3524,7 +3527,7 @@
       <c r="G50" s="5" t="s">
         <v>38</v>
       </c>
-      <c r="H50" s="38" t="s">
+      <c r="H50" s="39" t="s">
         <v>64</v>
       </c>
       <c r="I50" s="24" t="s">
@@ -3556,7 +3559,7 @@
       <c r="G51" s="5" t="s">
         <v>38</v>
       </c>
-      <c r="H51" s="38" t="s">
+      <c r="H51" s="39" t="s">
         <v>64</v>
       </c>
       <c r="I51" s="5" t="s">
@@ -3588,7 +3591,7 @@
       <c r="G52" s="5" t="s">
         <v>38</v>
       </c>
-      <c r="H52" s="38" t="s">
+      <c r="H52" s="39" t="s">
         <v>84</v>
       </c>
       <c r="I52" s="5" t="s">
@@ -3620,7 +3623,7 @@
       <c r="G53" s="5" t="s">
         <v>38</v>
       </c>
-      <c r="H53" s="38" t="s">
+      <c r="H53" s="39" t="s">
         <v>64</v>
       </c>
       <c r="I53" s="5" t="s">
@@ -3652,7 +3655,7 @@
       <c r="G54" s="5" t="s">
         <v>38</v>
       </c>
-      <c r="H54" s="38" t="s">
+      <c r="H54" s="39" t="s">
         <v>84</v>
       </c>
       <c r="I54" s="5" t="s">
@@ -3698,7 +3701,7 @@
       <c r="G56" s="5" t="s">
         <v>38</v>
       </c>
-      <c r="H56" s="38" t="s">
+      <c r="H56" s="39" t="s">
         <v>84</v>
       </c>
       <c r="I56" s="5" t="s">
@@ -3730,7 +3733,7 @@
       <c r="G57" s="5" t="s">
         <v>38</v>
       </c>
-      <c r="H57" s="38" t="s">
+      <c r="H57" s="39" t="s">
         <v>84</v>
       </c>
       <c r="I57" s="5" t="s">
@@ -3762,7 +3765,7 @@
       <c r="G58" s="5" t="s">
         <v>38</v>
       </c>
-      <c r="H58" s="38" t="s">
+      <c r="H58" s="39" t="s">
         <v>84</v>
       </c>
       <c r="I58" s="5" t="s">
@@ -3794,7 +3797,7 @@
       <c r="G59" s="5" t="s">
         <v>38</v>
       </c>
-      <c r="H59" s="38" t="s">
+      <c r="H59" s="39" t="s">
         <v>84</v>
       </c>
       <c r="I59" s="5" t="s">
@@ -3826,7 +3829,7 @@
       <c r="G60" s="5" t="s">
         <v>38</v>
       </c>
-      <c r="H60" s="38" t="s">
+      <c r="H60" s="39" t="s">
         <v>84</v>
       </c>
       <c r="I60" s="5" t="s">
@@ -3858,7 +3861,7 @@
       <c r="G61" s="5" t="s">
         <v>38</v>
       </c>
-      <c r="H61" s="38" t="s">
+      <c r="H61" s="39" t="s">
         <v>84</v>
       </c>
       <c r="I61" s="5" t="s">
@@ -3973,13 +3976,13 @@
       <c r="F5" s="27" t="s">
         <v>18</v>
       </c>
-      <c r="G5" s="24" t="s">
-        <v>20</v>
-      </c>
-      <c r="H5" s="24" t="s">
-        <v>20</v>
-      </c>
-      <c r="I5" s="28" t="s">
+      <c r="G5" s="28" t="s">
+        <v>20</v>
+      </c>
+      <c r="H5" s="28" t="s">
+        <v>20</v>
+      </c>
+      <c r="I5" s="29" t="s">
         <v>187</v>
       </c>
     </row>
@@ -4002,13 +4005,13 @@
       <c r="F6" s="27" t="s">
         <v>18</v>
       </c>
-      <c r="G6" s="24" t="s">
-        <v>20</v>
-      </c>
-      <c r="H6" s="24" t="s">
-        <v>20</v>
-      </c>
-      <c r="I6" s="28" t="s">
+      <c r="G6" s="28" t="s">
+        <v>20</v>
+      </c>
+      <c r="H6" s="28" t="s">
+        <v>20</v>
+      </c>
+      <c r="I6" s="29" t="s">
         <v>188</v>
       </c>
     </row>
@@ -4031,13 +4034,13 @@
       <c r="F7" s="27" t="s">
         <v>18</v>
       </c>
-      <c r="G7" s="24" t="s">
-        <v>20</v>
-      </c>
-      <c r="H7" s="24" t="s">
-        <v>20</v>
-      </c>
-      <c r="I7" s="28" t="s">
+      <c r="G7" s="28" t="s">
+        <v>20</v>
+      </c>
+      <c r="H7" s="28" t="s">
+        <v>20</v>
+      </c>
+      <c r="I7" s="29" t="s">
         <v>189</v>
       </c>
     </row>
@@ -4060,13 +4063,13 @@
       <c r="F8" s="27" t="s">
         <v>18</v>
       </c>
-      <c r="G8" s="24" t="s">
-        <v>20</v>
-      </c>
-      <c r="H8" s="24" t="s">
-        <v>20</v>
-      </c>
-      <c r="I8" s="28" t="s">
+      <c r="G8" s="28" t="s">
+        <v>20</v>
+      </c>
+      <c r="H8" s="28" t="s">
+        <v>20</v>
+      </c>
+      <c r="I8" s="29" t="s">
         <v>190</v>
       </c>
     </row>
@@ -4089,13 +4092,13 @@
       <c r="F9" s="27" t="s">
         <v>18</v>
       </c>
-      <c r="G9" s="24" t="s">
-        <v>20</v>
-      </c>
-      <c r="H9" s="24" t="s">
-        <v>20</v>
-      </c>
-      <c r="I9" s="28" t="s">
+      <c r="G9" s="28" t="s">
+        <v>20</v>
+      </c>
+      <c r="H9" s="28" t="s">
+        <v>20</v>
+      </c>
+      <c r="I9" s="29" t="s">
         <v>193</v>
       </c>
     </row>
@@ -4107,10 +4110,10 @@
       <c r="C10" s="22"/>
       <c r="D10" s="22"/>
       <c r="E10" s="22"/>
-      <c r="F10" s="29"/>
+      <c r="F10" s="30"/>
       <c r="G10" s="22"/>
       <c r="H10" s="22"/>
-      <c r="I10" s="30"/>
+      <c r="I10" s="31"/>
     </row>
     <row r="11" ht="45" customHeight="1" spans="1:9">
       <c r="A11" s="5">
@@ -4137,7 +4140,7 @@
       <c r="H11" s="5" t="s">
         <v>20</v>
       </c>
-      <c r="I11" s="31" t="s">
+      <c r="I11" s="32" t="s">
         <v>195</v>
       </c>
     </row>
@@ -4166,7 +4169,7 @@
       <c r="H12" s="5" t="s">
         <v>20</v>
       </c>
-      <c r="I12" s="31" t="s">
+      <c r="I12" s="32" t="s">
         <v>196</v>
       </c>
     </row>
@@ -4195,7 +4198,7 @@
       <c r="H13" s="5" t="s">
         <v>20</v>
       </c>
-      <c r="I13" s="31" t="s">
+      <c r="I13" s="32" t="s">
         <v>197</v>
       </c>
     </row>
@@ -4224,7 +4227,7 @@
       <c r="H14" s="5" t="s">
         <v>20</v>
       </c>
-      <c r="I14" s="31" t="s">
+      <c r="I14" s="32" t="s">
         <v>198</v>
       </c>
     </row>
@@ -4253,7 +4256,7 @@
       <c r="H15" s="5" t="s">
         <v>20</v>
       </c>
-      <c r="I15" s="31" t="s">
+      <c r="I15" s="32" t="s">
         <v>200</v>
       </c>
     </row>
@@ -4282,7 +4285,7 @@
       <c r="H16" s="5" t="s">
         <v>20</v>
       </c>
-      <c r="I16" s="31" t="s">
+      <c r="I16" s="32" t="s">
         <v>201</v>
       </c>
     </row>
@@ -4311,7 +4314,7 @@
       <c r="H17" s="5" t="s">
         <v>20</v>
       </c>
-      <c r="I17" s="31" t="s">
+      <c r="I17" s="32" t="s">
         <v>202</v>
       </c>
     </row>
@@ -4340,7 +4343,7 @@
       <c r="H18" s="5" t="s">
         <v>20</v>
       </c>
-      <c r="I18" s="31" t="s">
+      <c r="I18" s="32" t="s">
         <v>203</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Update Project_Tracking, Auth tests and UI adjustments
</commit_message>
<xml_diff>
--- a/Project_Tracking.xlsx
+++ b/Project_Tracking.xlsx
@@ -147,82 +147,82 @@
     <t>Sinh viên có thể cập nhật thông tin cá nhân: họ tên, SĐT, email, ảnh đại diện, địa chỉ.</t>
   </si>
   <si>
+    <t>Trạm dừng</t>
+  </si>
+  <si>
+    <t>Xem danh sách trạm dừng</t>
+  </si>
+  <si>
+    <t>Hiển thị danh sách các trạm dừng trên bản đồ và dạng list, bao gồm tên trạm, vị trí, tuyến đi qua.</t>
+  </si>
+  <si>
+    <t>Tìm tuyến xe</t>
+  </si>
+  <si>
+    <t>Tìm tuyến xe phù hợp</t>
+  </si>
+  <si>
+    <t>Sinh viên nhập điểm đi - điểm đến, hệ thống gợi ý tuyến xe phù hợp nhất.</t>
+  </si>
+  <si>
+    <t>Thời gian xe đến</t>
+  </si>
+  <si>
+    <t>Xem thời gian xe đến</t>
+  </si>
+  <si>
+    <t>Hiển thị thời gian dự kiến xe đến trạm dừng mà sinh viên chọn (ETA).</t>
+  </si>
+  <si>
+    <t>Theo dõi xe</t>
+  </si>
+  <si>
+    <t>Theo dõi vị trí xe theo thời gian thực</t>
+  </si>
+  <si>
+    <t>Hiển thị vị trí xe trên bản đồ realtime bằng GPS, cập nhật liên tục.</t>
+  </si>
+  <si>
+    <t>Nguyễn Tấn Phú</t>
+  </si>
+  <si>
+    <t>Đăng ký tuyến xe</t>
+  </si>
+  <si>
+    <t>Đăng ký sử dụng tuyến xe</t>
+  </si>
+  <si>
+    <t>Sinh viên chọn tuyến xe và đăng ký sử dụng, hệ thống xác nhận và lưu thông tin.</t>
+  </si>
+  <si>
+    <t>Quản lý tuyến xe</t>
+  </si>
+  <si>
+    <t>Đổi tuyến xe / Hủy tuyến xe</t>
+  </si>
+  <si>
+    <t>Sinh viên có thể đổi sang tuyến khác hoặc hủy đăng ký tuyến xe hiện tại.</t>
+  </si>
+  <si>
+    <t>Lịch sử chuyến đi</t>
+  </si>
+  <si>
+    <t>Xem lịch sử chuyến đi</t>
+  </si>
+  <si>
+    <t>Hiển thị danh sách các chuyến đi đã thực hiện, bao gồm ngày, tuyến, giờ lên/xuống xe.</t>
+  </si>
+  <si>
+    <t>Thông báo</t>
+  </si>
+  <si>
+    <t>Nhận thông báo</t>
+  </si>
+  <si>
+    <t>Sinh viên nhận thông báo từ hệ thống: thay đổi lịch trình, tuyến, thông tin khẩn cấp.</t>
+  </si>
+  <si>
     <t>Not Started</t>
-  </si>
-  <si>
-    <t>Trạm dừng</t>
-  </si>
-  <si>
-    <t>Xem danh sách trạm dừng</t>
-  </si>
-  <si>
-    <t>Hiển thị danh sách các trạm dừng trên bản đồ và dạng list, bao gồm tên trạm, vị trí, tuyến đi qua.</t>
-  </si>
-  <si>
-    <t>Tìm tuyến xe</t>
-  </si>
-  <si>
-    <t>Tìm tuyến xe phù hợp</t>
-  </si>
-  <si>
-    <t>Sinh viên nhập điểm đi - điểm đến, hệ thống gợi ý tuyến xe phù hợp nhất.</t>
-  </si>
-  <si>
-    <t>Thời gian xe đến</t>
-  </si>
-  <si>
-    <t>Xem thời gian xe đến</t>
-  </si>
-  <si>
-    <t>Hiển thị thời gian dự kiến xe đến trạm dừng mà sinh viên chọn (ETA).</t>
-  </si>
-  <si>
-    <t>Theo dõi xe</t>
-  </si>
-  <si>
-    <t>Theo dõi vị trí xe theo thời gian thực</t>
-  </si>
-  <si>
-    <t>Hiển thị vị trí xe trên bản đồ realtime bằng GPS, cập nhật liên tục.</t>
-  </si>
-  <si>
-    <t>Nguyễn Tấn Phú</t>
-  </si>
-  <si>
-    <t>Đăng ký tuyến xe</t>
-  </si>
-  <si>
-    <t>Đăng ký sử dụng tuyến xe</t>
-  </si>
-  <si>
-    <t>Sinh viên chọn tuyến xe và đăng ký sử dụng, hệ thống xác nhận và lưu thông tin.</t>
-  </si>
-  <si>
-    <t>Quản lý tuyến xe</t>
-  </si>
-  <si>
-    <t>Đổi tuyến xe / Hủy tuyến xe</t>
-  </si>
-  <si>
-    <t>Sinh viên có thể đổi sang tuyến khác hoặc hủy đăng ký tuyến xe hiện tại.</t>
-  </si>
-  <si>
-    <t>Lịch sử chuyến đi</t>
-  </si>
-  <si>
-    <t>Xem lịch sử chuyến đi</t>
-  </si>
-  <si>
-    <t>Hiển thị danh sách các chuyến đi đã thực hiện, bao gồm ngày, tuyến, giờ lên/xuống xe.</t>
-  </si>
-  <si>
-    <t>Thông báo</t>
-  </si>
-  <si>
-    <t>Nhận thông báo</t>
-  </si>
-  <si>
-    <t>Sinh viên nhận thông báo từ hệ thống: thay đổi lịch trình, tuyến, thông tin khẩn cấp.</t>
   </si>
   <si>
     <t>iter2</t>
@@ -2331,7 +2331,7 @@
         <v>17</v>
       </c>
       <c r="G11" s="5" t="s">
-        <v>38</v>
+        <v>18</v>
       </c>
       <c r="H11" s="39" t="s">
         <v>19</v>
@@ -2348,22 +2348,22 @@
         <v>7</v>
       </c>
       <c r="B12" s="6" t="s">
+        <v>38</v>
+      </c>
+      <c r="C12" s="6" t="s">
         <v>39</v>
-      </c>
-      <c r="C12" s="6" t="s">
-        <v>40</v>
       </c>
       <c r="D12" s="6" t="s">
         <v>23</v>
       </c>
       <c r="E12" s="6" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="F12" s="5" t="s">
         <v>17</v>
       </c>
       <c r="G12" s="5" t="s">
-        <v>38</v>
+        <v>18</v>
       </c>
       <c r="H12" s="39" t="s">
         <v>19</v>
@@ -2380,22 +2380,22 @@
         <v>8</v>
       </c>
       <c r="B13" s="6" t="s">
+        <v>41</v>
+      </c>
+      <c r="C13" s="6" t="s">
         <v>42</v>
-      </c>
-      <c r="C13" s="6" t="s">
-        <v>43</v>
       </c>
       <c r="D13" s="6" t="s">
         <v>23</v>
       </c>
       <c r="E13" s="6" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="F13" s="5" t="s">
         <v>17</v>
       </c>
       <c r="G13" s="5" t="s">
-        <v>38</v>
+        <v>18</v>
       </c>
       <c r="H13" s="39" t="s">
         <v>19</v>
@@ -2412,22 +2412,22 @@
         <v>9</v>
       </c>
       <c r="B14" s="6" t="s">
+        <v>44</v>
+      </c>
+      <c r="C14" s="6" t="s">
         <v>45</v>
-      </c>
-      <c r="C14" s="6" t="s">
-        <v>46</v>
       </c>
       <c r="D14" s="6" t="s">
         <v>23</v>
       </c>
       <c r="E14" s="6" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="F14" s="5" t="s">
         <v>17</v>
       </c>
       <c r="G14" s="5" t="s">
-        <v>38</v>
+        <v>18</v>
       </c>
       <c r="H14" s="39" t="s">
         <v>19</v>
@@ -2444,22 +2444,22 @@
         <v>10</v>
       </c>
       <c r="B15" s="6" t="s">
+        <v>47</v>
+      </c>
+      <c r="C15" s="6" t="s">
         <v>48</v>
-      </c>
-      <c r="C15" s="6" t="s">
-        <v>49</v>
       </c>
       <c r="D15" s="6" t="s">
         <v>23</v>
       </c>
       <c r="E15" s="6" t="s">
+        <v>49</v>
+      </c>
+      <c r="F15" s="5" t="s">
         <v>50</v>
       </c>
-      <c r="F15" s="5" t="s">
-        <v>51</v>
-      </c>
       <c r="G15" s="5" t="s">
-        <v>38</v>
+        <v>18</v>
       </c>
       <c r="H15" s="39" t="s">
         <v>19</v>
@@ -2476,22 +2476,22 @@
         <v>11</v>
       </c>
       <c r="B16" s="6" t="s">
+        <v>51</v>
+      </c>
+      <c r="C16" s="6" t="s">
         <v>52</v>
-      </c>
-      <c r="C16" s="6" t="s">
-        <v>53</v>
       </c>
       <c r="D16" s="6" t="s">
         <v>23</v>
       </c>
       <c r="E16" s="6" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="F16" s="5" t="s">
         <v>17</v>
       </c>
       <c r="G16" s="5" t="s">
-        <v>38</v>
+        <v>18</v>
       </c>
       <c r="H16" s="39" t="s">
         <v>19</v>
@@ -2508,22 +2508,22 @@
         <v>12</v>
       </c>
       <c r="B17" s="6" t="s">
+        <v>54</v>
+      </c>
+      <c r="C17" s="6" t="s">
         <v>55</v>
-      </c>
-      <c r="C17" s="6" t="s">
-        <v>56</v>
       </c>
       <c r="D17" s="6" t="s">
         <v>23</v>
       </c>
       <c r="E17" s="6" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="F17" s="5" t="s">
         <v>17</v>
       </c>
       <c r="G17" s="5" t="s">
-        <v>38</v>
+        <v>18</v>
       </c>
       <c r="H17" s="39" t="s">
         <v>19</v>
@@ -2540,22 +2540,22 @@
         <v>13</v>
       </c>
       <c r="B18" s="6" t="s">
+        <v>57</v>
+      </c>
+      <c r="C18" s="6" t="s">
         <v>58</v>
-      </c>
-      <c r="C18" s="6" t="s">
-        <v>59</v>
       </c>
       <c r="D18" s="6" t="s">
         <v>23</v>
       </c>
       <c r="E18" s="6" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="F18" s="5" t="s">
         <v>17</v>
       </c>
       <c r="G18" s="5" t="s">
-        <v>38</v>
+        <v>18</v>
       </c>
       <c r="H18" s="39" t="s">
         <v>19</v>
@@ -2572,22 +2572,22 @@
         <v>14</v>
       </c>
       <c r="B19" s="6" t="s">
+        <v>60</v>
+      </c>
+      <c r="C19" s="6" t="s">
         <v>61</v>
-      </c>
-      <c r="C19" s="6" t="s">
-        <v>62</v>
       </c>
       <c r="D19" s="6" t="s">
         <v>23</v>
       </c>
       <c r="E19" s="6" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="F19" s="5" t="s">
         <v>17</v>
       </c>
       <c r="G19" s="5" t="s">
-        <v>38</v>
+        <v>63</v>
       </c>
       <c r="H19" s="39" t="s">
         <v>64</v>
@@ -2619,7 +2619,7 @@
         <v>17</v>
       </c>
       <c r="G20" s="5" t="s">
-        <v>38</v>
+        <v>63</v>
       </c>
       <c r="H20" s="39" t="s">
         <v>64</v>
@@ -2648,10 +2648,10 @@
         <v>69</v>
       </c>
       <c r="F21" s="5" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="G21" s="5" t="s">
-        <v>38</v>
+        <v>63</v>
       </c>
       <c r="H21" s="39" t="s">
         <v>64</v>
@@ -2680,10 +2680,10 @@
         <v>72</v>
       </c>
       <c r="F22" s="5" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="G22" s="5" t="s">
-        <v>38</v>
+        <v>63</v>
       </c>
       <c r="H22" s="39" t="s">
         <v>64</v>
@@ -2712,10 +2712,10 @@
         <v>75</v>
       </c>
       <c r="F23" s="5" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="G23" s="5" t="s">
-        <v>38</v>
+        <v>63</v>
       </c>
       <c r="H23" s="39" t="s">
         <v>64</v>
@@ -2744,10 +2744,10 @@
         <v>78</v>
       </c>
       <c r="F24" s="5" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="G24" s="5" t="s">
-        <v>38</v>
+        <v>63</v>
       </c>
       <c r="H24" s="39" t="s">
         <v>64</v>
@@ -2776,10 +2776,10 @@
         <v>80</v>
       </c>
       <c r="F25" s="5" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="G25" s="5" t="s">
-        <v>38</v>
+        <v>63</v>
       </c>
       <c r="H25" s="39" t="s">
         <v>64</v>
@@ -2808,10 +2808,10 @@
         <v>83</v>
       </c>
       <c r="F26" s="5" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="G26" s="5" t="s">
-        <v>38</v>
+        <v>63</v>
       </c>
       <c r="H26" s="39" t="s">
         <v>84</v>
@@ -2840,10 +2840,10 @@
         <v>87</v>
       </c>
       <c r="F27" s="5" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="G27" s="5" t="s">
-        <v>38</v>
+        <v>63</v>
       </c>
       <c r="H27" s="39" t="s">
         <v>84</v>
@@ -2889,7 +2889,7 @@
         <v>93</v>
       </c>
       <c r="G29" s="5" t="s">
-        <v>38</v>
+        <v>63</v>
       </c>
       <c r="H29" s="39" t="s">
         <v>64</v>
@@ -2921,7 +2921,7 @@
         <v>93</v>
       </c>
       <c r="G30" s="5" t="s">
-        <v>38</v>
+        <v>63</v>
       </c>
       <c r="H30" s="39" t="s">
         <v>64</v>
@@ -2953,7 +2953,7 @@
         <v>93</v>
       </c>
       <c r="G31" s="5" t="s">
-        <v>38</v>
+        <v>63</v>
       </c>
       <c r="H31" s="39" t="s">
         <v>64</v>
@@ -2985,7 +2985,7 @@
         <v>93</v>
       </c>
       <c r="G32" s="5" t="s">
-        <v>38</v>
+        <v>63</v>
       </c>
       <c r="H32" s="39" t="s">
         <v>64</v>
@@ -3017,7 +3017,7 @@
         <v>93</v>
       </c>
       <c r="G33" s="5" t="s">
-        <v>38</v>
+        <v>63</v>
       </c>
       <c r="H33" s="39" t="s">
         <v>64</v>
@@ -3049,7 +3049,7 @@
         <v>93</v>
       </c>
       <c r="G34" s="5" t="s">
-        <v>38</v>
+        <v>63</v>
       </c>
       <c r="H34" s="39" t="s">
         <v>64</v>
@@ -3081,7 +3081,7 @@
         <v>93</v>
       </c>
       <c r="G35" s="5" t="s">
-        <v>38</v>
+        <v>63</v>
       </c>
       <c r="H35" s="39" t="s">
         <v>64</v>
@@ -3113,7 +3113,7 @@
         <v>93</v>
       </c>
       <c r="G36" s="5" t="s">
-        <v>38</v>
+        <v>63</v>
       </c>
       <c r="H36" s="39" t="s">
         <v>64</v>
@@ -3145,7 +3145,7 @@
         <v>93</v>
       </c>
       <c r="G37" s="5" t="s">
-        <v>38</v>
+        <v>63</v>
       </c>
       <c r="H37" s="39" t="s">
         <v>64</v>
@@ -3177,7 +3177,7 @@
         <v>93</v>
       </c>
       <c r="G38" s="5" t="s">
-        <v>38</v>
+        <v>63</v>
       </c>
       <c r="H38" s="39" t="s">
         <v>64</v>
@@ -3197,7 +3197,7 @@
         <v>116</v>
       </c>
       <c r="C39" s="6" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="D39" s="6" t="s">
         <v>91</v>
@@ -3209,7 +3209,7 @@
         <v>93</v>
       </c>
       <c r="G39" s="5" t="s">
-        <v>38</v>
+        <v>63</v>
       </c>
       <c r="H39" s="39" t="s">
         <v>64</v>
@@ -3255,7 +3255,7 @@
         <v>123</v>
       </c>
       <c r="G41" s="5" t="s">
-        <v>38</v>
+        <v>63</v>
       </c>
       <c r="H41" s="39" t="s">
         <v>64</v>
@@ -3287,7 +3287,7 @@
         <v>123</v>
       </c>
       <c r="G42" s="5" t="s">
-        <v>38</v>
+        <v>63</v>
       </c>
       <c r="H42" s="39" t="s">
         <v>64</v>
@@ -3319,7 +3319,7 @@
         <v>123</v>
       </c>
       <c r="G43" s="5" t="s">
-        <v>38</v>
+        <v>63</v>
       </c>
       <c r="H43" s="39" t="s">
         <v>64</v>
@@ -3351,7 +3351,7 @@
         <v>123</v>
       </c>
       <c r="G44" s="5" t="s">
-        <v>38</v>
+        <v>63</v>
       </c>
       <c r="H44" s="39" t="s">
         <v>64</v>
@@ -3383,7 +3383,7 @@
         <v>123</v>
       </c>
       <c r="G45" s="5" t="s">
-        <v>38</v>
+        <v>63</v>
       </c>
       <c r="H45" s="39" t="s">
         <v>64</v>
@@ -3429,7 +3429,7 @@
         <v>141</v>
       </c>
       <c r="G47" s="5" t="s">
-        <v>38</v>
+        <v>63</v>
       </c>
       <c r="H47" s="39" t="s">
         <v>64</v>
@@ -3461,7 +3461,7 @@
         <v>141</v>
       </c>
       <c r="G48" s="5" t="s">
-        <v>38</v>
+        <v>63</v>
       </c>
       <c r="H48" s="39" t="s">
         <v>64</v>
@@ -3493,7 +3493,7 @@
         <v>141</v>
       </c>
       <c r="G49" s="5" t="s">
-        <v>38</v>
+        <v>63</v>
       </c>
       <c r="H49" s="39" t="s">
         <v>64</v>
@@ -3525,7 +3525,7 @@
         <v>141</v>
       </c>
       <c r="G50" s="5" t="s">
-        <v>38</v>
+        <v>63</v>
       </c>
       <c r="H50" s="39" t="s">
         <v>64</v>
@@ -3557,7 +3557,7 @@
         <v>141</v>
       </c>
       <c r="G51" s="5" t="s">
-        <v>38</v>
+        <v>63</v>
       </c>
       <c r="H51" s="39" t="s">
         <v>64</v>
@@ -3589,7 +3589,7 @@
         <v>141</v>
       </c>
       <c r="G52" s="5" t="s">
-        <v>38</v>
+        <v>63</v>
       </c>
       <c r="H52" s="39" t="s">
         <v>84</v>
@@ -3621,7 +3621,7 @@
         <v>141</v>
       </c>
       <c r="G53" s="5" t="s">
-        <v>38</v>
+        <v>63</v>
       </c>
       <c r="H53" s="39" t="s">
         <v>64</v>
@@ -3653,7 +3653,7 @@
         <v>141</v>
       </c>
       <c r="G54" s="5" t="s">
-        <v>38</v>
+        <v>63</v>
       </c>
       <c r="H54" s="39" t="s">
         <v>84</v>
@@ -3699,7 +3699,7 @@
         <v>123</v>
       </c>
       <c r="G56" s="5" t="s">
-        <v>38</v>
+        <v>63</v>
       </c>
       <c r="H56" s="39" t="s">
         <v>84</v>
@@ -3731,7 +3731,7 @@
         <v>123</v>
       </c>
       <c r="G57" s="5" t="s">
-        <v>38</v>
+        <v>63</v>
       </c>
       <c r="H57" s="39" t="s">
         <v>84</v>
@@ -3763,7 +3763,7 @@
         <v>123</v>
       </c>
       <c r="G58" s="5" t="s">
-        <v>38</v>
+        <v>63</v>
       </c>
       <c r="H58" s="39" t="s">
         <v>84</v>
@@ -3795,7 +3795,7 @@
         <v>123</v>
       </c>
       <c r="G59" s="5" t="s">
-        <v>38</v>
+        <v>63</v>
       </c>
       <c r="H59" s="39" t="s">
         <v>84</v>
@@ -3827,7 +3827,7 @@
         <v>123</v>
       </c>
       <c r="G60" s="5" t="s">
-        <v>38</v>
+        <v>63</v>
       </c>
       <c r="H60" s="39" t="s">
         <v>84</v>
@@ -3859,7 +3859,7 @@
         <v>123</v>
       </c>
       <c r="G61" s="5" t="s">
-        <v>38</v>
+        <v>63</v>
       </c>
       <c r="H61" s="39" t="s">
         <v>84</v>
@@ -4149,13 +4149,13 @@
         <v>7</v>
       </c>
       <c r="B12" s="6" t="s">
+        <v>38</v>
+      </c>
+      <c r="C12" s="6" t="s">
         <v>39</v>
       </c>
-      <c r="C12" s="6" t="s">
+      <c r="D12" s="24" t="s">
         <v>40</v>
-      </c>
-      <c r="D12" s="24" t="s">
-        <v>41</v>
       </c>
       <c r="E12" s="5" t="s">
         <v>17</v>
@@ -4178,13 +4178,13 @@
         <v>8</v>
       </c>
       <c r="B13" s="6" t="s">
+        <v>41</v>
+      </c>
+      <c r="C13" s="6" t="s">
         <v>42</v>
       </c>
-      <c r="C13" s="6" t="s">
+      <c r="D13" s="6" t="s">
         <v>43</v>
-      </c>
-      <c r="D13" s="6" t="s">
-        <v>44</v>
       </c>
       <c r="E13" s="5" t="s">
         <v>17</v>
@@ -4207,13 +4207,13 @@
         <v>9</v>
       </c>
       <c r="B14" s="6" t="s">
+        <v>44</v>
+      </c>
+      <c r="C14" s="6" t="s">
         <v>45</v>
       </c>
-      <c r="C14" s="6" t="s">
+      <c r="D14" s="6" t="s">
         <v>46</v>
-      </c>
-      <c r="D14" s="6" t="s">
-        <v>47</v>
       </c>
       <c r="E14" s="5" t="s">
         <v>17</v>
@@ -4236,16 +4236,16 @@
         <v>10</v>
       </c>
       <c r="B15" s="6" t="s">
+        <v>47</v>
+      </c>
+      <c r="C15" s="6" t="s">
         <v>48</v>
       </c>
-      <c r="C15" s="6" t="s">
+      <c r="D15" s="6" t="s">
         <v>49</v>
       </c>
-      <c r="D15" s="6" t="s">
+      <c r="E15" s="5" t="s">
         <v>50</v>
-      </c>
-      <c r="E15" s="5" t="s">
-        <v>51</v>
       </c>
       <c r="F15" s="27" t="s">
         <v>199</v>
@@ -4265,13 +4265,13 @@
         <v>11</v>
       </c>
       <c r="B16" s="6" t="s">
+        <v>51</v>
+      </c>
+      <c r="C16" s="6" t="s">
         <v>52</v>
       </c>
-      <c r="C16" s="6" t="s">
+      <c r="D16" s="6" t="s">
         <v>53</v>
-      </c>
-      <c r="D16" s="6" t="s">
-        <v>54</v>
       </c>
       <c r="E16" s="5" t="s">
         <v>17</v>
@@ -4294,13 +4294,13 @@
         <v>12</v>
       </c>
       <c r="B17" s="6" t="s">
+        <v>54</v>
+      </c>
+      <c r="C17" s="6" t="s">
         <v>55</v>
       </c>
-      <c r="C17" s="6" t="s">
+      <c r="D17" s="6" t="s">
         <v>56</v>
-      </c>
-      <c r="D17" s="6" t="s">
-        <v>57</v>
       </c>
       <c r="E17" s="5" t="s">
         <v>17</v>
@@ -4323,13 +4323,13 @@
         <v>13</v>
       </c>
       <c r="B18" s="6" t="s">
+        <v>57</v>
+      </c>
+      <c r="C18" s="6" t="s">
         <v>58</v>
       </c>
-      <c r="C18" s="6" t="s">
+      <c r="D18" s="6" t="s">
         <v>59</v>
-      </c>
-      <c r="D18" s="6" t="s">
-        <v>60</v>
       </c>
       <c r="E18" s="5" t="s">
         <v>17</v>
@@ -4446,19 +4446,19 @@
         <v>1</v>
       </c>
       <c r="B5" s="6" t="s">
+        <v>60</v>
+      </c>
+      <c r="C5" s="6" t="s">
         <v>61</v>
       </c>
-      <c r="C5" s="6" t="s">
+      <c r="D5" s="6" t="s">
         <v>62</v>
-      </c>
-      <c r="D5" s="6" t="s">
-        <v>63</v>
       </c>
       <c r="E5" s="5" t="s">
         <v>17</v>
       </c>
       <c r="F5" s="5" t="s">
-        <v>38</v>
+        <v>63</v>
       </c>
       <c r="G5" s="5" t="s">
         <v>20</v>
@@ -4487,7 +4487,7 @@
         <v>17</v>
       </c>
       <c r="F6" s="5" t="s">
-        <v>38</v>
+        <v>63</v>
       </c>
       <c r="G6" s="5" t="s">
         <v>20</v>
@@ -4513,10 +4513,10 @@
         <v>69</v>
       </c>
       <c r="E7" s="5" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="F7" s="5" t="s">
-        <v>38</v>
+        <v>63</v>
       </c>
       <c r="G7" s="5" t="s">
         <v>20</v>
@@ -4542,10 +4542,10 @@
         <v>72</v>
       </c>
       <c r="E8" s="5" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="F8" s="5" t="s">
-        <v>38</v>
+        <v>63</v>
       </c>
       <c r="G8" s="5" t="s">
         <v>20</v>
@@ -4571,10 +4571,10 @@
         <v>75</v>
       </c>
       <c r="E9" s="5" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="F9" s="5" t="s">
-        <v>38</v>
+        <v>63</v>
       </c>
       <c r="G9" s="5" t="s">
         <v>20</v>
@@ -4600,10 +4600,10 @@
         <v>78</v>
       </c>
       <c r="E10" s="5" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="F10" s="5" t="s">
-        <v>38</v>
+        <v>63</v>
       </c>
       <c r="G10" s="5" t="s">
         <v>20</v>
@@ -4629,10 +4629,10 @@
         <v>80</v>
       </c>
       <c r="E11" s="5" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="F11" s="5" t="s">
-        <v>38</v>
+        <v>63</v>
       </c>
       <c r="G11" s="5" t="s">
         <v>20</v>
@@ -4674,7 +4674,7 @@
         <v>93</v>
       </c>
       <c r="F13" s="5" t="s">
-        <v>38</v>
+        <v>63</v>
       </c>
       <c r="G13" s="5" t="s">
         <v>20</v>
@@ -4703,7 +4703,7 @@
         <v>93</v>
       </c>
       <c r="F14" s="5" t="s">
-        <v>38</v>
+        <v>63</v>
       </c>
       <c r="G14" s="5" t="s">
         <v>20</v>
@@ -4732,7 +4732,7 @@
         <v>93</v>
       </c>
       <c r="F15" s="5" t="s">
-        <v>38</v>
+        <v>63</v>
       </c>
       <c r="G15" s="5" t="s">
         <v>20</v>
@@ -4761,7 +4761,7 @@
         <v>93</v>
       </c>
       <c r="F16" s="5" t="s">
-        <v>38</v>
+        <v>63</v>
       </c>
       <c r="G16" s="5" t="s">
         <v>20</v>
@@ -4790,7 +4790,7 @@
         <v>93</v>
       </c>
       <c r="F17" s="5" t="s">
-        <v>38</v>
+        <v>63</v>
       </c>
       <c r="G17" s="5" t="s">
         <v>20</v>
@@ -4819,7 +4819,7 @@
         <v>93</v>
       </c>
       <c r="F18" s="5" t="s">
-        <v>38</v>
+        <v>63</v>
       </c>
       <c r="G18" s="5" t="s">
         <v>20</v>
@@ -4848,7 +4848,7 @@
         <v>93</v>
       </c>
       <c r="F19" s="5" t="s">
-        <v>38</v>
+        <v>63</v>
       </c>
       <c r="G19" s="5" t="s">
         <v>20</v>
@@ -4877,7 +4877,7 @@
         <v>93</v>
       </c>
       <c r="F20" s="5" t="s">
-        <v>38</v>
+        <v>63</v>
       </c>
       <c r="G20" s="5" t="s">
         <v>20</v>
@@ -4906,7 +4906,7 @@
         <v>93</v>
       </c>
       <c r="F21" s="5" t="s">
-        <v>38</v>
+        <v>63</v>
       </c>
       <c r="G21" s="5" t="s">
         <v>20</v>
@@ -4935,7 +4935,7 @@
         <v>93</v>
       </c>
       <c r="F22" s="5" t="s">
-        <v>38</v>
+        <v>63</v>
       </c>
       <c r="G22" s="5" t="s">
         <v>20</v>
@@ -4955,7 +4955,7 @@
         <v>116</v>
       </c>
       <c r="C23" s="6" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="D23" s="6" t="s">
         <v>117</v>
@@ -4964,7 +4964,7 @@
         <v>93</v>
       </c>
       <c r="F23" s="5" t="s">
-        <v>38</v>
+        <v>63</v>
       </c>
       <c r="G23" s="5" t="s">
         <v>20</v>
@@ -5006,7 +5006,7 @@
         <v>123</v>
       </c>
       <c r="F25" s="5" t="s">
-        <v>38</v>
+        <v>63</v>
       </c>
       <c r="G25" s="5" t="s">
         <v>20</v>
@@ -5035,7 +5035,7 @@
         <v>123</v>
       </c>
       <c r="F26" s="5" t="s">
-        <v>38</v>
+        <v>63</v>
       </c>
       <c r="G26" s="5" t="s">
         <v>20</v>
@@ -5064,7 +5064,7 @@
         <v>123</v>
       </c>
       <c r="F27" s="5" t="s">
-        <v>38</v>
+        <v>63</v>
       </c>
       <c r="G27" s="5" t="s">
         <v>20</v>
@@ -5093,7 +5093,7 @@
         <v>123</v>
       </c>
       <c r="F28" s="5" t="s">
-        <v>38</v>
+        <v>63</v>
       </c>
       <c r="G28" s="5" t="s">
         <v>20</v>
@@ -5122,7 +5122,7 @@
         <v>123</v>
       </c>
       <c r="F29" s="5" t="s">
-        <v>38</v>
+        <v>63</v>
       </c>
       <c r="G29" s="5" t="s">
         <v>20</v>
@@ -5164,7 +5164,7 @@
         <v>141</v>
       </c>
       <c r="F31" s="25" t="s">
-        <v>38</v>
+        <v>63</v>
       </c>
       <c r="G31" s="25" t="s">
         <v>20</v>
@@ -5193,7 +5193,7 @@
         <v>141</v>
       </c>
       <c r="F32" s="5" t="s">
-        <v>38</v>
+        <v>63</v>
       </c>
       <c r="G32" s="5" t="s">
         <v>20</v>
@@ -5222,7 +5222,7 @@
         <v>141</v>
       </c>
       <c r="F33" s="5" t="s">
-        <v>38</v>
+        <v>63</v>
       </c>
       <c r="G33" s="5" t="s">
         <v>20</v>
@@ -5251,7 +5251,7 @@
         <v>141</v>
       </c>
       <c r="F34" s="5" t="s">
-        <v>38</v>
+        <v>63</v>
       </c>
       <c r="G34" s="5" t="s">
         <v>20</v>
@@ -5280,7 +5280,7 @@
         <v>141</v>
       </c>
       <c r="F35" s="5" t="s">
-        <v>38</v>
+        <v>63</v>
       </c>
       <c r="G35" s="5" t="s">
         <v>20</v>
@@ -5309,7 +5309,7 @@
         <v>141</v>
       </c>
       <c r="F36" s="5" t="s">
-        <v>38</v>
+        <v>63</v>
       </c>
       <c r="G36" s="5" t="s">
         <v>20</v>
@@ -5432,10 +5432,10 @@
         <v>83</v>
       </c>
       <c r="E5" s="5" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="F5" s="5" t="s">
-        <v>38</v>
+        <v>63</v>
       </c>
       <c r="G5" s="5" t="s">
         <v>20</v>
@@ -5461,10 +5461,10 @@
         <v>87</v>
       </c>
       <c r="E6" s="5" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="F6" s="5" t="s">
-        <v>38</v>
+        <v>63</v>
       </c>
       <c r="G6" s="5" t="s">
         <v>20</v>
@@ -5506,7 +5506,7 @@
         <v>141</v>
       </c>
       <c r="F8" s="5" t="s">
-        <v>38</v>
+        <v>63</v>
       </c>
       <c r="G8" s="5" t="s">
         <v>20</v>
@@ -5535,7 +5535,7 @@
         <v>141</v>
       </c>
       <c r="F9" s="5" t="s">
-        <v>38</v>
+        <v>63</v>
       </c>
       <c r="G9" s="5" t="s">
         <v>20</v>
@@ -5577,7 +5577,7 @@
         <v>123</v>
       </c>
       <c r="F11" s="5" t="s">
-        <v>38</v>
+        <v>63</v>
       </c>
       <c r="G11" s="5" t="s">
         <v>20</v>
@@ -5606,7 +5606,7 @@
         <v>123</v>
       </c>
       <c r="F12" s="5" t="s">
-        <v>38</v>
+        <v>63</v>
       </c>
       <c r="G12" s="5" t="s">
         <v>20</v>
@@ -5635,7 +5635,7 @@
         <v>123</v>
       </c>
       <c r="F13" s="5" t="s">
-        <v>38</v>
+        <v>63</v>
       </c>
       <c r="G13" s="5" t="s">
         <v>20</v>
@@ -5664,7 +5664,7 @@
         <v>123</v>
       </c>
       <c r="F14" s="5" t="s">
-        <v>38</v>
+        <v>63</v>
       </c>
       <c r="G14" s="5" t="s">
         <v>20</v>
@@ -5693,7 +5693,7 @@
         <v>123</v>
       </c>
       <c r="F15" s="5" t="s">
-        <v>38</v>
+        <v>63</v>
       </c>
       <c r="G15" s="5" t="s">
         <v>20</v>
@@ -5722,7 +5722,7 @@
         <v>123</v>
       </c>
       <c r="F16" s="5" t="s">
-        <v>38</v>
+        <v>63</v>
       </c>
       <c r="G16" s="5" t="s">
         <v>20</v>
@@ -5809,7 +5809,7 @@
     </row>
     <row r="4" ht="50" customHeight="1" spans="1:6">
       <c r="A4" s="5" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="B4" s="6" t="s">
         <v>219</v>

</xml_diff>

<commit_message>
Add Feature Manage Routes
</commit_message>
<xml_diff>
--- a/Project_Tracking.xlsx
+++ b/Project_Tracking.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="23040" windowHeight="9000" activeTab="1"/>
+    <workbookView windowWidth="23040" windowHeight="9707" activeTab="2"/>
   </bookViews>
   <sheets>
     <sheet name="Project Tracking" sheetId="1" r:id="rId1"/>
@@ -31,7 +31,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="984" uniqueCount="242">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="981" uniqueCount="239">
   <si>
     <t>PROJECT TRACKING</t>
   </si>
@@ -753,15 +753,6 @@
   </si>
   <si>
     <t>10 features</t>
-  </si>
-  <si>
-    <t>iter4</t>
-  </si>
-  <si>
-    <t>Polish - Hoan thien, toi uu</t>
-  </si>
-  <si>
-    <t>0 features</t>
   </si>
 </sst>
 </file>
@@ -954,7 +945,7 @@
       <charset val="134"/>
     </font>
   </fonts>
-  <fills count="40">
+  <fills count="39">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -988,12 +979,6 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFFCE4D6"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFE4DFEC"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -1389,7 +1374,7 @@
     <xf numFmtId="0" fontId="13" fillId="0" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="10" borderId="6">
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="6">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="14" fillId="0" borderId="0">
@@ -1413,16 +1398,16 @@
     <xf numFmtId="0" fontId="19" fillId="0" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="11" borderId="9">
+    <xf numFmtId="0" fontId="20" fillId="10" borderId="9">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="12" borderId="10">
+    <xf numFmtId="0" fontId="21" fillId="11" borderId="10">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="12" borderId="9">
+    <xf numFmtId="0" fontId="22" fillId="11" borderId="9">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="23" fillId="13" borderId="11">
+    <xf numFmtId="0" fontId="23" fillId="12" borderId="11">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="24" fillId="0" borderId="12">
@@ -1434,86 +1419,86 @@
     <xf numFmtId="0" fontId="25" fillId="4" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="26" fillId="14" borderId="0">
+    <xf numFmtId="0" fontId="26" fillId="13" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="27" fillId="15" borderId="0">
+    <xf numFmtId="0" fontId="27" fillId="14" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="16" borderId="0">
+    <xf numFmtId="0" fontId="8" fillId="15" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="16" borderId="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="17" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="18" borderId="0">
+    <xf numFmtId="0" fontId="8" fillId="18" borderId="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="19" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="20" borderId="0">
+    <xf numFmtId="0" fontId="0" fillId="20" borderId="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="21" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="22" borderId="0">
+    <xf numFmtId="0" fontId="8" fillId="22" borderId="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="23" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="24" borderId="0">
+    <xf numFmtId="0" fontId="0" fillId="24" borderId="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="25" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="26" borderId="0">
+    <xf numFmtId="0" fontId="8" fillId="26" borderId="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="27" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="28" borderId="0">
+    <xf numFmtId="0" fontId="0" fillId="28" borderId="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="29" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="30" borderId="0">
+    <xf numFmtId="0" fontId="8" fillId="30" borderId="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="31" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="32" borderId="0">
+    <xf numFmtId="0" fontId="0" fillId="32" borderId="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="33" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="34" borderId="0">
+    <xf numFmtId="0" fontId="8" fillId="34" borderId="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="35" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="36" borderId="0">
+    <xf numFmtId="0" fontId="0" fillId="36" borderId="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="37" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="38" borderId="0">
+    <xf numFmtId="0" fontId="8" fillId="38" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="39" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
   </cellStyleXfs>
-  <cellXfs count="40">
+  <cellXfs count="42">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -1547,7 +1532,13 @@
     <xf numFmtId="0" fontId="5" fillId="6" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="7" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -1564,40 +1555,40 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="8" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="7" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="9" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="8" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="9" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="8" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="9" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="8" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="8" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="8" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="9" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="9" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="8" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1610,11 +1601,11 @@
     </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="8" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="49">
@@ -1629,7 +1620,7 @@
     <cellStyle name="Note" xfId="8" builtinId="10"/>
     <cellStyle name="Warning Text" xfId="9" builtinId="11"/>
     <cellStyle name="Title" xfId="10" builtinId="15"/>
-    <cellStyle name="Explanatory Text" xfId="11" builtinId="53"/>
+    <cellStyle name="CExplanatory Text" xfId="11" builtinId="53"/>
     <cellStyle name="Heading 1" xfId="12" builtinId="16"/>
     <cellStyle name="Heading 2" xfId="13" builtinId="17"/>
     <cellStyle name="Heading 3" xfId="14" builtinId="18"/>
@@ -2076,13 +2067,13 @@
     <col min="4" max="4" width="22" customWidth="1"/>
     <col min="5" max="5" width="60" customWidth="1"/>
     <col min="6" max="7" width="14" customWidth="1"/>
-    <col min="8" max="8" width="10" style="34" customWidth="1"/>
+    <col min="8" max="8" width="10" style="36" customWidth="1"/>
     <col min="9" max="9" width="14" customWidth="1"/>
     <col min="10" max="10" width="30" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" ht="40" customHeight="1" spans="1:10">
-      <c r="A1" s="35" t="s">
+      <c r="A1" s="37" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="8"/>
@@ -2091,12 +2082,12 @@
       <c r="E1" s="8"/>
       <c r="F1" s="8"/>
       <c r="G1" s="8"/>
-      <c r="H1" s="36"/>
+      <c r="H1" s="38"/>
       <c r="I1" s="8"/>
       <c r="J1" s="9"/>
     </row>
     <row r="2" ht="25" customHeight="1" spans="1:10">
-      <c r="A2" s="19" t="s">
+      <c r="A2" s="21" t="s">
         <v>1</v>
       </c>
       <c r="B2" s="8"/>
@@ -2105,62 +2096,62 @@
       <c r="E2" s="8"/>
       <c r="F2" s="8"/>
       <c r="G2" s="8"/>
-      <c r="H2" s="36"/>
+      <c r="H2" s="38"/>
       <c r="I2" s="8"/>
       <c r="J2" s="9"/>
     </row>
     <row r="3" ht="35" customHeight="1" spans="1:10">
-      <c r="A3" s="20" t="s">
+      <c r="A3" s="22" t="s">
         <v>2</v>
       </c>
-      <c r="B3" s="20" t="s">
+      <c r="B3" s="22" t="s">
         <v>3</v>
       </c>
-      <c r="C3" s="20" t="s">
+      <c r="C3" s="22" t="s">
         <v>4</v>
       </c>
-      <c r="D3" s="20" t="s">
+      <c r="D3" s="22" t="s">
         <v>5</v>
       </c>
-      <c r="E3" s="20" t="s">
+      <c r="E3" s="22" t="s">
         <v>6</v>
       </c>
-      <c r="F3" s="20" t="s">
+      <c r="F3" s="22" t="s">
         <v>7</v>
       </c>
-      <c r="G3" s="20" t="s">
+      <c r="G3" s="22" t="s">
         <v>8</v>
       </c>
-      <c r="H3" s="20" t="s">
+      <c r="H3" s="22" t="s">
         <v>9</v>
       </c>
-      <c r="I3" s="20" t="s">
+      <c r="I3" s="22" t="s">
         <v>10</v>
       </c>
-      <c r="J3" s="20" t="s">
+      <c r="J3" s="22" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="4" s="33" customFormat="1" ht="28" customHeight="1" spans="1:10">
-      <c r="A4" s="26" t="s">
+    <row r="4" s="35" customFormat="1" ht="28" customHeight="1" spans="1:8">
+      <c r="A4" s="27" t="s">
         <v>12</v>
       </c>
-      <c r="H4" s="37"/>
+      <c r="H4" s="39"/>
     </row>
     <row r="5" ht="45" customHeight="1" spans="1:10">
-      <c r="A5" s="38">
+      <c r="A5" s="25">
         <v>1</v>
       </c>
-      <c r="B5" s="38" t="s">
+      <c r="B5" s="25" t="s">
         <v>13</v>
       </c>
-      <c r="C5" s="38" t="s">
+      <c r="C5" s="25" t="s">
         <v>14</v>
       </c>
-      <c r="D5" s="38" t="s">
+      <c r="D5" s="25" t="s">
         <v>15</v>
       </c>
-      <c r="E5" s="38" t="s">
+      <c r="E5" s="25" t="s">
         <v>16</v>
       </c>
       <c r="F5" s="5" t="s">
@@ -2169,28 +2160,28 @@
       <c r="G5" s="5" t="s">
         <v>18</v>
       </c>
-      <c r="H5" s="39" t="s">
+      <c r="H5" s="40" t="s">
         <v>19</v>
       </c>
-      <c r="I5" s="24"/>
-      <c r="J5" s="24" t="s">
+      <c r="I5" s="28"/>
+      <c r="J5" s="5" t="s">
         <v>20</v>
       </c>
     </row>
     <row r="6" ht="45" customHeight="1" spans="1:10">
-      <c r="A6" s="38">
+      <c r="A6" s="25">
         <v>2</v>
       </c>
-      <c r="B6" s="38" t="s">
+      <c r="B6" s="25" t="s">
         <v>21</v>
       </c>
-      <c r="C6" s="38" t="s">
+      <c r="C6" s="25" t="s">
         <v>22</v>
       </c>
-      <c r="D6" s="38" t="s">
+      <c r="D6" s="25" t="s">
         <v>23</v>
       </c>
-      <c r="E6" s="38" t="s">
+      <c r="E6" s="25" t="s">
         <v>24</v>
       </c>
       <c r="F6" s="5" t="s">
@@ -2199,28 +2190,28 @@
       <c r="G6" s="5" t="s">
         <v>18</v>
       </c>
-      <c r="H6" s="39" t="s">
+      <c r="H6" s="40" t="s">
         <v>19</v>
       </c>
-      <c r="I6" s="24"/>
-      <c r="J6" s="24" t="s">
+      <c r="I6" s="28"/>
+      <c r="J6" s="5" t="s">
         <v>20</v>
       </c>
     </row>
     <row r="7" ht="45" customHeight="1" spans="1:10">
-      <c r="A7" s="38">
+      <c r="A7" s="25">
         <v>3</v>
       </c>
-      <c r="B7" s="38" t="s">
+      <c r="B7" s="25" t="s">
         <v>25</v>
       </c>
-      <c r="C7" s="38" t="s">
+      <c r="C7" s="25" t="s">
         <v>26</v>
       </c>
-      <c r="D7" s="38" t="s">
+      <c r="D7" s="25" t="s">
         <v>15</v>
       </c>
-      <c r="E7" s="38" t="s">
+      <c r="E7" s="25" t="s">
         <v>27</v>
       </c>
       <c r="F7" s="5" t="s">
@@ -2229,28 +2220,28 @@
       <c r="G7" s="5" t="s">
         <v>18</v>
       </c>
-      <c r="H7" s="39" t="s">
+      <c r="H7" s="40" t="s">
         <v>19</v>
       </c>
-      <c r="I7" s="24"/>
-      <c r="J7" s="24" t="s">
+      <c r="I7" s="28"/>
+      <c r="J7" s="5" t="s">
         <v>20</v>
       </c>
     </row>
     <row r="8" ht="45" customHeight="1" spans="1:10">
-      <c r="A8" s="38">
+      <c r="A8" s="25">
         <v>4</v>
       </c>
-      <c r="B8" s="38" t="s">
+      <c r="B8" s="25" t="s">
         <v>28</v>
       </c>
-      <c r="C8" s="38" t="s">
+      <c r="C8" s="25" t="s">
         <v>29</v>
       </c>
-      <c r="D8" s="38" t="s">
+      <c r="D8" s="25" t="s">
         <v>15</v>
       </c>
-      <c r="E8" s="38" t="s">
+      <c r="E8" s="25" t="s">
         <v>30</v>
       </c>
       <c r="F8" s="5" t="s">
@@ -2259,28 +2250,28 @@
       <c r="G8" s="5" t="s">
         <v>18</v>
       </c>
-      <c r="H8" s="39" t="s">
+      <c r="H8" s="40" t="s">
         <v>19</v>
       </c>
-      <c r="I8" s="24"/>
-      <c r="J8" s="24" t="s">
+      <c r="I8" s="28"/>
+      <c r="J8" s="5" t="s">
         <v>20</v>
       </c>
     </row>
     <row r="9" ht="45" customHeight="1" spans="1:10">
-      <c r="A9" s="38">
+      <c r="A9" s="25">
         <v>5</v>
       </c>
-      <c r="B9" s="38" t="s">
+      <c r="B9" s="25" t="s">
         <v>31</v>
       </c>
-      <c r="C9" s="38" t="s">
+      <c r="C9" s="25" t="s">
         <v>32</v>
       </c>
-      <c r="D9" s="38" t="s">
+      <c r="D9" s="25" t="s">
         <v>15</v>
       </c>
-      <c r="E9" s="38" t="s">
+      <c r="E9" s="25" t="s">
         <v>33</v>
       </c>
       <c r="F9" s="5" t="s">
@@ -2289,27 +2280,27 @@
       <c r="G9" s="5" t="s">
         <v>18</v>
       </c>
-      <c r="H9" s="39" t="s">
+      <c r="H9" s="40" t="s">
         <v>19</v>
       </c>
-      <c r="I9" s="24"/>
-      <c r="J9" s="24" t="s">
+      <c r="I9" s="28"/>
+      <c r="J9" s="5" t="s">
         <v>20</v>
       </c>
     </row>
     <row r="10" ht="45" customHeight="1" spans="1:10">
-      <c r="A10" s="21" t="s">
+      <c r="A10" s="23" t="s">
         <v>34</v>
       </c>
-      <c r="B10" s="22"/>
-      <c r="C10" s="22"/>
-      <c r="D10" s="22"/>
-      <c r="E10" s="22"/>
-      <c r="F10" s="22"/>
-      <c r="G10" s="22"/>
-      <c r="H10" s="22"/>
-      <c r="I10" s="22"/>
-      <c r="J10" s="23"/>
+      <c r="B10" s="24"/>
+      <c r="C10" s="24"/>
+      <c r="D10" s="24"/>
+      <c r="E10" s="24"/>
+      <c r="F10" s="24"/>
+      <c r="G10" s="24"/>
+      <c r="H10" s="24"/>
+      <c r="I10" s="24"/>
+      <c r="J10" s="41"/>
     </row>
     <row r="11" ht="45" customHeight="1" spans="1:10">
       <c r="A11" s="5">
@@ -2333,13 +2324,13 @@
       <c r="G11" s="5" t="s">
         <v>18</v>
       </c>
-      <c r="H11" s="39" t="s">
+      <c r="H11" s="40" t="s">
         <v>19</v>
       </c>
       <c r="I11" s="5" t="s">
         <v>20</v>
       </c>
-      <c r="J11" s="6" t="s">
+      <c r="J11" s="5" t="s">
         <v>20</v>
       </c>
     </row>
@@ -2365,13 +2356,13 @@
       <c r="G12" s="5" t="s">
         <v>18</v>
       </c>
-      <c r="H12" s="39" t="s">
+      <c r="H12" s="40" t="s">
         <v>19</v>
       </c>
       <c r="I12" s="5" t="s">
         <v>20</v>
       </c>
-      <c r="J12" s="6" t="s">
+      <c r="J12" s="5" t="s">
         <v>20</v>
       </c>
     </row>
@@ -2397,13 +2388,13 @@
       <c r="G13" s="5" t="s">
         <v>18</v>
       </c>
-      <c r="H13" s="39" t="s">
+      <c r="H13" s="40" t="s">
         <v>19</v>
       </c>
       <c r="I13" s="5" t="s">
         <v>20</v>
       </c>
-      <c r="J13" s="6" t="s">
+      <c r="J13" s="5" t="s">
         <v>20</v>
       </c>
     </row>
@@ -2429,13 +2420,13 @@
       <c r="G14" s="5" t="s">
         <v>18</v>
       </c>
-      <c r="H14" s="39" t="s">
+      <c r="H14" s="40" t="s">
         <v>19</v>
       </c>
       <c r="I14" s="5" t="s">
         <v>20</v>
       </c>
-      <c r="J14" s="6" t="s">
+      <c r="J14" s="5" t="s">
         <v>20</v>
       </c>
     </row>
@@ -2461,13 +2452,13 @@
       <c r="G15" s="5" t="s">
         <v>18</v>
       </c>
-      <c r="H15" s="39" t="s">
+      <c r="H15" s="40" t="s">
         <v>19</v>
       </c>
       <c r="I15" s="5" t="s">
         <v>20</v>
       </c>
-      <c r="J15" s="6" t="s">
+      <c r="J15" s="5" t="s">
         <v>20</v>
       </c>
     </row>
@@ -2493,13 +2484,13 @@
       <c r="G16" s="5" t="s">
         <v>18</v>
       </c>
-      <c r="H16" s="39" t="s">
+      <c r="H16" s="40" t="s">
         <v>19</v>
       </c>
       <c r="I16" s="5" t="s">
         <v>20</v>
       </c>
-      <c r="J16" s="6" t="s">
+      <c r="J16" s="5" t="s">
         <v>20</v>
       </c>
     </row>
@@ -2525,13 +2516,13 @@
       <c r="G17" s="5" t="s">
         <v>18</v>
       </c>
-      <c r="H17" s="39" t="s">
+      <c r="H17" s="40" t="s">
         <v>19</v>
       </c>
       <c r="I17" s="5" t="s">
         <v>20</v>
       </c>
-      <c r="J17" s="6" t="s">
+      <c r="J17" s="5" t="s">
         <v>20</v>
       </c>
     </row>
@@ -2557,13 +2548,13 @@
       <c r="G18" s="5" t="s">
         <v>18</v>
       </c>
-      <c r="H18" s="39" t="s">
+      <c r="H18" s="40" t="s">
         <v>19</v>
       </c>
       <c r="I18" s="5" t="s">
         <v>20</v>
       </c>
-      <c r="J18" s="6" t="s">
+      <c r="J18" s="5" t="s">
         <v>20</v>
       </c>
     </row>
@@ -2589,13 +2580,13 @@
       <c r="G19" s="5" t="s">
         <v>63</v>
       </c>
-      <c r="H19" s="39" t="s">
+      <c r="H19" s="40" t="s">
         <v>64</v>
       </c>
       <c r="I19" s="5" t="s">
         <v>20</v>
       </c>
-      <c r="J19" s="6" t="s">
+      <c r="J19" s="5" t="s">
         <v>20</v>
       </c>
     </row>
@@ -2621,13 +2612,13 @@
       <c r="G20" s="5" t="s">
         <v>63</v>
       </c>
-      <c r="H20" s="39" t="s">
+      <c r="H20" s="40" t="s">
         <v>64</v>
       </c>
       <c r="I20" s="5" t="s">
         <v>20</v>
       </c>
-      <c r="J20" s="6" t="s">
+      <c r="J20" s="5" t="s">
         <v>20</v>
       </c>
     </row>
@@ -2653,17 +2644,17 @@
       <c r="G21" s="5" t="s">
         <v>63</v>
       </c>
-      <c r="H21" s="39" t="s">
+      <c r="H21" s="40" t="s">
         <v>64</v>
       </c>
       <c r="I21" s="5" t="s">
         <v>20</v>
       </c>
-      <c r="J21" s="6" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="22" s="33" customFormat="1" ht="28" customHeight="1" spans="1:10">
+      <c r="J21" s="5" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="22" s="35" customFormat="1" ht="28" customHeight="1" spans="1:10">
       <c r="A22" s="6">
         <v>17</v>
       </c>
@@ -2685,13 +2676,13 @@
       <c r="G22" s="5" t="s">
         <v>63</v>
       </c>
-      <c r="H22" s="39" t="s">
+      <c r="H22" s="40" t="s">
         <v>64</v>
       </c>
-      <c r="I22" s="24" t="s">
-        <v>20</v>
-      </c>
-      <c r="J22" s="24" t="s">
+      <c r="I22" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="J22" s="5" t="s">
         <v>20</v>
       </c>
     </row>
@@ -2717,13 +2708,13 @@
       <c r="G23" s="5" t="s">
         <v>63</v>
       </c>
-      <c r="H23" s="39" t="s">
+      <c r="H23" s="40" t="s">
         <v>64</v>
       </c>
       <c r="I23" s="5" t="s">
         <v>20</v>
       </c>
-      <c r="J23" s="6" t="s">
+      <c r="J23" s="5" t="s">
         <v>20</v>
       </c>
     </row>
@@ -2749,13 +2740,13 @@
       <c r="G24" s="5" t="s">
         <v>63</v>
       </c>
-      <c r="H24" s="39" t="s">
+      <c r="H24" s="40" t="s">
         <v>64</v>
       </c>
       <c r="I24" s="5" t="s">
         <v>20</v>
       </c>
-      <c r="J24" s="6" t="s">
+      <c r="J24" s="5" t="s">
         <v>20</v>
       </c>
     </row>
@@ -2781,13 +2772,13 @@
       <c r="G25" s="5" t="s">
         <v>63</v>
       </c>
-      <c r="H25" s="39" t="s">
+      <c r="H25" s="40" t="s">
         <v>64</v>
       </c>
       <c r="I25" s="5" t="s">
         <v>20</v>
       </c>
-      <c r="J25" s="6" t="s">
+      <c r="J25" s="5" t="s">
         <v>20</v>
       </c>
     </row>
@@ -2813,13 +2804,13 @@
       <c r="G26" s="5" t="s">
         <v>63</v>
       </c>
-      <c r="H26" s="39" t="s">
+      <c r="H26" s="40" t="s">
         <v>84</v>
       </c>
       <c r="I26" s="5" t="s">
         <v>20</v>
       </c>
-      <c r="J26" s="6" t="s">
+      <c r="J26" s="5" t="s">
         <v>20</v>
       </c>
     </row>
@@ -2845,29 +2836,29 @@
       <c r="G27" s="5" t="s">
         <v>63</v>
       </c>
-      <c r="H27" s="39" t="s">
+      <c r="H27" s="40" t="s">
         <v>84</v>
       </c>
       <c r="I27" s="5" t="s">
         <v>20</v>
       </c>
-      <c r="J27" s="6" t="s">
+      <c r="J27" s="5" t="s">
         <v>20</v>
       </c>
     </row>
     <row r="28" ht="45" customHeight="1" spans="1:10">
-      <c r="A28" s="21" t="s">
+      <c r="A28" s="23" t="s">
         <v>88</v>
       </c>
-      <c r="B28" s="22"/>
-      <c r="C28" s="22"/>
-      <c r="D28" s="22"/>
-      <c r="E28" s="22"/>
-      <c r="F28" s="22"/>
-      <c r="G28" s="22"/>
-      <c r="H28" s="22"/>
-      <c r="I28" s="22"/>
-      <c r="J28" s="23"/>
+      <c r="B28" s="24"/>
+      <c r="C28" s="24"/>
+      <c r="D28" s="24"/>
+      <c r="E28" s="24"/>
+      <c r="F28" s="24"/>
+      <c r="G28" s="24"/>
+      <c r="H28" s="24"/>
+      <c r="I28" s="24"/>
+      <c r="J28" s="41"/>
     </row>
     <row r="29" ht="45" customHeight="1" spans="1:10">
       <c r="A29" s="5">
@@ -2891,13 +2882,13 @@
       <c r="G29" s="5" t="s">
         <v>63</v>
       </c>
-      <c r="H29" s="39" t="s">
+      <c r="H29" s="40" t="s">
         <v>64</v>
       </c>
       <c r="I29" s="5" t="s">
         <v>20</v>
       </c>
-      <c r="J29" s="6" t="s">
+      <c r="J29" s="5" t="s">
         <v>20</v>
       </c>
     </row>
@@ -2923,13 +2914,13 @@
       <c r="G30" s="5" t="s">
         <v>63</v>
       </c>
-      <c r="H30" s="39" t="s">
+      <c r="H30" s="40" t="s">
         <v>64</v>
       </c>
       <c r="I30" s="5" t="s">
         <v>20</v>
       </c>
-      <c r="J30" s="6" t="s">
+      <c r="J30" s="5" t="s">
         <v>20</v>
       </c>
     </row>
@@ -2955,13 +2946,13 @@
       <c r="G31" s="5" t="s">
         <v>63</v>
       </c>
-      <c r="H31" s="39" t="s">
+      <c r="H31" s="40" t="s">
         <v>64</v>
       </c>
       <c r="I31" s="5" t="s">
         <v>20</v>
       </c>
-      <c r="J31" s="6" t="s">
+      <c r="J31" s="5" t="s">
         <v>20</v>
       </c>
     </row>
@@ -2987,13 +2978,13 @@
       <c r="G32" s="5" t="s">
         <v>63</v>
       </c>
-      <c r="H32" s="39" t="s">
+      <c r="H32" s="40" t="s">
         <v>64</v>
       </c>
       <c r="I32" s="5" t="s">
         <v>20</v>
       </c>
-      <c r="J32" s="6" t="s">
+      <c r="J32" s="5" t="s">
         <v>20</v>
       </c>
     </row>
@@ -3019,30 +3010,30 @@
       <c r="G33" s="5" t="s">
         <v>63</v>
       </c>
-      <c r="H33" s="39" t="s">
+      <c r="H33" s="40" t="s">
         <v>64</v>
       </c>
       <c r="I33" s="5" t="s">
         <v>20</v>
       </c>
-      <c r="J33" s="6" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="34" s="33" customFormat="1" ht="38" customHeight="1" spans="1:10">
+      <c r="J33" s="5" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="34" s="35" customFormat="1" ht="38" customHeight="1" spans="1:10">
       <c r="A34" s="5">
         <v>28</v>
       </c>
       <c r="B34" s="5" t="s">
         <v>103</v>
       </c>
-      <c r="C34" s="38" t="s">
+      <c r="C34" s="25" t="s">
         <v>104</v>
       </c>
-      <c r="D34" s="38" t="s">
+      <c r="D34" s="25" t="s">
         <v>91</v>
       </c>
-      <c r="E34" s="38" t="s">
+      <c r="E34" s="25" t="s">
         <v>105</v>
       </c>
       <c r="F34" s="5" t="s">
@@ -3051,13 +3042,13 @@
       <c r="G34" s="5" t="s">
         <v>63</v>
       </c>
-      <c r="H34" s="39" t="s">
+      <c r="H34" s="40" t="s">
         <v>64</v>
       </c>
-      <c r="I34" s="24" t="s">
-        <v>20</v>
-      </c>
-      <c r="J34" s="24" t="s">
+      <c r="I34" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="J34" s="5" t="s">
         <v>20</v>
       </c>
     </row>
@@ -3081,15 +3072,15 @@
         <v>93</v>
       </c>
       <c r="G35" s="5" t="s">
-        <v>63</v>
-      </c>
-      <c r="H35" s="39" t="s">
+        <v>18</v>
+      </c>
+      <c r="H35" s="40" t="s">
         <v>64</v>
       </c>
       <c r="I35" s="5" t="s">
         <v>20</v>
       </c>
-      <c r="J35" s="6" t="s">
+      <c r="J35" s="5" t="s">
         <v>20</v>
       </c>
     </row>
@@ -3113,15 +3104,15 @@
         <v>93</v>
       </c>
       <c r="G36" s="5" t="s">
-        <v>63</v>
-      </c>
-      <c r="H36" s="39" t="s">
+        <v>18</v>
+      </c>
+      <c r="H36" s="40" t="s">
         <v>64</v>
       </c>
       <c r="I36" s="5" t="s">
         <v>20</v>
       </c>
-      <c r="J36" s="6" t="s">
+      <c r="J36" s="5" t="s">
         <v>20</v>
       </c>
     </row>
@@ -3145,15 +3136,15 @@
         <v>93</v>
       </c>
       <c r="G37" s="5" t="s">
-        <v>63</v>
-      </c>
-      <c r="H37" s="39" t="s">
+        <v>18</v>
+      </c>
+      <c r="H37" s="40" t="s">
         <v>64</v>
       </c>
       <c r="I37" s="5" t="s">
         <v>20</v>
       </c>
-      <c r="J37" s="6" t="s">
+      <c r="J37" s="5" t="s">
         <v>20</v>
       </c>
     </row>
@@ -3177,15 +3168,15 @@
         <v>93</v>
       </c>
       <c r="G38" s="5" t="s">
-        <v>63</v>
-      </c>
-      <c r="H38" s="39" t="s">
+        <v>18</v>
+      </c>
+      <c r="H38" s="40" t="s">
         <v>64</v>
       </c>
       <c r="I38" s="5" t="s">
         <v>20</v>
       </c>
-      <c r="J38" s="6" t="s">
+      <c r="J38" s="5" t="s">
         <v>20</v>
       </c>
     </row>
@@ -3209,33 +3200,33 @@
         <v>93</v>
       </c>
       <c r="G39" s="5" t="s">
-        <v>63</v>
-      </c>
-      <c r="H39" s="39" t="s">
+        <v>18</v>
+      </c>
+      <c r="H39" s="40" t="s">
         <v>64</v>
       </c>
       <c r="I39" s="5" t="s">
         <v>20</v>
       </c>
-      <c r="J39" s="6" t="s">
+      <c r="J39" s="5" t="s">
         <v>20</v>
       </c>
     </row>
     <row r="40" ht="45" customHeight="1" spans="1:10">
-      <c r="A40" s="21" t="s">
+      <c r="A40" s="23" t="s">
         <v>118</v>
       </c>
-      <c r="B40" s="22"/>
-      <c r="C40" s="22"/>
-      <c r="D40" s="22"/>
-      <c r="E40" s="22"/>
-      <c r="F40" s="22"/>
-      <c r="G40" s="22"/>
-      <c r="H40" s="22"/>
-      <c r="I40" s="22"/>
-      <c r="J40" s="23"/>
-    </row>
-    <row r="41" s="33" customFormat="1" ht="46" customHeight="1" spans="1:10">
+      <c r="B40" s="24"/>
+      <c r="C40" s="24"/>
+      <c r="D40" s="24"/>
+      <c r="E40" s="24"/>
+      <c r="F40" s="24"/>
+      <c r="G40" s="24"/>
+      <c r="H40" s="24"/>
+      <c r="I40" s="24"/>
+      <c r="J40" s="41"/>
+    </row>
+    <row r="41" s="35" customFormat="1" ht="46" customHeight="1" spans="1:10">
       <c r="A41" s="6">
         <v>34</v>
       </c>
@@ -3257,13 +3248,13 @@
       <c r="G41" s="5" t="s">
         <v>63</v>
       </c>
-      <c r="H41" s="39" t="s">
+      <c r="H41" s="40" t="s">
         <v>64</v>
       </c>
-      <c r="I41" s="24" t="s">
-        <v>20</v>
-      </c>
-      <c r="J41" s="24" t="s">
+      <c r="I41" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="J41" s="5" t="s">
         <v>20</v>
       </c>
     </row>
@@ -3289,13 +3280,13 @@
       <c r="G42" s="5" t="s">
         <v>63</v>
       </c>
-      <c r="H42" s="39" t="s">
+      <c r="H42" s="40" t="s">
         <v>64</v>
       </c>
       <c r="I42" s="5" t="s">
         <v>20</v>
       </c>
-      <c r="J42" s="6" t="s">
+      <c r="J42" s="5" t="s">
         <v>20</v>
       </c>
     </row>
@@ -3321,13 +3312,13 @@
       <c r="G43" s="5" t="s">
         <v>63</v>
       </c>
-      <c r="H43" s="39" t="s">
+      <c r="H43" s="40" t="s">
         <v>64</v>
       </c>
       <c r="I43" s="5" t="s">
         <v>20</v>
       </c>
-      <c r="J43" s="6" t="s">
+      <c r="J43" s="5" t="s">
         <v>20</v>
       </c>
     </row>
@@ -3353,13 +3344,13 @@
       <c r="G44" s="5" t="s">
         <v>63</v>
       </c>
-      <c r="H44" s="39" t="s">
+      <c r="H44" s="40" t="s">
         <v>64</v>
       </c>
       <c r="I44" s="5" t="s">
         <v>20</v>
       </c>
-      <c r="J44" s="6" t="s">
+      <c r="J44" s="5" t="s">
         <v>20</v>
       </c>
     </row>
@@ -3385,29 +3376,29 @@
       <c r="G45" s="5" t="s">
         <v>63</v>
       </c>
-      <c r="H45" s="39" t="s">
+      <c r="H45" s="40" t="s">
         <v>64</v>
       </c>
       <c r="I45" s="5" t="s">
         <v>20</v>
       </c>
-      <c r="J45" s="6" t="s">
+      <c r="J45" s="5" t="s">
         <v>20</v>
       </c>
     </row>
     <row r="46" ht="45" customHeight="1" spans="1:10">
-      <c r="A46" s="21" t="s">
+      <c r="A46" s="23" t="s">
         <v>136</v>
       </c>
-      <c r="B46" s="22"/>
-      <c r="C46" s="22"/>
-      <c r="D46" s="22"/>
-      <c r="E46" s="22"/>
-      <c r="F46" s="22"/>
-      <c r="G46" s="22"/>
-      <c r="H46" s="22"/>
-      <c r="I46" s="22"/>
-      <c r="J46" s="23"/>
+      <c r="B46" s="24"/>
+      <c r="C46" s="24"/>
+      <c r="D46" s="24"/>
+      <c r="E46" s="24"/>
+      <c r="F46" s="24"/>
+      <c r="G46" s="24"/>
+      <c r="H46" s="24"/>
+      <c r="I46" s="24"/>
+      <c r="J46" s="41"/>
     </row>
     <row r="47" ht="45" customHeight="1" spans="1:10">
       <c r="A47" s="5">
@@ -3431,13 +3422,13 @@
       <c r="G47" s="5" t="s">
         <v>63</v>
       </c>
-      <c r="H47" s="39" t="s">
+      <c r="H47" s="40" t="s">
         <v>64</v>
       </c>
       <c r="I47" s="5" t="s">
         <v>20</v>
       </c>
-      <c r="J47" s="6" t="s">
+      <c r="J47" s="5" t="s">
         <v>20</v>
       </c>
     </row>
@@ -3463,13 +3454,13 @@
       <c r="G48" s="5" t="s">
         <v>63</v>
       </c>
-      <c r="H48" s="39" t="s">
+      <c r="H48" s="40" t="s">
         <v>64</v>
       </c>
       <c r="I48" s="5" t="s">
         <v>20</v>
       </c>
-      <c r="J48" s="6" t="s">
+      <c r="J48" s="5" t="s">
         <v>20</v>
       </c>
     </row>
@@ -3495,30 +3486,30 @@
       <c r="G49" s="5" t="s">
         <v>63</v>
       </c>
-      <c r="H49" s="39" t="s">
+      <c r="H49" s="40" t="s">
         <v>64</v>
       </c>
       <c r="I49" s="5" t="s">
         <v>20</v>
       </c>
-      <c r="J49" s="6" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="50" s="33" customFormat="1" ht="28" customHeight="1" spans="1:10">
+      <c r="J49" s="5" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="50" s="35" customFormat="1" ht="28" customHeight="1" spans="1:10">
       <c r="A50" s="5">
         <v>42</v>
       </c>
-      <c r="B50" s="38" t="s">
+      <c r="B50" s="25" t="s">
         <v>147</v>
       </c>
-      <c r="C50" s="38" t="s">
+      <c r="C50" s="25" t="s">
         <v>148</v>
       </c>
-      <c r="D50" s="38" t="s">
+      <c r="D50" s="25" t="s">
         <v>139</v>
       </c>
-      <c r="E50" s="38" t="s">
+      <c r="E50" s="25" t="s">
         <v>149</v>
       </c>
       <c r="F50" s="5" t="s">
@@ -3527,13 +3518,13 @@
       <c r="G50" s="5" t="s">
         <v>63</v>
       </c>
-      <c r="H50" s="39" t="s">
+      <c r="H50" s="40" t="s">
         <v>64</v>
       </c>
-      <c r="I50" s="24" t="s">
-        <v>20</v>
-      </c>
-      <c r="J50" s="24" t="s">
+      <c r="I50" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="J50" s="5" t="s">
         <v>20</v>
       </c>
     </row>
@@ -3559,13 +3550,13 @@
       <c r="G51" s="5" t="s">
         <v>63</v>
       </c>
-      <c r="H51" s="39" t="s">
+      <c r="H51" s="40" t="s">
         <v>64</v>
       </c>
       <c r="I51" s="5" t="s">
         <v>20</v>
       </c>
-      <c r="J51" s="6" t="s">
+      <c r="J51" s="5" t="s">
         <v>20</v>
       </c>
     </row>
@@ -3591,13 +3582,13 @@
       <c r="G52" s="5" t="s">
         <v>63</v>
       </c>
-      <c r="H52" s="39" t="s">
+      <c r="H52" s="40" t="s">
         <v>84</v>
       </c>
       <c r="I52" s="5" t="s">
         <v>20</v>
       </c>
-      <c r="J52" s="6" t="s">
+      <c r="J52" s="5" t="s">
         <v>20</v>
       </c>
     </row>
@@ -3623,13 +3614,13 @@
       <c r="G53" s="5" t="s">
         <v>63</v>
       </c>
-      <c r="H53" s="39" t="s">
+      <c r="H53" s="40" t="s">
         <v>64</v>
       </c>
       <c r="I53" s="5" t="s">
         <v>20</v>
       </c>
-      <c r="J53" s="6" t="s">
+      <c r="J53" s="5" t="s">
         <v>20</v>
       </c>
     </row>
@@ -3655,29 +3646,29 @@
       <c r="G54" s="5" t="s">
         <v>63</v>
       </c>
-      <c r="H54" s="39" t="s">
+      <c r="H54" s="40" t="s">
         <v>84</v>
       </c>
       <c r="I54" s="5" t="s">
         <v>20</v>
       </c>
-      <c r="J54" s="6" t="s">
+      <c r="J54" s="5" t="s">
         <v>20</v>
       </c>
     </row>
     <row r="55" ht="45" customHeight="1" spans="1:10">
-      <c r="A55" s="21" t="s">
+      <c r="A55" s="23" t="s">
         <v>161</v>
       </c>
-      <c r="B55" s="22"/>
-      <c r="C55" s="22"/>
-      <c r="D55" s="22"/>
-      <c r="E55" s="22"/>
-      <c r="F55" s="22"/>
-      <c r="G55" s="22"/>
-      <c r="H55" s="22"/>
-      <c r="I55" s="22"/>
-      <c r="J55" s="23"/>
+      <c r="B55" s="24"/>
+      <c r="C55" s="24"/>
+      <c r="D55" s="24"/>
+      <c r="E55" s="24"/>
+      <c r="F55" s="24"/>
+      <c r="G55" s="24"/>
+      <c r="H55" s="24"/>
+      <c r="I55" s="24"/>
+      <c r="J55" s="41"/>
     </row>
     <row r="56" ht="45" customHeight="1" spans="1:10">
       <c r="A56" s="5">
@@ -3701,13 +3692,13 @@
       <c r="G56" s="5" t="s">
         <v>63</v>
       </c>
-      <c r="H56" s="39" t="s">
+      <c r="H56" s="40" t="s">
         <v>84</v>
       </c>
       <c r="I56" s="5" t="s">
         <v>20</v>
       </c>
-      <c r="J56" s="6" t="s">
+      <c r="J56" s="5" t="s">
         <v>20</v>
       </c>
     </row>
@@ -3733,13 +3724,13 @@
       <c r="G57" s="5" t="s">
         <v>63</v>
       </c>
-      <c r="H57" s="39" t="s">
+      <c r="H57" s="40" t="s">
         <v>84</v>
       </c>
       <c r="I57" s="5" t="s">
         <v>20</v>
       </c>
-      <c r="J57" s="6" t="s">
+      <c r="J57" s="5" t="s">
         <v>20</v>
       </c>
     </row>
@@ -3765,13 +3756,13 @@
       <c r="G58" s="5" t="s">
         <v>63</v>
       </c>
-      <c r="H58" s="39" t="s">
+      <c r="H58" s="40" t="s">
         <v>84</v>
       </c>
       <c r="I58" s="5" t="s">
         <v>20</v>
       </c>
-      <c r="J58" s="6" t="s">
+      <c r="J58" s="5" t="s">
         <v>20</v>
       </c>
     </row>
@@ -3797,13 +3788,13 @@
       <c r="G59" s="5" t="s">
         <v>63</v>
       </c>
-      <c r="H59" s="39" t="s">
+      <c r="H59" s="40" t="s">
         <v>84</v>
       </c>
       <c r="I59" s="5" t="s">
         <v>20</v>
       </c>
-      <c r="J59" s="6" t="s">
+      <c r="J59" s="5" t="s">
         <v>20</v>
       </c>
     </row>
@@ -3829,13 +3820,13 @@
       <c r="G60" s="5" t="s">
         <v>63</v>
       </c>
-      <c r="H60" s="39" t="s">
+      <c r="H60" s="40" t="s">
         <v>84</v>
       </c>
       <c r="I60" s="5" t="s">
         <v>20</v>
       </c>
-      <c r="J60" s="6" t="s">
+      <c r="J60" s="5" t="s">
         <v>20</v>
       </c>
     </row>
@@ -3861,13 +3852,13 @@
       <c r="G61" s="5" t="s">
         <v>63</v>
       </c>
-      <c r="H61" s="39" t="s">
+      <c r="H61" s="40" t="s">
         <v>84</v>
       </c>
       <c r="I61" s="5" t="s">
         <v>20</v>
       </c>
-      <c r="J61" s="6" t="s">
+      <c r="J61" s="5" t="s">
         <v>20</v>
       </c>
     </row>
@@ -3898,7 +3889,7 @@
   </cols>
   <sheetData>
     <row r="1" ht="38" customHeight="1" spans="1:9">
-      <c r="A1" s="18" t="s">
+      <c r="A1" s="20" t="s">
         <v>181</v>
       </c>
       <c r="B1" s="8"/>
@@ -3911,7 +3902,7 @@
       <c r="I1" s="9"/>
     </row>
     <row r="2" ht="25" customHeight="1" spans="1:9">
-      <c r="A2" s="19" t="s">
+      <c r="A2" s="21" t="s">
         <v>182</v>
       </c>
       <c r="B2" s="8"/>
@@ -3924,196 +3915,196 @@
       <c r="I2" s="9"/>
     </row>
     <row r="3" ht="35" customHeight="1" spans="1:9">
-      <c r="A3" s="20" t="s">
+      <c r="A3" s="22" t="s">
         <v>2</v>
       </c>
-      <c r="B3" s="20" t="s">
+      <c r="B3" s="22" t="s">
         <v>183</v>
       </c>
-      <c r="C3" s="20" t="s">
+      <c r="C3" s="22" t="s">
         <v>4</v>
       </c>
-      <c r="D3" s="20" t="s">
+      <c r="D3" s="22" t="s">
         <v>6</v>
       </c>
-      <c r="E3" s="20" t="s">
+      <c r="E3" s="22" t="s">
         <v>7</v>
       </c>
-      <c r="F3" s="20" t="s">
+      <c r="F3" s="22" t="s">
         <v>8</v>
       </c>
-      <c r="G3" s="20" t="s">
+      <c r="G3" s="22" t="s">
         <v>184</v>
       </c>
-      <c r="H3" s="20" t="s">
+      <c r="H3" s="22" t="s">
         <v>185</v>
       </c>
-      <c r="I3" s="20" t="s">
+      <c r="I3" s="22" t="s">
         <v>186</v>
       </c>
     </row>
-    <row r="4" ht="28" customHeight="1" spans="1:9">
-      <c r="A4" s="26" t="s">
+    <row r="4" ht="28" customHeight="1" spans="1:1">
+      <c r="A4" s="27" t="s">
         <v>12</v>
       </c>
     </row>
     <row r="5" ht="45" customHeight="1" spans="1:9">
-      <c r="A5" s="24">
+      <c r="A5" s="28">
         <v>1</v>
       </c>
-      <c r="B5" s="24" t="s">
+      <c r="B5" s="28" t="s">
         <v>13</v>
       </c>
-      <c r="C5" s="24" t="s">
+      <c r="C5" s="28" t="s">
         <v>14</v>
       </c>
-      <c r="D5" s="24" t="s">
+      <c r="D5" s="28" t="s">
         <v>16</v>
       </c>
-      <c r="E5" s="24" t="s">
+      <c r="E5" s="28" t="s">
         <v>17</v>
       </c>
-      <c r="F5" s="27" t="s">
+      <c r="F5" s="29" t="s">
         <v>18</v>
       </c>
-      <c r="G5" s="28" t="s">
-        <v>20</v>
-      </c>
-      <c r="H5" s="28" t="s">
-        <v>20</v>
-      </c>
-      <c r="I5" s="29" t="s">
+      <c r="G5" s="30" t="s">
+        <v>20</v>
+      </c>
+      <c r="H5" s="30" t="s">
+        <v>20</v>
+      </c>
+      <c r="I5" s="32" t="s">
         <v>187</v>
       </c>
     </row>
     <row r="6" ht="45" customHeight="1" spans="1:9">
-      <c r="A6" s="24">
+      <c r="A6" s="28">
         <v>2</v>
       </c>
-      <c r="B6" s="24" t="s">
+      <c r="B6" s="28" t="s">
         <v>21</v>
       </c>
-      <c r="C6" s="24" t="s">
+      <c r="C6" s="28" t="s">
         <v>22</v>
       </c>
-      <c r="D6" s="24" t="s">
+      <c r="D6" s="28" t="s">
         <v>24</v>
       </c>
-      <c r="E6" s="24" t="s">
+      <c r="E6" s="28" t="s">
         <v>17</v>
       </c>
-      <c r="F6" s="27" t="s">
+      <c r="F6" s="29" t="s">
         <v>18</v>
       </c>
-      <c r="G6" s="28" t="s">
-        <v>20</v>
-      </c>
-      <c r="H6" s="28" t="s">
-        <v>20</v>
-      </c>
-      <c r="I6" s="29" t="s">
+      <c r="G6" s="30" t="s">
+        <v>20</v>
+      </c>
+      <c r="H6" s="30" t="s">
+        <v>20</v>
+      </c>
+      <c r="I6" s="32" t="s">
         <v>188</v>
       </c>
     </row>
     <row r="7" ht="45" customHeight="1" spans="1:9">
-      <c r="A7" s="24">
+      <c r="A7" s="28">
         <v>3</v>
       </c>
-      <c r="B7" s="24" t="s">
+      <c r="B7" s="28" t="s">
         <v>25</v>
       </c>
-      <c r="C7" s="24" t="s">
+      <c r="C7" s="28" t="s">
         <v>26</v>
       </c>
-      <c r="D7" s="24" t="s">
+      <c r="D7" s="28" t="s">
         <v>27</v>
       </c>
-      <c r="E7" s="24" t="s">
+      <c r="E7" s="28" t="s">
         <v>17</v>
       </c>
-      <c r="F7" s="27" t="s">
+      <c r="F7" s="29" t="s">
         <v>18</v>
       </c>
-      <c r="G7" s="28" t="s">
-        <v>20</v>
-      </c>
-      <c r="H7" s="28" t="s">
-        <v>20</v>
-      </c>
-      <c r="I7" s="29" t="s">
+      <c r="G7" s="30" t="s">
+        <v>20</v>
+      </c>
+      <c r="H7" s="30" t="s">
+        <v>20</v>
+      </c>
+      <c r="I7" s="32" t="s">
         <v>189</v>
       </c>
     </row>
     <row r="8" ht="45" customHeight="1" spans="1:9">
-      <c r="A8" s="24">
+      <c r="A8" s="28">
         <v>4</v>
       </c>
-      <c r="B8" s="24" t="s">
+      <c r="B8" s="28" t="s">
         <v>28</v>
       </c>
-      <c r="C8" s="24" t="s">
+      <c r="C8" s="28" t="s">
         <v>29</v>
       </c>
-      <c r="D8" s="24" t="s">
+      <c r="D8" s="28" t="s">
         <v>30</v>
       </c>
-      <c r="E8" s="24" t="s">
+      <c r="E8" s="28" t="s">
         <v>17</v>
       </c>
-      <c r="F8" s="27" t="s">
+      <c r="F8" s="29" t="s">
         <v>18</v>
       </c>
-      <c r="G8" s="28" t="s">
-        <v>20</v>
-      </c>
-      <c r="H8" s="28" t="s">
-        <v>20</v>
-      </c>
-      <c r="I8" s="29" t="s">
+      <c r="G8" s="30" t="s">
+        <v>20</v>
+      </c>
+      <c r="H8" s="30" t="s">
+        <v>20</v>
+      </c>
+      <c r="I8" s="32" t="s">
         <v>190</v>
       </c>
     </row>
     <row r="9" ht="45" customHeight="1" spans="1:9">
-      <c r="A9" s="24">
+      <c r="A9" s="28">
         <v>5</v>
       </c>
-      <c r="B9" s="24" t="s">
+      <c r="B9" s="28" t="s">
         <v>31</v>
       </c>
-      <c r="C9" s="24" t="s">
+      <c r="C9" s="28" t="s">
         <v>191</v>
       </c>
-      <c r="D9" s="24" t="s">
+      <c r="D9" s="28" t="s">
         <v>192</v>
       </c>
-      <c r="E9" s="24" t="s">
+      <c r="E9" s="28" t="s">
         <v>17</v>
       </c>
-      <c r="F9" s="27" t="s">
+      <c r="F9" s="29" t="s">
         <v>18</v>
       </c>
-      <c r="G9" s="28" t="s">
-        <v>20</v>
-      </c>
-      <c r="H9" s="28" t="s">
-        <v>20</v>
-      </c>
-      <c r="I9" s="29" t="s">
+      <c r="G9" s="30" t="s">
+        <v>20</v>
+      </c>
+      <c r="H9" s="30" t="s">
+        <v>20</v>
+      </c>
+      <c r="I9" s="32" t="s">
         <v>193</v>
       </c>
     </row>
     <row r="10" ht="45" customHeight="1" spans="1:9">
-      <c r="A10" s="21" t="s">
+      <c r="A10" s="23" t="s">
         <v>34</v>
       </c>
-      <c r="B10" s="22"/>
-      <c r="C10" s="22"/>
-      <c r="D10" s="22"/>
-      <c r="E10" s="22"/>
-      <c r="F10" s="30"/>
-      <c r="G10" s="22"/>
-      <c r="H10" s="22"/>
-      <c r="I10" s="31"/>
+      <c r="B10" s="24"/>
+      <c r="C10" s="24"/>
+      <c r="D10" s="24"/>
+      <c r="E10" s="24"/>
+      <c r="F10" s="31"/>
+      <c r="G10" s="24"/>
+      <c r="H10" s="24"/>
+      <c r="I10" s="33"/>
     </row>
     <row r="11" ht="45" customHeight="1" spans="1:9">
       <c r="A11" s="5">
@@ -4131,7 +4122,7 @@
       <c r="E11" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="F11" s="27" t="s">
+      <c r="F11" s="29" t="s">
         <v>194</v>
       </c>
       <c r="G11" s="5" t="s">
@@ -4140,7 +4131,7 @@
       <c r="H11" s="5" t="s">
         <v>20</v>
       </c>
-      <c r="I11" s="32" t="s">
+      <c r="I11" s="34" t="s">
         <v>195</v>
       </c>
     </row>
@@ -4154,13 +4145,13 @@
       <c r="C12" s="6" t="s">
         <v>39</v>
       </c>
-      <c r="D12" s="24" t="s">
+      <c r="D12" s="28" t="s">
         <v>40</v>
       </c>
       <c r="E12" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="F12" s="27" t="s">
+      <c r="F12" s="29" t="s">
         <v>18</v>
       </c>
       <c r="G12" s="5" t="s">
@@ -4169,7 +4160,7 @@
       <c r="H12" s="5" t="s">
         <v>20</v>
       </c>
-      <c r="I12" s="32" t="s">
+      <c r="I12" s="34" t="s">
         <v>196</v>
       </c>
     </row>
@@ -4189,7 +4180,7 @@
       <c r="E13" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="F13" s="27" t="s">
+      <c r="F13" s="29" t="s">
         <v>18</v>
       </c>
       <c r="G13" s="5" t="s">
@@ -4198,7 +4189,7 @@
       <c r="H13" s="5" t="s">
         <v>20</v>
       </c>
-      <c r="I13" s="32" t="s">
+      <c r="I13" s="34" t="s">
         <v>197</v>
       </c>
     </row>
@@ -4218,7 +4209,7 @@
       <c r="E14" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="F14" s="27" t="s">
+      <c r="F14" s="29" t="s">
         <v>18</v>
       </c>
       <c r="G14" s="5" t="s">
@@ -4227,7 +4218,7 @@
       <c r="H14" s="5" t="s">
         <v>20</v>
       </c>
-      <c r="I14" s="32" t="s">
+      <c r="I14" s="34" t="s">
         <v>198</v>
       </c>
     </row>
@@ -4247,7 +4238,7 @@
       <c r="E15" s="5" t="s">
         <v>50</v>
       </c>
-      <c r="F15" s="27" t="s">
+      <c r="F15" s="29" t="s">
         <v>199</v>
       </c>
       <c r="G15" s="5" t="s">
@@ -4256,7 +4247,7 @@
       <c r="H15" s="5" t="s">
         <v>20</v>
       </c>
-      <c r="I15" s="32" t="s">
+      <c r="I15" s="34" t="s">
         <v>200</v>
       </c>
     </row>
@@ -4276,7 +4267,7 @@
       <c r="E16" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="F16" s="27" t="s">
+      <c r="F16" s="29" t="s">
         <v>18</v>
       </c>
       <c r="G16" s="5" t="s">
@@ -4285,7 +4276,7 @@
       <c r="H16" s="5" t="s">
         <v>20</v>
       </c>
-      <c r="I16" s="32" t="s">
+      <c r="I16" s="34" t="s">
         <v>201</v>
       </c>
     </row>
@@ -4305,7 +4296,7 @@
       <c r="E17" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="F17" s="27" t="s">
+      <c r="F17" s="29" t="s">
         <v>194</v>
       </c>
       <c r="G17" s="5" t="s">
@@ -4314,7 +4305,7 @@
       <c r="H17" s="5" t="s">
         <v>20</v>
       </c>
-      <c r="I17" s="32" t="s">
+      <c r="I17" s="34" t="s">
         <v>202</v>
       </c>
     </row>
@@ -4334,7 +4325,7 @@
       <c r="E18" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="F18" s="27" t="s">
+      <c r="F18" s="29" t="s">
         <v>18</v>
       </c>
       <c r="G18" s="5" t="s">
@@ -4343,7 +4334,7 @@
       <c r="H18" s="5" t="s">
         <v>20</v>
       </c>
-      <c r="I18" s="32" t="s">
+      <c r="I18" s="34" t="s">
         <v>203</v>
       </c>
     </row>
@@ -4374,7 +4365,7 @@
   </cols>
   <sheetData>
     <row r="1" ht="38" customHeight="1" spans="1:9">
-      <c r="A1" s="18" t="s">
+      <c r="A1" s="20" t="s">
         <v>204</v>
       </c>
       <c r="B1" s="8"/>
@@ -4387,7 +4378,7 @@
       <c r="I1" s="9"/>
     </row>
     <row r="2" ht="25" customHeight="1" spans="1:9">
-      <c r="A2" s="19" t="s">
+      <c r="A2" s="21" t="s">
         <v>205</v>
       </c>
       <c r="B2" s="8"/>
@@ -4400,36 +4391,36 @@
       <c r="I2" s="9"/>
     </row>
     <row r="3" ht="35" customHeight="1" spans="1:9">
-      <c r="A3" s="20" t="s">
+      <c r="A3" s="22" t="s">
         <v>2</v>
       </c>
-      <c r="B3" s="20" t="s">
+      <c r="B3" s="22" t="s">
         <v>183</v>
       </c>
-      <c r="C3" s="20" t="s">
+      <c r="C3" s="22" t="s">
         <v>4</v>
       </c>
-      <c r="D3" s="20" t="s">
+      <c r="D3" s="22" t="s">
         <v>6</v>
       </c>
-      <c r="E3" s="20" t="s">
+      <c r="E3" s="22" t="s">
         <v>7</v>
       </c>
-      <c r="F3" s="20" t="s">
+      <c r="F3" s="22" t="s">
         <v>8</v>
       </c>
-      <c r="G3" s="20" t="s">
+      <c r="G3" s="22" t="s">
         <v>184</v>
       </c>
-      <c r="H3" s="20" t="s">
+      <c r="H3" s="22" t="s">
         <v>185</v>
       </c>
-      <c r="I3" s="20" t="s">
+      <c r="I3" s="22" t="s">
         <v>186</v>
       </c>
     </row>
     <row r="4" ht="28" customHeight="1" spans="1:9">
-      <c r="A4" s="21" t="s">
+      <c r="A4" s="23" t="s">
         <v>34</v>
       </c>
       <c r="B4" s="8"/>
@@ -4645,7 +4636,7 @@
       </c>
     </row>
     <row r="12" ht="28" customHeight="1" spans="1:9">
-      <c r="A12" s="21" t="s">
+      <c r="A12" s="23" t="s">
         <v>88</v>
       </c>
       <c r="B12" s="8"/>
@@ -4761,7 +4752,7 @@
         <v>93</v>
       </c>
       <c r="F16" s="5" t="s">
-        <v>63</v>
+        <v>18</v>
       </c>
       <c r="G16" s="5" t="s">
         <v>20</v>
@@ -4877,7 +4868,7 @@
         <v>93</v>
       </c>
       <c r="F20" s="5" t="s">
-        <v>63</v>
+        <v>18</v>
       </c>
       <c r="G20" s="5" t="s">
         <v>20</v>
@@ -4906,7 +4897,7 @@
         <v>93</v>
       </c>
       <c r="F21" s="5" t="s">
-        <v>63</v>
+        <v>18</v>
       </c>
       <c r="G21" s="5" t="s">
         <v>20</v>
@@ -4935,7 +4926,7 @@
         <v>93</v>
       </c>
       <c r="F22" s="5" t="s">
-        <v>63</v>
+        <v>18</v>
       </c>
       <c r="G22" s="5" t="s">
         <v>20</v>
@@ -4964,7 +4955,7 @@
         <v>93</v>
       </c>
       <c r="F23" s="5" t="s">
-        <v>63</v>
+        <v>18</v>
       </c>
       <c r="G23" s="5" t="s">
         <v>20</v>
@@ -4977,7 +4968,7 @@
       </c>
     </row>
     <row r="24" ht="28" customHeight="1" spans="1:9">
-      <c r="A24" s="21" t="s">
+      <c r="A24" s="23" t="s">
         <v>118</v>
       </c>
       <c r="B24" s="8"/>
@@ -5135,20 +5126,20 @@
       </c>
     </row>
     <row r="30" ht="45" customHeight="1" spans="1:9">
-      <c r="A30" s="21" t="s">
+      <c r="A30" s="23" t="s">
         <v>136</v>
       </c>
-      <c r="B30" s="22"/>
-      <c r="C30" s="22"/>
-      <c r="D30" s="22"/>
-      <c r="E30" s="22"/>
-      <c r="F30" s="22"/>
-      <c r="G30" s="22"/>
-      <c r="H30" s="22"/>
-      <c r="I30" s="23"/>
+      <c r="B30" s="24"/>
+      <c r="C30" s="24"/>
+      <c r="D30" s="24"/>
+      <c r="E30" s="24"/>
+      <c r="F30" s="24"/>
+      <c r="G30" s="24"/>
+      <c r="H30" s="24"/>
+      <c r="I30" s="26"/>
     </row>
     <row r="31" ht="28" customHeight="1" spans="1:9">
-      <c r="A31" s="24">
+      <c r="A31" s="25">
         <v>24</v>
       </c>
       <c r="B31" s="25" t="s">
@@ -5160,19 +5151,19 @@
       <c r="D31" s="25" t="s">
         <v>140</v>
       </c>
-      <c r="E31" s="25" t="s">
+      <c r="E31" s="5" t="s">
         <v>141</v>
       </c>
-      <c r="F31" s="25" t="s">
-        <v>63</v>
-      </c>
-      <c r="G31" s="25" t="s">
-        <v>20</v>
-      </c>
-      <c r="H31" s="25" t="s">
-        <v>20</v>
-      </c>
-      <c r="I31" s="25" t="s">
+      <c r="F31" s="5" t="s">
+        <v>63</v>
+      </c>
+      <c r="G31" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="H31" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="I31" s="5" t="s">
         <v>20</v>
       </c>
     </row>
@@ -5351,7 +5342,7 @@
   </cols>
   <sheetData>
     <row r="1" ht="38" customHeight="1" spans="1:9">
-      <c r="A1" s="18" t="s">
+      <c r="A1" s="20" t="s">
         <v>206</v>
       </c>
       <c r="B1" s="8"/>
@@ -5364,7 +5355,7 @@
       <c r="I1" s="9"/>
     </row>
     <row r="2" ht="25" customHeight="1" spans="1:9">
-      <c r="A2" s="19" t="s">
+      <c r="A2" s="21" t="s">
         <v>207</v>
       </c>
       <c r="B2" s="8"/>
@@ -5377,36 +5368,36 @@
       <c r="I2" s="9"/>
     </row>
     <row r="3" ht="35" customHeight="1" spans="1:9">
-      <c r="A3" s="20" t="s">
+      <c r="A3" s="22" t="s">
         <v>2</v>
       </c>
-      <c r="B3" s="20" t="s">
+      <c r="B3" s="22" t="s">
         <v>183</v>
       </c>
-      <c r="C3" s="20" t="s">
+      <c r="C3" s="22" t="s">
         <v>4</v>
       </c>
-      <c r="D3" s="20" t="s">
+      <c r="D3" s="22" t="s">
         <v>6</v>
       </c>
-      <c r="E3" s="20" t="s">
+      <c r="E3" s="22" t="s">
         <v>7</v>
       </c>
-      <c r="F3" s="20" t="s">
+      <c r="F3" s="22" t="s">
         <v>8</v>
       </c>
-      <c r="G3" s="20" t="s">
+      <c r="G3" s="22" t="s">
         <v>184</v>
       </c>
-      <c r="H3" s="20" t="s">
+      <c r="H3" s="22" t="s">
         <v>185</v>
       </c>
-      <c r="I3" s="20" t="s">
+      <c r="I3" s="22" t="s">
         <v>186</v>
       </c>
     </row>
     <row r="4" ht="28" customHeight="1" spans="1:9">
-      <c r="A4" s="21" t="s">
+      <c r="A4" s="23" t="s">
         <v>34</v>
       </c>
       <c r="B4" s="8"/>
@@ -5477,7 +5468,7 @@
       </c>
     </row>
     <row r="7" ht="28" customHeight="1" spans="1:9">
-      <c r="A7" s="21" t="s">
+      <c r="A7" s="23" t="s">
         <v>136</v>
       </c>
       <c r="B7" s="8"/>
@@ -5548,7 +5539,7 @@
       </c>
     </row>
     <row r="10" ht="28" customHeight="1" spans="1:9">
-      <c r="A10" s="21" t="s">
+      <c r="A10" s="23" t="s">
         <v>161</v>
       </c>
       <c r="B10" s="8"/>
@@ -5762,7 +5753,7 @@
     <col min="6" max="6" width="30" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="35" customHeight="1" spans="1:6">
+    <row r="1" ht="35" customHeight="1" spans="1:1">
       <c r="A1" s="1" t="s">
         <v>208</v>
       </c>
@@ -5897,7 +5888,7 @@
       <c r="E10" s="8"/>
       <c r="F10" s="9"/>
     </row>
-    <row r="11" spans="1:6">
+    <row r="11" spans="1:3">
       <c r="A11" s="10" t="s">
         <v>19</v>
       </c>
@@ -5908,7 +5899,7 @@
         <v>234</v>
       </c>
     </row>
-    <row r="12" ht="26.4" customHeight="1" spans="1:6">
+    <row r="12" ht="26.4" customHeight="1" spans="1:3">
       <c r="A12" s="11" t="s">
         <v>64</v>
       </c>
@@ -5919,7 +5910,7 @@
         <v>236</v>
       </c>
     </row>
-    <row r="13" spans="1:6">
+    <row r="13" spans="1:3">
       <c r="A13" s="12" t="s">
         <v>84</v>
       </c>
@@ -5930,126 +5921,120 @@
         <v>238</v>
       </c>
     </row>
-    <row r="14" spans="1:6">
-      <c r="A14" s="13" t="s">
-        <v>239</v>
-      </c>
-      <c r="B14" s="6" t="s">
-        <v>240</v>
-      </c>
-      <c r="C14" s="5" t="s">
-        <v>241</v>
-      </c>
-    </row>
-    <row r="16" spans="1:6">
-      <c r="A16" s="14"/>
+    <row r="14" spans="1:3">
+      <c r="A14" s="13"/>
+      <c r="B14" s="14"/>
+      <c r="C14" s="15"/>
+    </row>
+    <row r="16" spans="1:1">
+      <c r="A16" s="16"/>
     </row>
     <row r="17" spans="1:6">
-      <c r="A17" s="15"/>
-      <c r="B17" s="16"/>
-      <c r="C17" s="17"/>
-      <c r="D17" s="17"/>
-      <c r="E17" s="17"/>
-      <c r="F17" s="17"/>
+      <c r="A17" s="17"/>
+      <c r="B17" s="18"/>
+      <c r="C17" s="19"/>
+      <c r="D17" s="19"/>
+      <c r="E17" s="19"/>
+      <c r="F17" s="19"/>
     </row>
     <row r="18" spans="1:6">
-      <c r="A18" s="15"/>
-      <c r="B18" s="16"/>
-      <c r="C18" s="17"/>
-      <c r="D18" s="17"/>
-      <c r="E18" s="17"/>
-      <c r="F18" s="17"/>
+      <c r="A18" s="17"/>
+      <c r="B18" s="18"/>
+      <c r="C18" s="19"/>
+      <c r="D18" s="19"/>
+      <c r="E18" s="19"/>
+      <c r="F18" s="19"/>
     </row>
     <row r="19" spans="1:6">
-      <c r="A19" s="15"/>
-      <c r="B19" s="16"/>
-      <c r="C19" s="17"/>
-      <c r="D19" s="17"/>
-      <c r="E19" s="17"/>
-      <c r="F19" s="17"/>
+      <c r="A19" s="17"/>
+      <c r="B19" s="18"/>
+      <c r="C19" s="19"/>
+      <c r="D19" s="19"/>
+      <c r="E19" s="19"/>
+      <c r="F19" s="19"/>
     </row>
     <row r="20" spans="1:6">
-      <c r="A20" s="15"/>
-      <c r="B20" s="16"/>
-      <c r="C20" s="17"/>
-      <c r="D20" s="17"/>
-      <c r="E20" s="17"/>
-      <c r="F20" s="17"/>
+      <c r="A20" s="17"/>
+      <c r="B20" s="18"/>
+      <c r="C20" s="19"/>
+      <c r="D20" s="19"/>
+      <c r="E20" s="19"/>
+      <c r="F20" s="19"/>
     </row>
     <row r="21" spans="1:6">
-      <c r="A21" s="15"/>
-      <c r="B21" s="16"/>
-      <c r="C21" s="17"/>
-      <c r="D21" s="17"/>
-      <c r="E21" s="17"/>
-      <c r="F21" s="17"/>
+      <c r="A21" s="17"/>
+      <c r="B21" s="18"/>
+      <c r="C21" s="19"/>
+      <c r="D21" s="19"/>
+      <c r="E21" s="19"/>
+      <c r="F21" s="19"/>
     </row>
     <row r="22" spans="1:6">
-      <c r="A22" s="15"/>
-      <c r="B22" s="16"/>
-      <c r="C22" s="17"/>
-      <c r="D22" s="17"/>
-      <c r="E22" s="17"/>
-      <c r="F22" s="17"/>
+      <c r="A22" s="17"/>
+      <c r="B22" s="18"/>
+      <c r="C22" s="19"/>
+      <c r="D22" s="19"/>
+      <c r="E22" s="19"/>
+      <c r="F22" s="19"/>
     </row>
     <row r="23" spans="1:6">
-      <c r="A23" s="17"/>
-      <c r="B23" s="17"/>
-      <c r="C23" s="17"/>
-      <c r="D23" s="17"/>
-      <c r="E23" s="17"/>
-      <c r="F23" s="17"/>
-    </row>
-    <row r="24" spans="1:6">
-      <c r="A24" s="14"/>
+      <c r="A23" s="19"/>
+      <c r="B23" s="19"/>
+      <c r="C23" s="19"/>
+      <c r="D23" s="19"/>
+      <c r="E23" s="19"/>
+      <c r="F23" s="19"/>
+    </row>
+    <row r="24" spans="1:1">
+      <c r="A24" s="16"/>
     </row>
     <row r="25" spans="1:6">
-      <c r="A25" s="15"/>
-      <c r="B25" s="16"/>
-      <c r="C25" s="17"/>
-      <c r="D25" s="17"/>
-      <c r="E25" s="17"/>
-      <c r="F25" s="17"/>
+      <c r="A25" s="17"/>
+      <c r="B25" s="18"/>
+      <c r="C25" s="19"/>
+      <c r="D25" s="19"/>
+      <c r="E25" s="19"/>
+      <c r="F25" s="19"/>
     </row>
     <row r="26" spans="1:6">
-      <c r="A26" s="15"/>
-      <c r="B26" s="16"/>
-      <c r="C26" s="17"/>
-      <c r="D26" s="17"/>
-      <c r="E26" s="17"/>
-      <c r="F26" s="17"/>
+      <c r="A26" s="17"/>
+      <c r="B26" s="18"/>
+      <c r="C26" s="19"/>
+      <c r="D26" s="19"/>
+      <c r="E26" s="19"/>
+      <c r="F26" s="19"/>
     </row>
     <row r="27" spans="1:6">
-      <c r="A27" s="15"/>
-      <c r="B27" s="16"/>
-      <c r="C27" s="17"/>
-      <c r="D27" s="17"/>
-      <c r="E27" s="17"/>
-      <c r="F27" s="17"/>
+      <c r="A27" s="17"/>
+      <c r="B27" s="18"/>
+      <c r="C27" s="19"/>
+      <c r="D27" s="19"/>
+      <c r="E27" s="19"/>
+      <c r="F27" s="19"/>
     </row>
     <row r="28" spans="1:6">
-      <c r="A28" s="15"/>
-      <c r="B28" s="16"/>
-      <c r="C28" s="17"/>
-      <c r="D28" s="17"/>
-      <c r="E28" s="17"/>
-      <c r="F28" s="17"/>
+      <c r="A28" s="17"/>
+      <c r="B28" s="18"/>
+      <c r="C28" s="19"/>
+      <c r="D28" s="19"/>
+      <c r="E28" s="19"/>
+      <c r="F28" s="19"/>
     </row>
     <row r="29" spans="1:6">
-      <c r="A29" s="15"/>
-      <c r="B29" s="16"/>
-      <c r="C29" s="17"/>
-      <c r="D29" s="17"/>
-      <c r="E29" s="17"/>
-      <c r="F29" s="17"/>
+      <c r="A29" s="17"/>
+      <c r="B29" s="18"/>
+      <c r="C29" s="19"/>
+      <c r="D29" s="19"/>
+      <c r="E29" s="19"/>
+      <c r="F29" s="19"/>
     </row>
     <row r="30" spans="1:6">
-      <c r="A30" s="17"/>
-      <c r="B30" s="17"/>
-      <c r="C30" s="17"/>
-      <c r="D30" s="17"/>
-      <c r="E30" s="17"/>
-      <c r="F30" s="17"/>
+      <c r="A30" s="19"/>
+      <c r="B30" s="19"/>
+      <c r="C30" s="19"/>
+      <c r="D30" s="19"/>
+      <c r="E30" s="19"/>
+      <c r="F30" s="19"/>
     </row>
   </sheetData>
   <mergeCells count="4">

</xml_diff>

<commit_message>
Đã xong chức năng lịch trình và phân công
</commit_message>
<xml_diff>
--- a/Project_Tracking.xlsx
+++ b/Project_Tracking.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="23040" windowHeight="9707" activeTab="2"/>
+    <workbookView windowWidth="16608" windowHeight="9240" activeTab="2"/>
   </bookViews>
   <sheets>
     <sheet name="Project Tracking" sheetId="1" r:id="rId1"/>
@@ -945,7 +945,7 @@
       <charset val="134"/>
     </font>
   </fonts>
-  <fills count="39">
+  <fills count="40">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -991,6 +991,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FF0070C0"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.4"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -1374,7 +1380,7 @@
     <xf numFmtId="0" fontId="13" fillId="0" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="6">
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="6">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="14" fillId="0" borderId="0">
@@ -1398,16 +1404,16 @@
     <xf numFmtId="0" fontId="19" fillId="0" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="10" borderId="9">
+    <xf numFmtId="0" fontId="20" fillId="11" borderId="9">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="11" borderId="10">
+    <xf numFmtId="0" fontId="21" fillId="12" borderId="10">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="11" borderId="9">
+    <xf numFmtId="0" fontId="22" fillId="12" borderId="9">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="23" fillId="12" borderId="11">
+    <xf numFmtId="0" fontId="23" fillId="13" borderId="11">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="24" fillId="0" borderId="12">
@@ -1419,86 +1425,86 @@
     <xf numFmtId="0" fontId="25" fillId="4" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="26" fillId="13" borderId="0">
+    <xf numFmtId="0" fontId="26" fillId="14" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="27" fillId="14" borderId="0">
+    <xf numFmtId="0" fontId="27" fillId="15" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="15" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="16" borderId="0">
+    <xf numFmtId="0" fontId="8" fillId="16" borderId="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="17" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="18" borderId="0">
+    <xf numFmtId="0" fontId="0" fillId="18" borderId="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="19" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="20" borderId="0">
+    <xf numFmtId="0" fontId="8" fillId="20" borderId="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="21" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="22" borderId="0">
+    <xf numFmtId="0" fontId="0" fillId="22" borderId="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="23" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="24" borderId="0">
+    <xf numFmtId="0" fontId="8" fillId="24" borderId="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="25" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="26" borderId="0">
+    <xf numFmtId="0" fontId="0" fillId="26" borderId="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="27" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="28" borderId="0">
+    <xf numFmtId="0" fontId="8" fillId="28" borderId="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="29" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="30" borderId="0">
+    <xf numFmtId="0" fontId="0" fillId="30" borderId="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="31" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="32" borderId="0">
+    <xf numFmtId="0" fontId="8" fillId="32" borderId="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="33" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="34" borderId="0">
+    <xf numFmtId="0" fontId="0" fillId="34" borderId="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="35" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="36" borderId="0">
+    <xf numFmtId="0" fontId="8" fillId="36" borderId="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="37" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="38" borderId="0">
+    <xf numFmtId="0" fontId="0" fillId="38" borderId="0">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="8" fillId="39" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
   </cellStyleXfs>
-  <cellXfs count="42">
+  <cellXfs count="43">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -1560,6 +1566,9 @@
     </xf>
     <xf numFmtId="0" fontId="2" fillId="8" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="9" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="8" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
@@ -2067,13 +2076,13 @@
     <col min="4" max="4" width="22" customWidth="1"/>
     <col min="5" max="5" width="60" customWidth="1"/>
     <col min="6" max="7" width="14" customWidth="1"/>
-    <col min="8" max="8" width="10" style="36" customWidth="1"/>
+    <col min="8" max="8" width="10" style="37" customWidth="1"/>
     <col min="9" max="9" width="14" customWidth="1"/>
     <col min="10" max="10" width="30" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" ht="40" customHeight="1" spans="1:10">
-      <c r="A1" s="37" t="s">
+      <c r="A1" s="38" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="8"/>
@@ -2082,7 +2091,7 @@
       <c r="E1" s="8"/>
       <c r="F1" s="8"/>
       <c r="G1" s="8"/>
-      <c r="H1" s="38"/>
+      <c r="H1" s="39"/>
       <c r="I1" s="8"/>
       <c r="J1" s="9"/>
     </row>
@@ -2096,7 +2105,7 @@
       <c r="E2" s="8"/>
       <c r="F2" s="8"/>
       <c r="G2" s="8"/>
-      <c r="H2" s="38"/>
+      <c r="H2" s="39"/>
       <c r="I2" s="8"/>
       <c r="J2" s="9"/>
     </row>
@@ -2132,26 +2141,26 @@
         <v>11</v>
       </c>
     </row>
-    <row r="4" s="35" customFormat="1" ht="28" customHeight="1" spans="1:8">
-      <c r="A4" s="27" t="s">
+    <row r="4" s="36" customFormat="1" ht="28" customHeight="1" spans="1:8">
+      <c r="A4" s="28" t="s">
         <v>12</v>
       </c>
-      <c r="H4" s="39"/>
+      <c r="H4" s="40"/>
     </row>
     <row r="5" ht="45" customHeight="1" spans="1:10">
-      <c r="A5" s="25">
+      <c r="A5" s="26">
         <v>1</v>
       </c>
-      <c r="B5" s="25" t="s">
+      <c r="B5" s="26" t="s">
         <v>13</v>
       </c>
-      <c r="C5" s="25" t="s">
+      <c r="C5" s="26" t="s">
         <v>14</v>
       </c>
-      <c r="D5" s="25" t="s">
+      <c r="D5" s="26" t="s">
         <v>15</v>
       </c>
-      <c r="E5" s="25" t="s">
+      <c r="E5" s="26" t="s">
         <v>16</v>
       </c>
       <c r="F5" s="5" t="s">
@@ -2160,28 +2169,28 @@
       <c r="G5" s="5" t="s">
         <v>18</v>
       </c>
-      <c r="H5" s="40" t="s">
+      <c r="H5" s="41" t="s">
         <v>19</v>
       </c>
-      <c r="I5" s="28"/>
+      <c r="I5" s="29"/>
       <c r="J5" s="5" t="s">
         <v>20</v>
       </c>
     </row>
     <row r="6" ht="45" customHeight="1" spans="1:10">
-      <c r="A6" s="25">
+      <c r="A6" s="26">
         <v>2</v>
       </c>
-      <c r="B6" s="25" t="s">
+      <c r="B6" s="26" t="s">
         <v>21</v>
       </c>
-      <c r="C6" s="25" t="s">
+      <c r="C6" s="26" t="s">
         <v>22</v>
       </c>
-      <c r="D6" s="25" t="s">
+      <c r="D6" s="26" t="s">
         <v>23</v>
       </c>
-      <c r="E6" s="25" t="s">
+      <c r="E6" s="26" t="s">
         <v>24</v>
       </c>
       <c r="F6" s="5" t="s">
@@ -2190,28 +2199,28 @@
       <c r="G6" s="5" t="s">
         <v>18</v>
       </c>
-      <c r="H6" s="40" t="s">
+      <c r="H6" s="41" t="s">
         <v>19</v>
       </c>
-      <c r="I6" s="28"/>
+      <c r="I6" s="29"/>
       <c r="J6" s="5" t="s">
         <v>20</v>
       </c>
     </row>
     <row r="7" ht="45" customHeight="1" spans="1:10">
-      <c r="A7" s="25">
+      <c r="A7" s="26">
         <v>3</v>
       </c>
-      <c r="B7" s="25" t="s">
+      <c r="B7" s="26" t="s">
         <v>25</v>
       </c>
-      <c r="C7" s="25" t="s">
+      <c r="C7" s="26" t="s">
         <v>26</v>
       </c>
-      <c r="D7" s="25" t="s">
+      <c r="D7" s="26" t="s">
         <v>15</v>
       </c>
-      <c r="E7" s="25" t="s">
+      <c r="E7" s="26" t="s">
         <v>27</v>
       </c>
       <c r="F7" s="5" t="s">
@@ -2220,28 +2229,28 @@
       <c r="G7" s="5" t="s">
         <v>18</v>
       </c>
-      <c r="H7" s="40" t="s">
+      <c r="H7" s="41" t="s">
         <v>19</v>
       </c>
-      <c r="I7" s="28"/>
+      <c r="I7" s="29"/>
       <c r="J7" s="5" t="s">
         <v>20</v>
       </c>
     </row>
     <row r="8" ht="45" customHeight="1" spans="1:10">
-      <c r="A8" s="25">
+      <c r="A8" s="26">
         <v>4</v>
       </c>
-      <c r="B8" s="25" t="s">
+      <c r="B8" s="26" t="s">
         <v>28</v>
       </c>
-      <c r="C8" s="25" t="s">
+      <c r="C8" s="26" t="s">
         <v>29</v>
       </c>
-      <c r="D8" s="25" t="s">
+      <c r="D8" s="26" t="s">
         <v>15</v>
       </c>
-      <c r="E8" s="25" t="s">
+      <c r="E8" s="26" t="s">
         <v>30</v>
       </c>
       <c r="F8" s="5" t="s">
@@ -2250,28 +2259,28 @@
       <c r="G8" s="5" t="s">
         <v>18</v>
       </c>
-      <c r="H8" s="40" t="s">
+      <c r="H8" s="41" t="s">
         <v>19</v>
       </c>
-      <c r="I8" s="28"/>
+      <c r="I8" s="29"/>
       <c r="J8" s="5" t="s">
         <v>20</v>
       </c>
     </row>
     <row r="9" ht="45" customHeight="1" spans="1:10">
-      <c r="A9" s="25">
+      <c r="A9" s="26">
         <v>5</v>
       </c>
-      <c r="B9" s="25" t="s">
+      <c r="B9" s="26" t="s">
         <v>31</v>
       </c>
-      <c r="C9" s="25" t="s">
+      <c r="C9" s="26" t="s">
         <v>32</v>
       </c>
-      <c r="D9" s="25" t="s">
+      <c r="D9" s="26" t="s">
         <v>15</v>
       </c>
-      <c r="E9" s="25" t="s">
+      <c r="E9" s="26" t="s">
         <v>33</v>
       </c>
       <c r="F9" s="5" t="s">
@@ -2280,10 +2289,10 @@
       <c r="G9" s="5" t="s">
         <v>18</v>
       </c>
-      <c r="H9" s="40" t="s">
+      <c r="H9" s="41" t="s">
         <v>19</v>
       </c>
-      <c r="I9" s="28"/>
+      <c r="I9" s="29"/>
       <c r="J9" s="5" t="s">
         <v>20</v>
       </c>
@@ -2292,15 +2301,15 @@
       <c r="A10" s="23" t="s">
         <v>34</v>
       </c>
-      <c r="B10" s="24"/>
-      <c r="C10" s="24"/>
-      <c r="D10" s="24"/>
-      <c r="E10" s="24"/>
-      <c r="F10" s="24"/>
-      <c r="G10" s="24"/>
-      <c r="H10" s="24"/>
-      <c r="I10" s="24"/>
-      <c r="J10" s="41"/>
+      <c r="B10" s="25"/>
+      <c r="C10" s="25"/>
+      <c r="D10" s="25"/>
+      <c r="E10" s="25"/>
+      <c r="F10" s="25"/>
+      <c r="G10" s="25"/>
+      <c r="H10" s="25"/>
+      <c r="I10" s="25"/>
+      <c r="J10" s="42"/>
     </row>
     <row r="11" ht="45" customHeight="1" spans="1:10">
       <c r="A11" s="5">
@@ -2324,7 +2333,7 @@
       <c r="G11" s="5" t="s">
         <v>18</v>
       </c>
-      <c r="H11" s="40" t="s">
+      <c r="H11" s="41" t="s">
         <v>19</v>
       </c>
       <c r="I11" s="5" t="s">
@@ -2356,7 +2365,7 @@
       <c r="G12" s="5" t="s">
         <v>18</v>
       </c>
-      <c r="H12" s="40" t="s">
+      <c r="H12" s="41" t="s">
         <v>19</v>
       </c>
       <c r="I12" s="5" t="s">
@@ -2388,7 +2397,7 @@
       <c r="G13" s="5" t="s">
         <v>18</v>
       </c>
-      <c r="H13" s="40" t="s">
+      <c r="H13" s="41" t="s">
         <v>19</v>
       </c>
       <c r="I13" s="5" t="s">
@@ -2420,7 +2429,7 @@
       <c r="G14" s="5" t="s">
         <v>18</v>
       </c>
-      <c r="H14" s="40" t="s">
+      <c r="H14" s="41" t="s">
         <v>19</v>
       </c>
       <c r="I14" s="5" t="s">
@@ -2452,7 +2461,7 @@
       <c r="G15" s="5" t="s">
         <v>18</v>
       </c>
-      <c r="H15" s="40" t="s">
+      <c r="H15" s="41" t="s">
         <v>19</v>
       </c>
       <c r="I15" s="5" t="s">
@@ -2484,7 +2493,7 @@
       <c r="G16" s="5" t="s">
         <v>18</v>
       </c>
-      <c r="H16" s="40" t="s">
+      <c r="H16" s="41" t="s">
         <v>19</v>
       </c>
       <c r="I16" s="5" t="s">
@@ -2516,7 +2525,7 @@
       <c r="G17" s="5" t="s">
         <v>18</v>
       </c>
-      <c r="H17" s="40" t="s">
+      <c r="H17" s="41" t="s">
         <v>19</v>
       </c>
       <c r="I17" s="5" t="s">
@@ -2548,7 +2557,7 @@
       <c r="G18" s="5" t="s">
         <v>18</v>
       </c>
-      <c r="H18" s="40" t="s">
+      <c r="H18" s="41" t="s">
         <v>19</v>
       </c>
       <c r="I18" s="5" t="s">
@@ -2580,7 +2589,7 @@
       <c r="G19" s="5" t="s">
         <v>63</v>
       </c>
-      <c r="H19" s="40" t="s">
+      <c r="H19" s="41" t="s">
         <v>64</v>
       </c>
       <c r="I19" s="5" t="s">
@@ -2612,7 +2621,7 @@
       <c r="G20" s="5" t="s">
         <v>63</v>
       </c>
-      <c r="H20" s="40" t="s">
+      <c r="H20" s="41" t="s">
         <v>64</v>
       </c>
       <c r="I20" s="5" t="s">
@@ -2644,7 +2653,7 @@
       <c r="G21" s="5" t="s">
         <v>63</v>
       </c>
-      <c r="H21" s="40" t="s">
+      <c r="H21" s="41" t="s">
         <v>64</v>
       </c>
       <c r="I21" s="5" t="s">
@@ -2654,7 +2663,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="22" s="35" customFormat="1" ht="28" customHeight="1" spans="1:10">
+    <row r="22" s="36" customFormat="1" ht="28" customHeight="1" spans="1:10">
       <c r="A22" s="6">
         <v>17</v>
       </c>
@@ -2676,7 +2685,7 @@
       <c r="G22" s="5" t="s">
         <v>63</v>
       </c>
-      <c r="H22" s="40" t="s">
+      <c r="H22" s="41" t="s">
         <v>64</v>
       </c>
       <c r="I22" s="5" t="s">
@@ -2708,7 +2717,7 @@
       <c r="G23" s="5" t="s">
         <v>63</v>
       </c>
-      <c r="H23" s="40" t="s">
+      <c r="H23" s="41" t="s">
         <v>64</v>
       </c>
       <c r="I23" s="5" t="s">
@@ -2740,7 +2749,7 @@
       <c r="G24" s="5" t="s">
         <v>63</v>
       </c>
-      <c r="H24" s="40" t="s">
+      <c r="H24" s="41" t="s">
         <v>64</v>
       </c>
       <c r="I24" s="5" t="s">
@@ -2772,7 +2781,7 @@
       <c r="G25" s="5" t="s">
         <v>63</v>
       </c>
-      <c r="H25" s="40" t="s">
+      <c r="H25" s="41" t="s">
         <v>64</v>
       </c>
       <c r="I25" s="5" t="s">
@@ -2804,7 +2813,7 @@
       <c r="G26" s="5" t="s">
         <v>63</v>
       </c>
-      <c r="H26" s="40" t="s">
+      <c r="H26" s="41" t="s">
         <v>84</v>
       </c>
       <c r="I26" s="5" t="s">
@@ -2836,7 +2845,7 @@
       <c r="G27" s="5" t="s">
         <v>63</v>
       </c>
-      <c r="H27" s="40" t="s">
+      <c r="H27" s="41" t="s">
         <v>84</v>
       </c>
       <c r="I27" s="5" t="s">
@@ -2850,15 +2859,15 @@
       <c r="A28" s="23" t="s">
         <v>88</v>
       </c>
-      <c r="B28" s="24"/>
-      <c r="C28" s="24"/>
-      <c r="D28" s="24"/>
-      <c r="E28" s="24"/>
-      <c r="F28" s="24"/>
-      <c r="G28" s="24"/>
-      <c r="H28" s="24"/>
-      <c r="I28" s="24"/>
-      <c r="J28" s="41"/>
+      <c r="B28" s="25"/>
+      <c r="C28" s="25"/>
+      <c r="D28" s="25"/>
+      <c r="E28" s="25"/>
+      <c r="F28" s="25"/>
+      <c r="G28" s="25"/>
+      <c r="H28" s="25"/>
+      <c r="I28" s="25"/>
+      <c r="J28" s="42"/>
     </row>
     <row r="29" ht="45" customHeight="1" spans="1:10">
       <c r="A29" s="5">
@@ -2882,7 +2891,7 @@
       <c r="G29" s="5" t="s">
         <v>63</v>
       </c>
-      <c r="H29" s="40" t="s">
+      <c r="H29" s="41" t="s">
         <v>64</v>
       </c>
       <c r="I29" s="5" t="s">
@@ -2914,7 +2923,7 @@
       <c r="G30" s="5" t="s">
         <v>63</v>
       </c>
-      <c r="H30" s="40" t="s">
+      <c r="H30" s="41" t="s">
         <v>64</v>
       </c>
       <c r="I30" s="5" t="s">
@@ -2946,7 +2955,7 @@
       <c r="G31" s="5" t="s">
         <v>63</v>
       </c>
-      <c r="H31" s="40" t="s">
+      <c r="H31" s="41" t="s">
         <v>64</v>
       </c>
       <c r="I31" s="5" t="s">
@@ -2978,7 +2987,7 @@
       <c r="G32" s="5" t="s">
         <v>63</v>
       </c>
-      <c r="H32" s="40" t="s">
+      <c r="H32" s="41" t="s">
         <v>64</v>
       </c>
       <c r="I32" s="5" t="s">
@@ -3010,7 +3019,7 @@
       <c r="G33" s="5" t="s">
         <v>63</v>
       </c>
-      <c r="H33" s="40" t="s">
+      <c r="H33" s="41" t="s">
         <v>64</v>
       </c>
       <c r="I33" s="5" t="s">
@@ -3020,20 +3029,20 @@
         <v>20</v>
       </c>
     </row>
-    <row r="34" s="35" customFormat="1" ht="38" customHeight="1" spans="1:10">
+    <row r="34" s="36" customFormat="1" ht="38" customHeight="1" spans="1:10">
       <c r="A34" s="5">
         <v>28</v>
       </c>
       <c r="B34" s="5" t="s">
         <v>103</v>
       </c>
-      <c r="C34" s="25" t="s">
+      <c r="C34" s="26" t="s">
         <v>104</v>
       </c>
-      <c r="D34" s="25" t="s">
+      <c r="D34" s="26" t="s">
         <v>91</v>
       </c>
-      <c r="E34" s="25" t="s">
+      <c r="E34" s="26" t="s">
         <v>105</v>
       </c>
       <c r="F34" s="5" t="s">
@@ -3042,7 +3051,7 @@
       <c r="G34" s="5" t="s">
         <v>63</v>
       </c>
-      <c r="H34" s="40" t="s">
+      <c r="H34" s="41" t="s">
         <v>64</v>
       </c>
       <c r="I34" s="5" t="s">
@@ -3074,7 +3083,7 @@
       <c r="G35" s="5" t="s">
         <v>18</v>
       </c>
-      <c r="H35" s="40" t="s">
+      <c r="H35" s="41" t="s">
         <v>64</v>
       </c>
       <c r="I35" s="5" t="s">
@@ -3106,7 +3115,7 @@
       <c r="G36" s="5" t="s">
         <v>18</v>
       </c>
-      <c r="H36" s="40" t="s">
+      <c r="H36" s="41" t="s">
         <v>64</v>
       </c>
       <c r="I36" s="5" t="s">
@@ -3138,7 +3147,7 @@
       <c r="G37" s="5" t="s">
         <v>18</v>
       </c>
-      <c r="H37" s="40" t="s">
+      <c r="H37" s="41" t="s">
         <v>64</v>
       </c>
       <c r="I37" s="5" t="s">
@@ -3170,7 +3179,7 @@
       <c r="G38" s="5" t="s">
         <v>18</v>
       </c>
-      <c r="H38" s="40" t="s">
+      <c r="H38" s="41" t="s">
         <v>64</v>
       </c>
       <c r="I38" s="5" t="s">
@@ -3202,7 +3211,7 @@
       <c r="G39" s="5" t="s">
         <v>18</v>
       </c>
-      <c r="H39" s="40" t="s">
+      <c r="H39" s="41" t="s">
         <v>64</v>
       </c>
       <c r="I39" s="5" t="s">
@@ -3216,17 +3225,17 @@
       <c r="A40" s="23" t="s">
         <v>118</v>
       </c>
-      <c r="B40" s="24"/>
-      <c r="C40" s="24"/>
-      <c r="D40" s="24"/>
-      <c r="E40" s="24"/>
-      <c r="F40" s="24"/>
-      <c r="G40" s="24"/>
-      <c r="H40" s="24"/>
-      <c r="I40" s="24"/>
-      <c r="J40" s="41"/>
-    </row>
-    <row r="41" s="35" customFormat="1" ht="46" customHeight="1" spans="1:10">
+      <c r="B40" s="25"/>
+      <c r="C40" s="25"/>
+      <c r="D40" s="25"/>
+      <c r="E40" s="25"/>
+      <c r="F40" s="25"/>
+      <c r="G40" s="25"/>
+      <c r="H40" s="25"/>
+      <c r="I40" s="25"/>
+      <c r="J40" s="42"/>
+    </row>
+    <row r="41" s="36" customFormat="1" ht="46" customHeight="1" spans="1:10">
       <c r="A41" s="6">
         <v>34</v>
       </c>
@@ -3248,7 +3257,7 @@
       <c r="G41" s="5" t="s">
         <v>63</v>
       </c>
-      <c r="H41" s="40" t="s">
+      <c r="H41" s="41" t="s">
         <v>64</v>
       </c>
       <c r="I41" s="5" t="s">
@@ -3280,7 +3289,7 @@
       <c r="G42" s="5" t="s">
         <v>63</v>
       </c>
-      <c r="H42" s="40" t="s">
+      <c r="H42" s="41" t="s">
         <v>64</v>
       </c>
       <c r="I42" s="5" t="s">
@@ -3312,7 +3321,7 @@
       <c r="G43" s="5" t="s">
         <v>63</v>
       </c>
-      <c r="H43" s="40" t="s">
+      <c r="H43" s="41" t="s">
         <v>64</v>
       </c>
       <c r="I43" s="5" t="s">
@@ -3344,7 +3353,7 @@
       <c r="G44" s="5" t="s">
         <v>63</v>
       </c>
-      <c r="H44" s="40" t="s">
+      <c r="H44" s="41" t="s">
         <v>64</v>
       </c>
       <c r="I44" s="5" t="s">
@@ -3376,7 +3385,7 @@
       <c r="G45" s="5" t="s">
         <v>63</v>
       </c>
-      <c r="H45" s="40" t="s">
+      <c r="H45" s="41" t="s">
         <v>64</v>
       </c>
       <c r="I45" s="5" t="s">
@@ -3390,15 +3399,15 @@
       <c r="A46" s="23" t="s">
         <v>136</v>
       </c>
-      <c r="B46" s="24"/>
-      <c r="C46" s="24"/>
-      <c r="D46" s="24"/>
-      <c r="E46" s="24"/>
-      <c r="F46" s="24"/>
-      <c r="G46" s="24"/>
-      <c r="H46" s="24"/>
-      <c r="I46" s="24"/>
-      <c r="J46" s="41"/>
+      <c r="B46" s="25"/>
+      <c r="C46" s="25"/>
+      <c r="D46" s="25"/>
+      <c r="E46" s="25"/>
+      <c r="F46" s="25"/>
+      <c r="G46" s="25"/>
+      <c r="H46" s="25"/>
+      <c r="I46" s="25"/>
+      <c r="J46" s="42"/>
     </row>
     <row r="47" ht="45" customHeight="1" spans="1:10">
       <c r="A47" s="5">
@@ -3422,7 +3431,7 @@
       <c r="G47" s="5" t="s">
         <v>63</v>
       </c>
-      <c r="H47" s="40" t="s">
+      <c r="H47" s="41" t="s">
         <v>64</v>
       </c>
       <c r="I47" s="5" t="s">
@@ -3454,7 +3463,7 @@
       <c r="G48" s="5" t="s">
         <v>63</v>
       </c>
-      <c r="H48" s="40" t="s">
+      <c r="H48" s="41" t="s">
         <v>64</v>
       </c>
       <c r="I48" s="5" t="s">
@@ -3486,7 +3495,7 @@
       <c r="G49" s="5" t="s">
         <v>63</v>
       </c>
-      <c r="H49" s="40" t="s">
+      <c r="H49" s="41" t="s">
         <v>64</v>
       </c>
       <c r="I49" s="5" t="s">
@@ -3496,20 +3505,20 @@
         <v>20</v>
       </c>
     </row>
-    <row r="50" s="35" customFormat="1" ht="28" customHeight="1" spans="1:10">
+    <row r="50" s="36" customFormat="1" ht="28" customHeight="1" spans="1:10">
       <c r="A50" s="5">
         <v>42</v>
       </c>
-      <c r="B50" s="25" t="s">
+      <c r="B50" s="26" t="s">
         <v>147</v>
       </c>
-      <c r="C50" s="25" t="s">
+      <c r="C50" s="26" t="s">
         <v>148</v>
       </c>
-      <c r="D50" s="25" t="s">
+      <c r="D50" s="26" t="s">
         <v>139</v>
       </c>
-      <c r="E50" s="25" t="s">
+      <c r="E50" s="26" t="s">
         <v>149</v>
       </c>
       <c r="F50" s="5" t="s">
@@ -3518,7 +3527,7 @@
       <c r="G50" s="5" t="s">
         <v>63</v>
       </c>
-      <c r="H50" s="40" t="s">
+      <c r="H50" s="41" t="s">
         <v>64</v>
       </c>
       <c r="I50" s="5" t="s">
@@ -3550,7 +3559,7 @@
       <c r="G51" s="5" t="s">
         <v>63</v>
       </c>
-      <c r="H51" s="40" t="s">
+      <c r="H51" s="41" t="s">
         <v>64</v>
       </c>
       <c r="I51" s="5" t="s">
@@ -3582,7 +3591,7 @@
       <c r="G52" s="5" t="s">
         <v>63</v>
       </c>
-      <c r="H52" s="40" t="s">
+      <c r="H52" s="41" t="s">
         <v>84</v>
       </c>
       <c r="I52" s="5" t="s">
@@ -3614,7 +3623,7 @@
       <c r="G53" s="5" t="s">
         <v>63</v>
       </c>
-      <c r="H53" s="40" t="s">
+      <c r="H53" s="41" t="s">
         <v>64</v>
       </c>
       <c r="I53" s="5" t="s">
@@ -3646,7 +3655,7 @@
       <c r="G54" s="5" t="s">
         <v>63</v>
       </c>
-      <c r="H54" s="40" t="s">
+      <c r="H54" s="41" t="s">
         <v>84</v>
       </c>
       <c r="I54" s="5" t="s">
@@ -3660,15 +3669,15 @@
       <c r="A55" s="23" t="s">
         <v>161</v>
       </c>
-      <c r="B55" s="24"/>
-      <c r="C55" s="24"/>
-      <c r="D55" s="24"/>
-      <c r="E55" s="24"/>
-      <c r="F55" s="24"/>
-      <c r="G55" s="24"/>
-      <c r="H55" s="24"/>
-      <c r="I55" s="24"/>
-      <c r="J55" s="41"/>
+      <c r="B55" s="25"/>
+      <c r="C55" s="25"/>
+      <c r="D55" s="25"/>
+      <c r="E55" s="25"/>
+      <c r="F55" s="25"/>
+      <c r="G55" s="25"/>
+      <c r="H55" s="25"/>
+      <c r="I55" s="25"/>
+      <c r="J55" s="42"/>
     </row>
     <row r="56" ht="45" customHeight="1" spans="1:10">
       <c r="A56" s="5">
@@ -3692,7 +3701,7 @@
       <c r="G56" s="5" t="s">
         <v>63</v>
       </c>
-      <c r="H56" s="40" t="s">
+      <c r="H56" s="41" t="s">
         <v>84</v>
       </c>
       <c r="I56" s="5" t="s">
@@ -3724,7 +3733,7 @@
       <c r="G57" s="5" t="s">
         <v>63</v>
       </c>
-      <c r="H57" s="40" t="s">
+      <c r="H57" s="41" t="s">
         <v>84</v>
       </c>
       <c r="I57" s="5" t="s">
@@ -3756,7 +3765,7 @@
       <c r="G58" s="5" t="s">
         <v>63</v>
       </c>
-      <c r="H58" s="40" t="s">
+      <c r="H58" s="41" t="s">
         <v>84</v>
       </c>
       <c r="I58" s="5" t="s">
@@ -3788,7 +3797,7 @@
       <c r="G59" s="5" t="s">
         <v>63</v>
       </c>
-      <c r="H59" s="40" t="s">
+      <c r="H59" s="41" t="s">
         <v>84</v>
       </c>
       <c r="I59" s="5" t="s">
@@ -3820,7 +3829,7 @@
       <c r="G60" s="5" t="s">
         <v>63</v>
       </c>
-      <c r="H60" s="40" t="s">
+      <c r="H60" s="41" t="s">
         <v>84</v>
       </c>
       <c r="I60" s="5" t="s">
@@ -3852,7 +3861,7 @@
       <c r="G61" s="5" t="s">
         <v>63</v>
       </c>
-      <c r="H61" s="40" t="s">
+      <c r="H61" s="41" t="s">
         <v>84</v>
       </c>
       <c r="I61" s="5" t="s">
@@ -3944,152 +3953,152 @@
       </c>
     </row>
     <row r="4" ht="28" customHeight="1" spans="1:1">
-      <c r="A4" s="27" t="s">
+      <c r="A4" s="28" t="s">
         <v>12</v>
       </c>
     </row>
     <row r="5" ht="45" customHeight="1" spans="1:9">
-      <c r="A5" s="28">
+      <c r="A5" s="29">
         <v>1</v>
       </c>
-      <c r="B5" s="28" t="s">
+      <c r="B5" s="29" t="s">
         <v>13</v>
       </c>
-      <c r="C5" s="28" t="s">
+      <c r="C5" s="29" t="s">
         <v>14</v>
       </c>
-      <c r="D5" s="28" t="s">
+      <c r="D5" s="29" t="s">
         <v>16</v>
       </c>
-      <c r="E5" s="28" t="s">
+      <c r="E5" s="29" t="s">
         <v>17</v>
       </c>
-      <c r="F5" s="29" t="s">
+      <c r="F5" s="30" t="s">
         <v>18</v>
       </c>
-      <c r="G5" s="30" t="s">
-        <v>20</v>
-      </c>
-      <c r="H5" s="30" t="s">
-        <v>20</v>
-      </c>
-      <c r="I5" s="32" t="s">
+      <c r="G5" s="31" t="s">
+        <v>20</v>
+      </c>
+      <c r="H5" s="31" t="s">
+        <v>20</v>
+      </c>
+      <c r="I5" s="33" t="s">
         <v>187</v>
       </c>
     </row>
     <row r="6" ht="45" customHeight="1" spans="1:9">
-      <c r="A6" s="28">
+      <c r="A6" s="29">
         <v>2</v>
       </c>
-      <c r="B6" s="28" t="s">
+      <c r="B6" s="29" t="s">
         <v>21</v>
       </c>
-      <c r="C6" s="28" t="s">
+      <c r="C6" s="29" t="s">
         <v>22</v>
       </c>
-      <c r="D6" s="28" t="s">
+      <c r="D6" s="29" t="s">
         <v>24</v>
       </c>
-      <c r="E6" s="28" t="s">
+      <c r="E6" s="29" t="s">
         <v>17</v>
       </c>
-      <c r="F6" s="29" t="s">
+      <c r="F6" s="30" t="s">
         <v>18</v>
       </c>
-      <c r="G6" s="30" t="s">
-        <v>20</v>
-      </c>
-      <c r="H6" s="30" t="s">
-        <v>20</v>
-      </c>
-      <c r="I6" s="32" t="s">
+      <c r="G6" s="31" t="s">
+        <v>20</v>
+      </c>
+      <c r="H6" s="31" t="s">
+        <v>20</v>
+      </c>
+      <c r="I6" s="33" t="s">
         <v>188</v>
       </c>
     </row>
     <row r="7" ht="45" customHeight="1" spans="1:9">
-      <c r="A7" s="28">
+      <c r="A7" s="29">
         <v>3</v>
       </c>
-      <c r="B7" s="28" t="s">
+      <c r="B7" s="29" t="s">
         <v>25</v>
       </c>
-      <c r="C7" s="28" t="s">
+      <c r="C7" s="29" t="s">
         <v>26</v>
       </c>
-      <c r="D7" s="28" t="s">
+      <c r="D7" s="29" t="s">
         <v>27</v>
       </c>
-      <c r="E7" s="28" t="s">
+      <c r="E7" s="29" t="s">
         <v>17</v>
       </c>
-      <c r="F7" s="29" t="s">
+      <c r="F7" s="30" t="s">
         <v>18</v>
       </c>
-      <c r="G7" s="30" t="s">
-        <v>20</v>
-      </c>
-      <c r="H7" s="30" t="s">
-        <v>20</v>
-      </c>
-      <c r="I7" s="32" t="s">
+      <c r="G7" s="31" t="s">
+        <v>20</v>
+      </c>
+      <c r="H7" s="31" t="s">
+        <v>20</v>
+      </c>
+      <c r="I7" s="33" t="s">
         <v>189</v>
       </c>
     </row>
     <row r="8" ht="45" customHeight="1" spans="1:9">
-      <c r="A8" s="28">
+      <c r="A8" s="29">
         <v>4</v>
       </c>
-      <c r="B8" s="28" t="s">
+      <c r="B8" s="29" t="s">
         <v>28</v>
       </c>
-      <c r="C8" s="28" t="s">
+      <c r="C8" s="29" t="s">
         <v>29</v>
       </c>
-      <c r="D8" s="28" t="s">
+      <c r="D8" s="29" t="s">
         <v>30</v>
       </c>
-      <c r="E8" s="28" t="s">
+      <c r="E8" s="29" t="s">
         <v>17</v>
       </c>
-      <c r="F8" s="29" t="s">
+      <c r="F8" s="30" t="s">
         <v>18</v>
       </c>
-      <c r="G8" s="30" t="s">
-        <v>20</v>
-      </c>
-      <c r="H8" s="30" t="s">
-        <v>20</v>
-      </c>
-      <c r="I8" s="32" t="s">
+      <c r="G8" s="31" t="s">
+        <v>20</v>
+      </c>
+      <c r="H8" s="31" t="s">
+        <v>20</v>
+      </c>
+      <c r="I8" s="33" t="s">
         <v>190</v>
       </c>
     </row>
     <row r="9" ht="45" customHeight="1" spans="1:9">
-      <c r="A9" s="28">
+      <c r="A9" s="29">
         <v>5</v>
       </c>
-      <c r="B9" s="28" t="s">
+      <c r="B9" s="29" t="s">
         <v>31</v>
       </c>
-      <c r="C9" s="28" t="s">
+      <c r="C9" s="29" t="s">
         <v>191</v>
       </c>
-      <c r="D9" s="28" t="s">
+      <c r="D9" s="29" t="s">
         <v>192</v>
       </c>
-      <c r="E9" s="28" t="s">
+      <c r="E9" s="29" t="s">
         <v>17</v>
       </c>
-      <c r="F9" s="29" t="s">
+      <c r="F9" s="30" t="s">
         <v>18</v>
       </c>
-      <c r="G9" s="30" t="s">
-        <v>20</v>
-      </c>
-      <c r="H9" s="30" t="s">
-        <v>20</v>
-      </c>
-      <c r="I9" s="32" t="s">
+      <c r="G9" s="31" t="s">
+        <v>20</v>
+      </c>
+      <c r="H9" s="31" t="s">
+        <v>20</v>
+      </c>
+      <c r="I9" s="33" t="s">
         <v>193</v>
       </c>
     </row>
@@ -4097,14 +4106,14 @@
       <c r="A10" s="23" t="s">
         <v>34</v>
       </c>
-      <c r="B10" s="24"/>
-      <c r="C10" s="24"/>
-      <c r="D10" s="24"/>
-      <c r="E10" s="24"/>
-      <c r="F10" s="31"/>
-      <c r="G10" s="24"/>
-      <c r="H10" s="24"/>
-      <c r="I10" s="33"/>
+      <c r="B10" s="25"/>
+      <c r="C10" s="25"/>
+      <c r="D10" s="25"/>
+      <c r="E10" s="25"/>
+      <c r="F10" s="32"/>
+      <c r="G10" s="25"/>
+      <c r="H10" s="25"/>
+      <c r="I10" s="34"/>
     </row>
     <row r="11" ht="45" customHeight="1" spans="1:9">
       <c r="A11" s="5">
@@ -4122,7 +4131,7 @@
       <c r="E11" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="F11" s="29" t="s">
+      <c r="F11" s="30" t="s">
         <v>194</v>
       </c>
       <c r="G11" s="5" t="s">
@@ -4131,7 +4140,7 @@
       <c r="H11" s="5" t="s">
         <v>20</v>
       </c>
-      <c r="I11" s="34" t="s">
+      <c r="I11" s="35" t="s">
         <v>195</v>
       </c>
     </row>
@@ -4145,13 +4154,13 @@
       <c r="C12" s="6" t="s">
         <v>39</v>
       </c>
-      <c r="D12" s="28" t="s">
+      <c r="D12" s="29" t="s">
         <v>40</v>
       </c>
       <c r="E12" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="F12" s="29" t="s">
+      <c r="F12" s="30" t="s">
         <v>18</v>
       </c>
       <c r="G12" s="5" t="s">
@@ -4160,7 +4169,7 @@
       <c r="H12" s="5" t="s">
         <v>20</v>
       </c>
-      <c r="I12" s="34" t="s">
+      <c r="I12" s="35" t="s">
         <v>196</v>
       </c>
     </row>
@@ -4180,7 +4189,7 @@
       <c r="E13" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="F13" s="29" t="s">
+      <c r="F13" s="30" t="s">
         <v>18</v>
       </c>
       <c r="G13" s="5" t="s">
@@ -4189,7 +4198,7 @@
       <c r="H13" s="5" t="s">
         <v>20</v>
       </c>
-      <c r="I13" s="34" t="s">
+      <c r="I13" s="35" t="s">
         <v>197</v>
       </c>
     </row>
@@ -4209,7 +4218,7 @@
       <c r="E14" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="F14" s="29" t="s">
+      <c r="F14" s="30" t="s">
         <v>18</v>
       </c>
       <c r="G14" s="5" t="s">
@@ -4218,7 +4227,7 @@
       <c r="H14" s="5" t="s">
         <v>20</v>
       </c>
-      <c r="I14" s="34" t="s">
+      <c r="I14" s="35" t="s">
         <v>198</v>
       </c>
     </row>
@@ -4238,7 +4247,7 @@
       <c r="E15" s="5" t="s">
         <v>50</v>
       </c>
-      <c r="F15" s="29" t="s">
+      <c r="F15" s="30" t="s">
         <v>199</v>
       </c>
       <c r="G15" s="5" t="s">
@@ -4247,7 +4256,7 @@
       <c r="H15" s="5" t="s">
         <v>20</v>
       </c>
-      <c r="I15" s="34" t="s">
+      <c r="I15" s="35" t="s">
         <v>200</v>
       </c>
     </row>
@@ -4267,7 +4276,7 @@
       <c r="E16" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="F16" s="29" t="s">
+      <c r="F16" s="30" t="s">
         <v>18</v>
       </c>
       <c r="G16" s="5" t="s">
@@ -4276,7 +4285,7 @@
       <c r="H16" s="5" t="s">
         <v>20</v>
       </c>
-      <c r="I16" s="34" t="s">
+      <c r="I16" s="35" t="s">
         <v>201</v>
       </c>
     </row>
@@ -4296,7 +4305,7 @@
       <c r="E17" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="F17" s="29" t="s">
+      <c r="F17" s="30" t="s">
         <v>194</v>
       </c>
       <c r="G17" s="5" t="s">
@@ -4305,7 +4314,7 @@
       <c r="H17" s="5" t="s">
         <v>20</v>
       </c>
-      <c r="I17" s="34" t="s">
+      <c r="I17" s="35" t="s">
         <v>202</v>
       </c>
     </row>
@@ -4325,7 +4334,7 @@
       <c r="E18" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="F18" s="29" t="s">
+      <c r="F18" s="30" t="s">
         <v>18</v>
       </c>
       <c r="G18" s="5" t="s">
@@ -4334,7 +4343,7 @@
       <c r="H18" s="5" t="s">
         <v>20</v>
       </c>
-      <c r="I18" s="34" t="s">
+      <c r="I18" s="35" t="s">
         <v>203</v>
       </c>
     </row>
@@ -4664,7 +4673,7 @@
       <c r="E13" s="5" t="s">
         <v>93</v>
       </c>
-      <c r="F13" s="5" t="s">
+      <c r="F13" s="24" t="s">
         <v>63</v>
       </c>
       <c r="G13" s="5" t="s">
@@ -4694,7 +4703,7 @@
         <v>93</v>
       </c>
       <c r="F14" s="5" t="s">
-        <v>63</v>
+        <v>18</v>
       </c>
       <c r="G14" s="5" t="s">
         <v>20</v>
@@ -4723,7 +4732,7 @@
         <v>93</v>
       </c>
       <c r="F15" s="5" t="s">
-        <v>63</v>
+        <v>18</v>
       </c>
       <c r="G15" s="5" t="s">
         <v>20</v>
@@ -4780,7 +4789,7 @@
       <c r="E17" s="5" t="s">
         <v>93</v>
       </c>
-      <c r="F17" s="5" t="s">
+      <c r="F17" s="24" t="s">
         <v>63</v>
       </c>
       <c r="G17" s="5" t="s">
@@ -4809,7 +4818,7 @@
       <c r="E18" s="5" t="s">
         <v>93</v>
       </c>
-      <c r="F18" s="5" t="s">
+      <c r="F18" s="24" t="s">
         <v>63</v>
       </c>
       <c r="G18" s="5" t="s">
@@ -4838,7 +4847,7 @@
       <c r="E19" s="5" t="s">
         <v>93</v>
       </c>
-      <c r="F19" s="5" t="s">
+      <c r="F19" s="24" t="s">
         <v>63</v>
       </c>
       <c r="G19" s="5" t="s">
@@ -5129,26 +5138,26 @@
       <c r="A30" s="23" t="s">
         <v>136</v>
       </c>
-      <c r="B30" s="24"/>
-      <c r="C30" s="24"/>
-      <c r="D30" s="24"/>
-      <c r="E30" s="24"/>
-      <c r="F30" s="24"/>
-      <c r="G30" s="24"/>
-      <c r="H30" s="24"/>
-      <c r="I30" s="26"/>
+      <c r="B30" s="25"/>
+      <c r="C30" s="25"/>
+      <c r="D30" s="25"/>
+      <c r="E30" s="25"/>
+      <c r="F30" s="25"/>
+      <c r="G30" s="25"/>
+      <c r="H30" s="25"/>
+      <c r="I30" s="27"/>
     </row>
     <row r="31" ht="28" customHeight="1" spans="1:9">
-      <c r="A31" s="25">
+      <c r="A31" s="26">
         <v>24</v>
       </c>
-      <c r="B31" s="25" t="s">
+      <c r="B31" s="26" t="s">
         <v>137</v>
       </c>
-      <c r="C31" s="25" t="s">
+      <c r="C31" s="26" t="s">
         <v>138</v>
       </c>
-      <c r="D31" s="25" t="s">
+      <c r="D31" s="26" t="s">
         <v>140</v>
       </c>
       <c r="E31" s="5" t="s">

</xml_diff>

<commit_message>
Thêm sửa đổi trong quản lý tuyến
</commit_message>
<xml_diff>
--- a/Project_Tracking.xlsx
+++ b/Project_Tracking.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="16608" windowHeight="9240" activeTab="2"/>
+    <workbookView windowWidth="16608" windowHeight="9240"/>
   </bookViews>
   <sheets>
     <sheet name="Project Tracking" sheetId="1" r:id="rId1"/>
@@ -1504,7 +1504,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="43">
+  <cellXfs count="44">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -1566,6 +1566,9 @@
     </xf>
     <xf numFmtId="0" fontId="2" fillId="8" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="9" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -2076,13 +2079,13 @@
     <col min="4" max="4" width="22" customWidth="1"/>
     <col min="5" max="5" width="60" customWidth="1"/>
     <col min="6" max="7" width="14" customWidth="1"/>
-    <col min="8" max="8" width="10" style="37" customWidth="1"/>
+    <col min="8" max="8" width="10" style="38" customWidth="1"/>
     <col min="9" max="9" width="14" customWidth="1"/>
     <col min="10" max="10" width="30" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" ht="40" customHeight="1" spans="1:10">
-      <c r="A1" s="38" t="s">
+      <c r="A1" s="39" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="8"/>
@@ -2091,7 +2094,7 @@
       <c r="E1" s="8"/>
       <c r="F1" s="8"/>
       <c r="G1" s="8"/>
-      <c r="H1" s="39"/>
+      <c r="H1" s="40"/>
       <c r="I1" s="8"/>
       <c r="J1" s="9"/>
     </row>
@@ -2105,7 +2108,7 @@
       <c r="E2" s="8"/>
       <c r="F2" s="8"/>
       <c r="G2" s="8"/>
-      <c r="H2" s="39"/>
+      <c r="H2" s="40"/>
       <c r="I2" s="8"/>
       <c r="J2" s="9"/>
     </row>
@@ -2141,26 +2144,26 @@
         <v>11</v>
       </c>
     </row>
-    <row r="4" s="36" customFormat="1" ht="28" customHeight="1" spans="1:8">
-      <c r="A4" s="28" t="s">
+    <row r="4" s="37" customFormat="1" ht="28" customHeight="1" spans="1:8">
+      <c r="A4" s="29" t="s">
         <v>12</v>
       </c>
-      <c r="H4" s="40"/>
+      <c r="H4" s="41"/>
     </row>
     <row r="5" ht="45" customHeight="1" spans="1:10">
-      <c r="A5" s="26">
+      <c r="A5" s="27">
         <v>1</v>
       </c>
-      <c r="B5" s="26" t="s">
+      <c r="B5" s="27" t="s">
         <v>13</v>
       </c>
-      <c r="C5" s="26" t="s">
+      <c r="C5" s="27" t="s">
         <v>14</v>
       </c>
-      <c r="D5" s="26" t="s">
+      <c r="D5" s="27" t="s">
         <v>15</v>
       </c>
-      <c r="E5" s="26" t="s">
+      <c r="E5" s="27" t="s">
         <v>16</v>
       </c>
       <c r="F5" s="5" t="s">
@@ -2169,28 +2172,28 @@
       <c r="G5" s="5" t="s">
         <v>18</v>
       </c>
-      <c r="H5" s="41" t="s">
+      <c r="H5" s="42" t="s">
         <v>19</v>
       </c>
-      <c r="I5" s="29"/>
+      <c r="I5" s="30"/>
       <c r="J5" s="5" t="s">
         <v>20</v>
       </c>
     </row>
     <row r="6" ht="45" customHeight="1" spans="1:10">
-      <c r="A6" s="26">
+      <c r="A6" s="27">
         <v>2</v>
       </c>
-      <c r="B6" s="26" t="s">
+      <c r="B6" s="27" t="s">
         <v>21</v>
       </c>
-      <c r="C6" s="26" t="s">
+      <c r="C6" s="27" t="s">
         <v>22</v>
       </c>
-      <c r="D6" s="26" t="s">
+      <c r="D6" s="27" t="s">
         <v>23</v>
       </c>
-      <c r="E6" s="26" t="s">
+      <c r="E6" s="27" t="s">
         <v>24</v>
       </c>
       <c r="F6" s="5" t="s">
@@ -2199,28 +2202,28 @@
       <c r="G6" s="5" t="s">
         <v>18</v>
       </c>
-      <c r="H6" s="41" t="s">
+      <c r="H6" s="42" t="s">
         <v>19</v>
       </c>
-      <c r="I6" s="29"/>
+      <c r="I6" s="30"/>
       <c r="J6" s="5" t="s">
         <v>20</v>
       </c>
     </row>
     <row r="7" ht="45" customHeight="1" spans="1:10">
-      <c r="A7" s="26">
+      <c r="A7" s="27">
         <v>3</v>
       </c>
-      <c r="B7" s="26" t="s">
+      <c r="B7" s="27" t="s">
         <v>25</v>
       </c>
-      <c r="C7" s="26" t="s">
+      <c r="C7" s="27" t="s">
         <v>26</v>
       </c>
-      <c r="D7" s="26" t="s">
+      <c r="D7" s="27" t="s">
         <v>15</v>
       </c>
-      <c r="E7" s="26" t="s">
+      <c r="E7" s="27" t="s">
         <v>27</v>
       </c>
       <c r="F7" s="5" t="s">
@@ -2229,28 +2232,28 @@
       <c r="G7" s="5" t="s">
         <v>18</v>
       </c>
-      <c r="H7" s="41" t="s">
+      <c r="H7" s="42" t="s">
         <v>19</v>
       </c>
-      <c r="I7" s="29"/>
+      <c r="I7" s="30"/>
       <c r="J7" s="5" t="s">
         <v>20</v>
       </c>
     </row>
     <row r="8" ht="45" customHeight="1" spans="1:10">
-      <c r="A8" s="26">
+      <c r="A8" s="27">
         <v>4</v>
       </c>
-      <c r="B8" s="26" t="s">
+      <c r="B8" s="27" t="s">
         <v>28</v>
       </c>
-      <c r="C8" s="26" t="s">
+      <c r="C8" s="27" t="s">
         <v>29</v>
       </c>
-      <c r="D8" s="26" t="s">
+      <c r="D8" s="27" t="s">
         <v>15</v>
       </c>
-      <c r="E8" s="26" t="s">
+      <c r="E8" s="27" t="s">
         <v>30</v>
       </c>
       <c r="F8" s="5" t="s">
@@ -2259,28 +2262,28 @@
       <c r="G8" s="5" t="s">
         <v>18</v>
       </c>
-      <c r="H8" s="41" t="s">
+      <c r="H8" s="42" t="s">
         <v>19</v>
       </c>
-      <c r="I8" s="29"/>
+      <c r="I8" s="30"/>
       <c r="J8" s="5" t="s">
         <v>20</v>
       </c>
     </row>
     <row r="9" ht="45" customHeight="1" spans="1:10">
-      <c r="A9" s="26">
+      <c r="A9" s="27">
         <v>5</v>
       </c>
-      <c r="B9" s="26" t="s">
+      <c r="B9" s="27" t="s">
         <v>31</v>
       </c>
-      <c r="C9" s="26" t="s">
+      <c r="C9" s="27" t="s">
         <v>32</v>
       </c>
-      <c r="D9" s="26" t="s">
+      <c r="D9" s="27" t="s">
         <v>15</v>
       </c>
-      <c r="E9" s="26" t="s">
+      <c r="E9" s="27" t="s">
         <v>33</v>
       </c>
       <c r="F9" s="5" t="s">
@@ -2289,10 +2292,10 @@
       <c r="G9" s="5" t="s">
         <v>18</v>
       </c>
-      <c r="H9" s="41" t="s">
+      <c r="H9" s="42" t="s">
         <v>19</v>
       </c>
-      <c r="I9" s="29"/>
+      <c r="I9" s="30"/>
       <c r="J9" s="5" t="s">
         <v>20</v>
       </c>
@@ -2301,15 +2304,15 @@
       <c r="A10" s="23" t="s">
         <v>34</v>
       </c>
-      <c r="B10" s="25"/>
-      <c r="C10" s="25"/>
-      <c r="D10" s="25"/>
-      <c r="E10" s="25"/>
-      <c r="F10" s="25"/>
-      <c r="G10" s="25"/>
-      <c r="H10" s="25"/>
-      <c r="I10" s="25"/>
-      <c r="J10" s="42"/>
+      <c r="B10" s="26"/>
+      <c r="C10" s="26"/>
+      <c r="D10" s="26"/>
+      <c r="E10" s="26"/>
+      <c r="F10" s="26"/>
+      <c r="G10" s="26"/>
+      <c r="H10" s="26"/>
+      <c r="I10" s="26"/>
+      <c r="J10" s="43"/>
     </row>
     <row r="11" ht="45" customHeight="1" spans="1:10">
       <c r="A11" s="5">
@@ -2333,7 +2336,7 @@
       <c r="G11" s="5" t="s">
         <v>18</v>
       </c>
-      <c r="H11" s="41" t="s">
+      <c r="H11" s="42" t="s">
         <v>19</v>
       </c>
       <c r="I11" s="5" t="s">
@@ -2365,7 +2368,7 @@
       <c r="G12" s="5" t="s">
         <v>18</v>
       </c>
-      <c r="H12" s="41" t="s">
+      <c r="H12" s="42" t="s">
         <v>19</v>
       </c>
       <c r="I12" s="5" t="s">
@@ -2397,7 +2400,7 @@
       <c r="G13" s="5" t="s">
         <v>18</v>
       </c>
-      <c r="H13" s="41" t="s">
+      <c r="H13" s="42" t="s">
         <v>19</v>
       </c>
       <c r="I13" s="5" t="s">
@@ -2429,7 +2432,7 @@
       <c r="G14" s="5" t="s">
         <v>18</v>
       </c>
-      <c r="H14" s="41" t="s">
+      <c r="H14" s="42" t="s">
         <v>19</v>
       </c>
       <c r="I14" s="5" t="s">
@@ -2461,7 +2464,7 @@
       <c r="G15" s="5" t="s">
         <v>18</v>
       </c>
-      <c r="H15" s="41" t="s">
+      <c r="H15" s="42" t="s">
         <v>19</v>
       </c>
       <c r="I15" s="5" t="s">
@@ -2493,7 +2496,7 @@
       <c r="G16" s="5" t="s">
         <v>18</v>
       </c>
-      <c r="H16" s="41" t="s">
+      <c r="H16" s="42" t="s">
         <v>19</v>
       </c>
       <c r="I16" s="5" t="s">
@@ -2525,7 +2528,7 @@
       <c r="G17" s="5" t="s">
         <v>18</v>
       </c>
-      <c r="H17" s="41" t="s">
+      <c r="H17" s="42" t="s">
         <v>19</v>
       </c>
       <c r="I17" s="5" t="s">
@@ -2557,7 +2560,7 @@
       <c r="G18" s="5" t="s">
         <v>18</v>
       </c>
-      <c r="H18" s="41" t="s">
+      <c r="H18" s="42" t="s">
         <v>19</v>
       </c>
       <c r="I18" s="5" t="s">
@@ -2589,7 +2592,7 @@
       <c r="G19" s="5" t="s">
         <v>63</v>
       </c>
-      <c r="H19" s="41" t="s">
+      <c r="H19" s="42" t="s">
         <v>64</v>
       </c>
       <c r="I19" s="5" t="s">
@@ -2621,7 +2624,7 @@
       <c r="G20" s="5" t="s">
         <v>63</v>
       </c>
-      <c r="H20" s="41" t="s">
+      <c r="H20" s="42" t="s">
         <v>64</v>
       </c>
       <c r="I20" s="5" t="s">
@@ -2653,7 +2656,7 @@
       <c r="G21" s="5" t="s">
         <v>63</v>
       </c>
-      <c r="H21" s="41" t="s">
+      <c r="H21" s="42" t="s">
         <v>64</v>
       </c>
       <c r="I21" s="5" t="s">
@@ -2663,7 +2666,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="22" s="36" customFormat="1" ht="28" customHeight="1" spans="1:10">
+    <row r="22" s="37" customFormat="1" ht="28" customHeight="1" spans="1:10">
       <c r="A22" s="6">
         <v>17</v>
       </c>
@@ -2685,7 +2688,7 @@
       <c r="G22" s="5" t="s">
         <v>63</v>
       </c>
-      <c r="H22" s="41" t="s">
+      <c r="H22" s="42" t="s">
         <v>64</v>
       </c>
       <c r="I22" s="5" t="s">
@@ -2717,7 +2720,7 @@
       <c r="G23" s="5" t="s">
         <v>63</v>
       </c>
-      <c r="H23" s="41" t="s">
+      <c r="H23" s="42" t="s">
         <v>64</v>
       </c>
       <c r="I23" s="5" t="s">
@@ -2749,7 +2752,7 @@
       <c r="G24" s="5" t="s">
         <v>63</v>
       </c>
-      <c r="H24" s="41" t="s">
+      <c r="H24" s="42" t="s">
         <v>64</v>
       </c>
       <c r="I24" s="5" t="s">
@@ -2781,7 +2784,7 @@
       <c r="G25" s="5" t="s">
         <v>63</v>
       </c>
-      <c r="H25" s="41" t="s">
+      <c r="H25" s="42" t="s">
         <v>64</v>
       </c>
       <c r="I25" s="5" t="s">
@@ -2813,7 +2816,7 @@
       <c r="G26" s="5" t="s">
         <v>63</v>
       </c>
-      <c r="H26" s="41" t="s">
+      <c r="H26" s="42" t="s">
         <v>84</v>
       </c>
       <c r="I26" s="5" t="s">
@@ -2845,7 +2848,7 @@
       <c r="G27" s="5" t="s">
         <v>63</v>
       </c>
-      <c r="H27" s="41" t="s">
+      <c r="H27" s="42" t="s">
         <v>84</v>
       </c>
       <c r="I27" s="5" t="s">
@@ -2859,15 +2862,15 @@
       <c r="A28" s="23" t="s">
         <v>88</v>
       </c>
-      <c r="B28" s="25"/>
-      <c r="C28" s="25"/>
-      <c r="D28" s="25"/>
-      <c r="E28" s="25"/>
-      <c r="F28" s="25"/>
-      <c r="G28" s="25"/>
-      <c r="H28" s="25"/>
-      <c r="I28" s="25"/>
-      <c r="J28" s="42"/>
+      <c r="B28" s="26"/>
+      <c r="C28" s="26"/>
+      <c r="D28" s="26"/>
+      <c r="E28" s="26"/>
+      <c r="F28" s="26"/>
+      <c r="G28" s="26"/>
+      <c r="H28" s="26"/>
+      <c r="I28" s="26"/>
+      <c r="J28" s="43"/>
     </row>
     <row r="29" ht="45" customHeight="1" spans="1:10">
       <c r="A29" s="5">
@@ -2891,7 +2894,7 @@
       <c r="G29" s="5" t="s">
         <v>63</v>
       </c>
-      <c r="H29" s="41" t="s">
+      <c r="H29" s="42" t="s">
         <v>64</v>
       </c>
       <c r="I29" s="5" t="s">
@@ -2923,7 +2926,7 @@
       <c r="G30" s="5" t="s">
         <v>63</v>
       </c>
-      <c r="H30" s="41" t="s">
+      <c r="H30" s="42" t="s">
         <v>64</v>
       </c>
       <c r="I30" s="5" t="s">
@@ -2955,7 +2958,7 @@
       <c r="G31" s="5" t="s">
         <v>63</v>
       </c>
-      <c r="H31" s="41" t="s">
+      <c r="H31" s="42" t="s">
         <v>64</v>
       </c>
       <c r="I31" s="5" t="s">
@@ -2987,7 +2990,7 @@
       <c r="G32" s="5" t="s">
         <v>63</v>
       </c>
-      <c r="H32" s="41" t="s">
+      <c r="H32" s="42" t="s">
         <v>64</v>
       </c>
       <c r="I32" s="5" t="s">
@@ -3019,7 +3022,7 @@
       <c r="G33" s="5" t="s">
         <v>63</v>
       </c>
-      <c r="H33" s="41" t="s">
+      <c r="H33" s="42" t="s">
         <v>64</v>
       </c>
       <c r="I33" s="5" t="s">
@@ -3029,20 +3032,20 @@
         <v>20</v>
       </c>
     </row>
-    <row r="34" s="36" customFormat="1" ht="38" customHeight="1" spans="1:10">
+    <row r="34" s="37" customFormat="1" ht="38" customHeight="1" spans="1:10">
       <c r="A34" s="5">
         <v>28</v>
       </c>
       <c r="B34" s="5" t="s">
         <v>103</v>
       </c>
-      <c r="C34" s="26" t="s">
+      <c r="C34" s="27" t="s">
         <v>104</v>
       </c>
-      <c r="D34" s="26" t="s">
+      <c r="D34" s="27" t="s">
         <v>91</v>
       </c>
-      <c r="E34" s="26" t="s">
+      <c r="E34" s="27" t="s">
         <v>105</v>
       </c>
       <c r="F34" s="5" t="s">
@@ -3051,7 +3054,7 @@
       <c r="G34" s="5" t="s">
         <v>63</v>
       </c>
-      <c r="H34" s="41" t="s">
+      <c r="H34" s="42" t="s">
         <v>64</v>
       </c>
       <c r="I34" s="5" t="s">
@@ -3083,7 +3086,7 @@
       <c r="G35" s="5" t="s">
         <v>18</v>
       </c>
-      <c r="H35" s="41" t="s">
+      <c r="H35" s="42" t="s">
         <v>64</v>
       </c>
       <c r="I35" s="5" t="s">
@@ -3115,7 +3118,7 @@
       <c r="G36" s="5" t="s">
         <v>18</v>
       </c>
-      <c r="H36" s="41" t="s">
+      <c r="H36" s="42" t="s">
         <v>64</v>
       </c>
       <c r="I36" s="5" t="s">
@@ -3147,7 +3150,7 @@
       <c r="G37" s="5" t="s">
         <v>18</v>
       </c>
-      <c r="H37" s="41" t="s">
+      <c r="H37" s="42" t="s">
         <v>64</v>
       </c>
       <c r="I37" s="5" t="s">
@@ -3179,7 +3182,7 @@
       <c r="G38" s="5" t="s">
         <v>18</v>
       </c>
-      <c r="H38" s="41" t="s">
+      <c r="H38" s="42" t="s">
         <v>64</v>
       </c>
       <c r="I38" s="5" t="s">
@@ -3211,7 +3214,7 @@
       <c r="G39" s="5" t="s">
         <v>18</v>
       </c>
-      <c r="H39" s="41" t="s">
+      <c r="H39" s="42" t="s">
         <v>64</v>
       </c>
       <c r="I39" s="5" t="s">
@@ -3225,17 +3228,17 @@
       <c r="A40" s="23" t="s">
         <v>118</v>
       </c>
-      <c r="B40" s="25"/>
-      <c r="C40" s="25"/>
-      <c r="D40" s="25"/>
-      <c r="E40" s="25"/>
-      <c r="F40" s="25"/>
-      <c r="G40" s="25"/>
-      <c r="H40" s="25"/>
-      <c r="I40" s="25"/>
-      <c r="J40" s="42"/>
-    </row>
-    <row r="41" s="36" customFormat="1" ht="46" customHeight="1" spans="1:10">
+      <c r="B40" s="26"/>
+      <c r="C40" s="26"/>
+      <c r="D40" s="26"/>
+      <c r="E40" s="26"/>
+      <c r="F40" s="26"/>
+      <c r="G40" s="26"/>
+      <c r="H40" s="26"/>
+      <c r="I40" s="26"/>
+      <c r="J40" s="43"/>
+    </row>
+    <row r="41" s="37" customFormat="1" ht="46" customHeight="1" spans="1:10">
       <c r="A41" s="6">
         <v>34</v>
       </c>
@@ -3257,7 +3260,7 @@
       <c r="G41" s="5" t="s">
         <v>63</v>
       </c>
-      <c r="H41" s="41" t="s">
+      <c r="H41" s="42" t="s">
         <v>64</v>
       </c>
       <c r="I41" s="5" t="s">
@@ -3289,7 +3292,7 @@
       <c r="G42" s="5" t="s">
         <v>63</v>
       </c>
-      <c r="H42" s="41" t="s">
+      <c r="H42" s="42" t="s">
         <v>64</v>
       </c>
       <c r="I42" s="5" t="s">
@@ -3321,7 +3324,7 @@
       <c r="G43" s="5" t="s">
         <v>63</v>
       </c>
-      <c r="H43" s="41" t="s">
+      <c r="H43" s="42" t="s">
         <v>64</v>
       </c>
       <c r="I43" s="5" t="s">
@@ -3353,7 +3356,7 @@
       <c r="G44" s="5" t="s">
         <v>63</v>
       </c>
-      <c r="H44" s="41" t="s">
+      <c r="H44" s="42" t="s">
         <v>64</v>
       </c>
       <c r="I44" s="5" t="s">
@@ -3385,7 +3388,7 @@
       <c r="G45" s="5" t="s">
         <v>63</v>
       </c>
-      <c r="H45" s="41" t="s">
+      <c r="H45" s="42" t="s">
         <v>64</v>
       </c>
       <c r="I45" s="5" t="s">
@@ -3399,15 +3402,15 @@
       <c r="A46" s="23" t="s">
         <v>136</v>
       </c>
-      <c r="B46" s="25"/>
-      <c r="C46" s="25"/>
-      <c r="D46" s="25"/>
-      <c r="E46" s="25"/>
-      <c r="F46" s="25"/>
-      <c r="G46" s="25"/>
-      <c r="H46" s="25"/>
-      <c r="I46" s="25"/>
-      <c r="J46" s="42"/>
+      <c r="B46" s="26"/>
+      <c r="C46" s="26"/>
+      <c r="D46" s="26"/>
+      <c r="E46" s="26"/>
+      <c r="F46" s="26"/>
+      <c r="G46" s="26"/>
+      <c r="H46" s="26"/>
+      <c r="I46" s="26"/>
+      <c r="J46" s="43"/>
     </row>
     <row r="47" ht="45" customHeight="1" spans="1:10">
       <c r="A47" s="5">
@@ -3431,7 +3434,7 @@
       <c r="G47" s="5" t="s">
         <v>63</v>
       </c>
-      <c r="H47" s="41" t="s">
+      <c r="H47" s="42" t="s">
         <v>64</v>
       </c>
       <c r="I47" s="5" t="s">
@@ -3463,7 +3466,7 @@
       <c r="G48" s="5" t="s">
         <v>63</v>
       </c>
-      <c r="H48" s="41" t="s">
+      <c r="H48" s="42" t="s">
         <v>64</v>
       </c>
       <c r="I48" s="5" t="s">
@@ -3495,7 +3498,7 @@
       <c r="G49" s="5" t="s">
         <v>63</v>
       </c>
-      <c r="H49" s="41" t="s">
+      <c r="H49" s="42" t="s">
         <v>64</v>
       </c>
       <c r="I49" s="5" t="s">
@@ -3505,20 +3508,20 @@
         <v>20</v>
       </c>
     </row>
-    <row r="50" s="36" customFormat="1" ht="28" customHeight="1" spans="1:10">
+    <row r="50" s="37" customFormat="1" ht="28" customHeight="1" spans="1:10">
       <c r="A50" s="5">
         <v>42</v>
       </c>
-      <c r="B50" s="26" t="s">
+      <c r="B50" s="27" t="s">
         <v>147</v>
       </c>
-      <c r="C50" s="26" t="s">
+      <c r="C50" s="27" t="s">
         <v>148</v>
       </c>
-      <c r="D50" s="26" t="s">
+      <c r="D50" s="27" t="s">
         <v>139</v>
       </c>
-      <c r="E50" s="26" t="s">
+      <c r="E50" s="27" t="s">
         <v>149</v>
       </c>
       <c r="F50" s="5" t="s">
@@ -3527,7 +3530,7 @@
       <c r="G50" s="5" t="s">
         <v>63</v>
       </c>
-      <c r="H50" s="41" t="s">
+      <c r="H50" s="42" t="s">
         <v>64</v>
       </c>
       <c r="I50" s="5" t="s">
@@ -3559,7 +3562,7 @@
       <c r="G51" s="5" t="s">
         <v>63</v>
       </c>
-      <c r="H51" s="41" t="s">
+      <c r="H51" s="42" t="s">
         <v>64</v>
       </c>
       <c r="I51" s="5" t="s">
@@ -3591,7 +3594,7 @@
       <c r="G52" s="5" t="s">
         <v>63</v>
       </c>
-      <c r="H52" s="41" t="s">
+      <c r="H52" s="42" t="s">
         <v>84</v>
       </c>
       <c r="I52" s="5" t="s">
@@ -3623,7 +3626,7 @@
       <c r="G53" s="5" t="s">
         <v>63</v>
       </c>
-      <c r="H53" s="41" t="s">
+      <c r="H53" s="42" t="s">
         <v>64</v>
       </c>
       <c r="I53" s="5" t="s">
@@ -3655,7 +3658,7 @@
       <c r="G54" s="5" t="s">
         <v>63</v>
       </c>
-      <c r="H54" s="41" t="s">
+      <c r="H54" s="42" t="s">
         <v>84</v>
       </c>
       <c r="I54" s="5" t="s">
@@ -3669,15 +3672,15 @@
       <c r="A55" s="23" t="s">
         <v>161</v>
       </c>
-      <c r="B55" s="25"/>
-      <c r="C55" s="25"/>
-      <c r="D55" s="25"/>
-      <c r="E55" s="25"/>
-      <c r="F55" s="25"/>
-      <c r="G55" s="25"/>
-      <c r="H55" s="25"/>
-      <c r="I55" s="25"/>
-      <c r="J55" s="42"/>
+      <c r="B55" s="26"/>
+      <c r="C55" s="26"/>
+      <c r="D55" s="26"/>
+      <c r="E55" s="26"/>
+      <c r="F55" s="26"/>
+      <c r="G55" s="26"/>
+      <c r="H55" s="26"/>
+      <c r="I55" s="26"/>
+      <c r="J55" s="43"/>
     </row>
     <row r="56" ht="45" customHeight="1" spans="1:10">
       <c r="A56" s="5">
@@ -3701,7 +3704,7 @@
       <c r="G56" s="5" t="s">
         <v>63</v>
       </c>
-      <c r="H56" s="41" t="s">
+      <c r="H56" s="42" t="s">
         <v>84</v>
       </c>
       <c r="I56" s="5" t="s">
@@ -3733,7 +3736,7 @@
       <c r="G57" s="5" t="s">
         <v>63</v>
       </c>
-      <c r="H57" s="41" t="s">
+      <c r="H57" s="42" t="s">
         <v>84</v>
       </c>
       <c r="I57" s="5" t="s">
@@ -3765,7 +3768,7 @@
       <c r="G58" s="5" t="s">
         <v>63</v>
       </c>
-      <c r="H58" s="41" t="s">
+      <c r="H58" s="42" t="s">
         <v>84</v>
       </c>
       <c r="I58" s="5" t="s">
@@ -3797,7 +3800,7 @@
       <c r="G59" s="5" t="s">
         <v>63</v>
       </c>
-      <c r="H59" s="41" t="s">
+      <c r="H59" s="42" t="s">
         <v>84</v>
       </c>
       <c r="I59" s="5" t="s">
@@ -3829,7 +3832,7 @@
       <c r="G60" s="5" t="s">
         <v>63</v>
       </c>
-      <c r="H60" s="41" t="s">
+      <c r="H60" s="42" t="s">
         <v>84</v>
       </c>
       <c r="I60" s="5" t="s">
@@ -3861,7 +3864,7 @@
       <c r="G61" s="5" t="s">
         <v>63</v>
       </c>
-      <c r="H61" s="41" t="s">
+      <c r="H61" s="42" t="s">
         <v>84</v>
       </c>
       <c r="I61" s="5" t="s">
@@ -3953,152 +3956,152 @@
       </c>
     </row>
     <row r="4" ht="28" customHeight="1" spans="1:1">
-      <c r="A4" s="28" t="s">
+      <c r="A4" s="29" t="s">
         <v>12</v>
       </c>
     </row>
     <row r="5" ht="45" customHeight="1" spans="1:9">
-      <c r="A5" s="29">
+      <c r="A5" s="30">
         <v>1</v>
       </c>
-      <c r="B5" s="29" t="s">
+      <c r="B5" s="30" t="s">
         <v>13</v>
       </c>
-      <c r="C5" s="29" t="s">
+      <c r="C5" s="30" t="s">
         <v>14</v>
       </c>
-      <c r="D5" s="29" t="s">
+      <c r="D5" s="30" t="s">
         <v>16</v>
       </c>
-      <c r="E5" s="29" t="s">
+      <c r="E5" s="30" t="s">
         <v>17</v>
       </c>
-      <c r="F5" s="30" t="s">
+      <c r="F5" s="31" t="s">
         <v>18</v>
       </c>
-      <c r="G5" s="31" t="s">
-        <v>20</v>
-      </c>
-      <c r="H5" s="31" t="s">
-        <v>20</v>
-      </c>
-      <c r="I5" s="33" t="s">
+      <c r="G5" s="32" t="s">
+        <v>20</v>
+      </c>
+      <c r="H5" s="32" t="s">
+        <v>20</v>
+      </c>
+      <c r="I5" s="34" t="s">
         <v>187</v>
       </c>
     </row>
     <row r="6" ht="45" customHeight="1" spans="1:9">
-      <c r="A6" s="29">
+      <c r="A6" s="30">
         <v>2</v>
       </c>
-      <c r="B6" s="29" t="s">
+      <c r="B6" s="30" t="s">
         <v>21</v>
       </c>
-      <c r="C6" s="29" t="s">
+      <c r="C6" s="30" t="s">
         <v>22</v>
       </c>
-      <c r="D6" s="29" t="s">
+      <c r="D6" s="30" t="s">
         <v>24</v>
       </c>
-      <c r="E6" s="29" t="s">
+      <c r="E6" s="30" t="s">
         <v>17</v>
       </c>
-      <c r="F6" s="30" t="s">
+      <c r="F6" s="31" t="s">
         <v>18</v>
       </c>
-      <c r="G6" s="31" t="s">
-        <v>20</v>
-      </c>
-      <c r="H6" s="31" t="s">
-        <v>20</v>
-      </c>
-      <c r="I6" s="33" t="s">
+      <c r="G6" s="32" t="s">
+        <v>20</v>
+      </c>
+      <c r="H6" s="32" t="s">
+        <v>20</v>
+      </c>
+      <c r="I6" s="34" t="s">
         <v>188</v>
       </c>
     </row>
     <row r="7" ht="45" customHeight="1" spans="1:9">
-      <c r="A7" s="29">
+      <c r="A7" s="30">
         <v>3</v>
       </c>
-      <c r="B7" s="29" t="s">
+      <c r="B7" s="30" t="s">
         <v>25</v>
       </c>
-      <c r="C7" s="29" t="s">
+      <c r="C7" s="30" t="s">
         <v>26</v>
       </c>
-      <c r="D7" s="29" t="s">
+      <c r="D7" s="30" t="s">
         <v>27</v>
       </c>
-      <c r="E7" s="29" t="s">
+      <c r="E7" s="30" t="s">
         <v>17</v>
       </c>
-      <c r="F7" s="30" t="s">
+      <c r="F7" s="31" t="s">
         <v>18</v>
       </c>
-      <c r="G7" s="31" t="s">
-        <v>20</v>
-      </c>
-      <c r="H7" s="31" t="s">
-        <v>20</v>
-      </c>
-      <c r="I7" s="33" t="s">
+      <c r="G7" s="32" t="s">
+        <v>20</v>
+      </c>
+      <c r="H7" s="32" t="s">
+        <v>20</v>
+      </c>
+      <c r="I7" s="34" t="s">
         <v>189</v>
       </c>
     </row>
     <row r="8" ht="45" customHeight="1" spans="1:9">
-      <c r="A8" s="29">
+      <c r="A8" s="30">
         <v>4</v>
       </c>
-      <c r="B8" s="29" t="s">
+      <c r="B8" s="30" t="s">
         <v>28</v>
       </c>
-      <c r="C8" s="29" t="s">
+      <c r="C8" s="30" t="s">
         <v>29</v>
       </c>
-      <c r="D8" s="29" t="s">
+      <c r="D8" s="30" t="s">
         <v>30</v>
       </c>
-      <c r="E8" s="29" t="s">
+      <c r="E8" s="30" t="s">
         <v>17</v>
       </c>
-      <c r="F8" s="30" t="s">
+      <c r="F8" s="31" t="s">
         <v>18</v>
       </c>
-      <c r="G8" s="31" t="s">
-        <v>20</v>
-      </c>
-      <c r="H8" s="31" t="s">
-        <v>20</v>
-      </c>
-      <c r="I8" s="33" t="s">
+      <c r="G8" s="32" t="s">
+        <v>20</v>
+      </c>
+      <c r="H8" s="32" t="s">
+        <v>20</v>
+      </c>
+      <c r="I8" s="34" t="s">
         <v>190</v>
       </c>
     </row>
     <row r="9" ht="45" customHeight="1" spans="1:9">
-      <c r="A9" s="29">
+      <c r="A9" s="30">
         <v>5</v>
       </c>
-      <c r="B9" s="29" t="s">
+      <c r="B9" s="30" t="s">
         <v>31</v>
       </c>
-      <c r="C9" s="29" t="s">
+      <c r="C9" s="30" t="s">
         <v>191</v>
       </c>
-      <c r="D9" s="29" t="s">
+      <c r="D9" s="30" t="s">
         <v>192</v>
       </c>
-      <c r="E9" s="29" t="s">
+      <c r="E9" s="30" t="s">
         <v>17</v>
       </c>
-      <c r="F9" s="30" t="s">
+      <c r="F9" s="31" t="s">
         <v>18</v>
       </c>
-      <c r="G9" s="31" t="s">
-        <v>20</v>
-      </c>
-      <c r="H9" s="31" t="s">
-        <v>20</v>
-      </c>
-      <c r="I9" s="33" t="s">
+      <c r="G9" s="32" t="s">
+        <v>20</v>
+      </c>
+      <c r="H9" s="32" t="s">
+        <v>20</v>
+      </c>
+      <c r="I9" s="34" t="s">
         <v>193</v>
       </c>
     </row>
@@ -4106,14 +4109,14 @@
       <c r="A10" s="23" t="s">
         <v>34</v>
       </c>
-      <c r="B10" s="25"/>
-      <c r="C10" s="25"/>
-      <c r="D10" s="25"/>
-      <c r="E10" s="25"/>
-      <c r="F10" s="32"/>
-      <c r="G10" s="25"/>
-      <c r="H10" s="25"/>
-      <c r="I10" s="34"/>
+      <c r="B10" s="26"/>
+      <c r="C10" s="26"/>
+      <c r="D10" s="26"/>
+      <c r="E10" s="26"/>
+      <c r="F10" s="33"/>
+      <c r="G10" s="26"/>
+      <c r="H10" s="26"/>
+      <c r="I10" s="35"/>
     </row>
     <row r="11" ht="45" customHeight="1" spans="1:9">
       <c r="A11" s="5">
@@ -4131,7 +4134,7 @@
       <c r="E11" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="F11" s="30" t="s">
+      <c r="F11" s="31" t="s">
         <v>194</v>
       </c>
       <c r="G11" s="5" t="s">
@@ -4140,7 +4143,7 @@
       <c r="H11" s="5" t="s">
         <v>20</v>
       </c>
-      <c r="I11" s="35" t="s">
+      <c r="I11" s="36" t="s">
         <v>195</v>
       </c>
     </row>
@@ -4154,13 +4157,13 @@
       <c r="C12" s="6" t="s">
         <v>39</v>
       </c>
-      <c r="D12" s="29" t="s">
+      <c r="D12" s="30" t="s">
         <v>40</v>
       </c>
       <c r="E12" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="F12" s="30" t="s">
+      <c r="F12" s="31" t="s">
         <v>18</v>
       </c>
       <c r="G12" s="5" t="s">
@@ -4169,7 +4172,7 @@
       <c r="H12" s="5" t="s">
         <v>20</v>
       </c>
-      <c r="I12" s="35" t="s">
+      <c r="I12" s="36" t="s">
         <v>196</v>
       </c>
     </row>
@@ -4189,7 +4192,7 @@
       <c r="E13" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="F13" s="30" t="s">
+      <c r="F13" s="31" t="s">
         <v>18</v>
       </c>
       <c r="G13" s="5" t="s">
@@ -4198,7 +4201,7 @@
       <c r="H13" s="5" t="s">
         <v>20</v>
       </c>
-      <c r="I13" s="35" t="s">
+      <c r="I13" s="36" t="s">
         <v>197</v>
       </c>
     </row>
@@ -4218,7 +4221,7 @@
       <c r="E14" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="F14" s="30" t="s">
+      <c r="F14" s="31" t="s">
         <v>18</v>
       </c>
       <c r="G14" s="5" t="s">
@@ -4227,7 +4230,7 @@
       <c r="H14" s="5" t="s">
         <v>20</v>
       </c>
-      <c r="I14" s="35" t="s">
+      <c r="I14" s="36" t="s">
         <v>198</v>
       </c>
     </row>
@@ -4247,7 +4250,7 @@
       <c r="E15" s="5" t="s">
         <v>50</v>
       </c>
-      <c r="F15" s="30" t="s">
+      <c r="F15" s="31" t="s">
         <v>199</v>
       </c>
       <c r="G15" s="5" t="s">
@@ -4256,7 +4259,7 @@
       <c r="H15" s="5" t="s">
         <v>20</v>
       </c>
-      <c r="I15" s="35" t="s">
+      <c r="I15" s="36" t="s">
         <v>200</v>
       </c>
     </row>
@@ -4276,7 +4279,7 @@
       <c r="E16" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="F16" s="30" t="s">
+      <c r="F16" s="31" t="s">
         <v>18</v>
       </c>
       <c r="G16" s="5" t="s">
@@ -4285,7 +4288,7 @@
       <c r="H16" s="5" t="s">
         <v>20</v>
       </c>
-      <c r="I16" s="35" t="s">
+      <c r="I16" s="36" t="s">
         <v>201</v>
       </c>
     </row>
@@ -4305,7 +4308,7 @@
       <c r="E17" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="F17" s="30" t="s">
+      <c r="F17" s="31" t="s">
         <v>194</v>
       </c>
       <c r="G17" s="5" t="s">
@@ -4314,7 +4317,7 @@
       <c r="H17" s="5" t="s">
         <v>20</v>
       </c>
-      <c r="I17" s="35" t="s">
+      <c r="I17" s="36" t="s">
         <v>202</v>
       </c>
     </row>
@@ -4334,7 +4337,7 @@
       <c r="E18" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="F18" s="30" t="s">
+      <c r="F18" s="31" t="s">
         <v>18</v>
       </c>
       <c r="G18" s="5" t="s">
@@ -4343,7 +4346,7 @@
       <c r="H18" s="5" t="s">
         <v>20</v>
       </c>
-      <c r="I18" s="35" t="s">
+      <c r="I18" s="36" t="s">
         <v>203</v>
       </c>
     </row>
@@ -4674,7 +4677,7 @@
         <v>93</v>
       </c>
       <c r="F13" s="24" t="s">
-        <v>63</v>
+        <v>18</v>
       </c>
       <c r="G13" s="5" t="s">
         <v>20</v>
@@ -4789,7 +4792,7 @@
       <c r="E17" s="5" t="s">
         <v>93</v>
       </c>
-      <c r="F17" s="24" t="s">
+      <c r="F17" s="25" t="s">
         <v>63</v>
       </c>
       <c r="G17" s="5" t="s">
@@ -4818,7 +4821,7 @@
       <c r="E18" s="5" t="s">
         <v>93</v>
       </c>
-      <c r="F18" s="24" t="s">
+      <c r="F18" s="25" t="s">
         <v>63</v>
       </c>
       <c r="G18" s="5" t="s">
@@ -4847,7 +4850,7 @@
       <c r="E19" s="5" t="s">
         <v>93</v>
       </c>
-      <c r="F19" s="24" t="s">
+      <c r="F19" s="25" t="s">
         <v>63</v>
       </c>
       <c r="G19" s="5" t="s">
@@ -5138,26 +5141,26 @@
       <c r="A30" s="23" t="s">
         <v>136</v>
       </c>
-      <c r="B30" s="25"/>
-      <c r="C30" s="25"/>
-      <c r="D30" s="25"/>
-      <c r="E30" s="25"/>
-      <c r="F30" s="25"/>
-      <c r="G30" s="25"/>
-      <c r="H30" s="25"/>
-      <c r="I30" s="27"/>
+      <c r="B30" s="26"/>
+      <c r="C30" s="26"/>
+      <c r="D30" s="26"/>
+      <c r="E30" s="26"/>
+      <c r="F30" s="26"/>
+      <c r="G30" s="26"/>
+      <c r="H30" s="26"/>
+      <c r="I30" s="28"/>
     </row>
     <row r="31" ht="28" customHeight="1" spans="1:9">
-      <c r="A31" s="26">
+      <c r="A31" s="27">
         <v>24</v>
       </c>
-      <c r="B31" s="26" t="s">
+      <c r="B31" s="27" t="s">
         <v>137</v>
       </c>
-      <c r="C31" s="26" t="s">
+      <c r="C31" s="27" t="s">
         <v>138</v>
       </c>
-      <c r="D31" s="26" t="s">
+      <c r="D31" s="27" t="s">
         <v>140</v>
       </c>
       <c r="E31" s="5" t="s">

</xml_diff>

<commit_message>
Cập nhật file tracking
</commit_message>
<xml_diff>
--- a/Project_Tracking.xlsx
+++ b/Project_Tracking.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="16608" windowHeight="9240"/>
+    <workbookView windowWidth="20760" windowHeight="12300"/>
   </bookViews>
   <sheets>
     <sheet name="Project Tracking" sheetId="1" r:id="rId1"/>
@@ -945,7 +945,7 @@
       <charset val="134"/>
     </font>
   </fonts>
-  <fills count="40">
+  <fills count="41">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -997,6 +997,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="4" tint="0.4"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -1380,7 +1386,7 @@
     <xf numFmtId="0" fontId="13" fillId="0" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="10" borderId="6">
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="6">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="14" fillId="0" borderId="0">
@@ -1404,16 +1410,16 @@
     <xf numFmtId="0" fontId="19" fillId="0" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="11" borderId="9">
+    <xf numFmtId="0" fontId="20" fillId="12" borderId="9">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="12" borderId="10">
+    <xf numFmtId="0" fontId="21" fillId="13" borderId="10">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="12" borderId="9">
+    <xf numFmtId="0" fontId="22" fillId="13" borderId="9">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="23" fillId="13" borderId="11">
+    <xf numFmtId="0" fontId="23" fillId="14" borderId="11">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="24" fillId="0" borderId="12">
@@ -1425,86 +1431,86 @@
     <xf numFmtId="0" fontId="25" fillId="4" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="26" fillId="14" borderId="0">
+    <xf numFmtId="0" fontId="26" fillId="15" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="27" fillId="15" borderId="0">
+    <xf numFmtId="0" fontId="27" fillId="16" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="16" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="17" borderId="0">
+    <xf numFmtId="0" fontId="8" fillId="17" borderId="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="18" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="19" borderId="0">
+    <xf numFmtId="0" fontId="0" fillId="19" borderId="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="20" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="21" borderId="0">
+    <xf numFmtId="0" fontId="8" fillId="21" borderId="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="22" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="23" borderId="0">
+    <xf numFmtId="0" fontId="0" fillId="23" borderId="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="24" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="25" borderId="0">
+    <xf numFmtId="0" fontId="8" fillId="25" borderId="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="26" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="27" borderId="0">
+    <xf numFmtId="0" fontId="0" fillId="27" borderId="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="28" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="29" borderId="0">
+    <xf numFmtId="0" fontId="8" fillId="29" borderId="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="30" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="31" borderId="0">
+    <xf numFmtId="0" fontId="0" fillId="31" borderId="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="32" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="33" borderId="0">
+    <xf numFmtId="0" fontId="8" fillId="33" borderId="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="34" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="35" borderId="0">
+    <xf numFmtId="0" fontId="0" fillId="35" borderId="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="36" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="37" borderId="0">
+    <xf numFmtId="0" fontId="8" fillId="37" borderId="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="38" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="39" borderId="0">
+    <xf numFmtId="0" fontId="0" fillId="39" borderId="0">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="8" fillId="40" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
   </cellStyleXfs>
-  <cellXfs count="44">
+  <cellXfs count="45">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -1614,6 +1620,9 @@
     <xf numFmtId="0" fontId="9" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="10" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="8" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -2071,7 +2080,7 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
   <dimension ref="A1:J61"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.4"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="5" customWidth="1"/>
     <col min="2" max="2" width="25" customWidth="1"/>
@@ -2312,7 +2321,7 @@
       <c r="G10" s="26"/>
       <c r="H10" s="26"/>
       <c r="I10" s="26"/>
-      <c r="J10" s="43"/>
+      <c r="J10" s="44"/>
     </row>
     <row r="11" ht="45" customHeight="1" spans="1:10">
       <c r="A11" s="5">
@@ -2870,7 +2879,7 @@
       <c r="G28" s="26"/>
       <c r="H28" s="26"/>
       <c r="I28" s="26"/>
-      <c r="J28" s="43"/>
+      <c r="J28" s="44"/>
     </row>
     <row r="29" ht="45" customHeight="1" spans="1:10">
       <c r="A29" s="5">
@@ -2891,8 +2900,8 @@
       <c r="F29" s="5" t="s">
         <v>93</v>
       </c>
-      <c r="G29" s="5" t="s">
-        <v>63</v>
+      <c r="G29" s="24" t="s">
+        <v>18</v>
       </c>
       <c r="H29" s="42" t="s">
         <v>64</v>
@@ -2923,8 +2932,8 @@
       <c r="F30" s="5" t="s">
         <v>93</v>
       </c>
-      <c r="G30" s="5" t="s">
-        <v>63</v>
+      <c r="G30" s="24" t="s">
+        <v>18</v>
       </c>
       <c r="H30" s="42" t="s">
         <v>64</v>
@@ -2955,8 +2964,8 @@
       <c r="F31" s="5" t="s">
         <v>93</v>
       </c>
-      <c r="G31" s="5" t="s">
-        <v>63</v>
+      <c r="G31" s="24" t="s">
+        <v>18</v>
       </c>
       <c r="H31" s="42" t="s">
         <v>64</v>
@@ -2987,8 +2996,8 @@
       <c r="F32" s="5" t="s">
         <v>93</v>
       </c>
-      <c r="G32" s="5" t="s">
-        <v>63</v>
+      <c r="G32" s="24" t="s">
+        <v>18</v>
       </c>
       <c r="H32" s="42" t="s">
         <v>64</v>
@@ -3019,7 +3028,7 @@
       <c r="F33" s="5" t="s">
         <v>93</v>
       </c>
-      <c r="G33" s="5" t="s">
+      <c r="G33" s="43" t="s">
         <v>63</v>
       </c>
       <c r="H33" s="42" t="s">
@@ -3051,7 +3060,7 @@
       <c r="F34" s="5" t="s">
         <v>93</v>
       </c>
-      <c r="G34" s="5" t="s">
+      <c r="G34" s="43" t="s">
         <v>63</v>
       </c>
       <c r="H34" s="42" t="s">
@@ -3236,7 +3245,7 @@
       <c r="G40" s="26"/>
       <c r="H40" s="26"/>
       <c r="I40" s="26"/>
-      <c r="J40" s="43"/>
+      <c r="J40" s="44"/>
     </row>
     <row r="41" s="37" customFormat="1" ht="46" customHeight="1" spans="1:10">
       <c r="A41" s="6">
@@ -3410,7 +3419,7 @@
       <c r="G46" s="26"/>
       <c r="H46" s="26"/>
       <c r="I46" s="26"/>
-      <c r="J46" s="43"/>
+      <c r="J46" s="44"/>
     </row>
     <row r="47" ht="45" customHeight="1" spans="1:10">
       <c r="A47" s="5">
@@ -3680,7 +3689,7 @@
       <c r="G55" s="26"/>
       <c r="H55" s="26"/>
       <c r="I55" s="26"/>
-      <c r="J55" s="43"/>
+      <c r="J55" s="44"/>
     </row>
     <row r="56" ht="45" customHeight="1" spans="1:10">
       <c r="A56" s="5">
@@ -3889,7 +3898,7 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
   <dimension ref="A1:I18"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.4"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="5" customWidth="1"/>
     <col min="2" max="2" width="25" customWidth="1"/>
@@ -4176,7 +4185,7 @@
         <v>196</v>
       </c>
     </row>
-    <row r="13" ht="26.4" spans="1:9">
+    <row r="13" ht="25.5" spans="1:9">
       <c r="A13" s="5">
         <v>8</v>
       </c>
@@ -4205,7 +4214,7 @@
         <v>197</v>
       </c>
     </row>
-    <row r="14" ht="26.4" spans="1:9">
+    <row r="14" ht="25.5" spans="1:9">
       <c r="A14" s="5">
         <v>9</v>
       </c>
@@ -4234,7 +4243,7 @@
         <v>198</v>
       </c>
     </row>
-    <row r="15" ht="26.4" spans="1:9">
+    <row r="15" ht="25.5" spans="1:9">
       <c r="A15" s="5">
         <v>10</v>
       </c>
@@ -4263,7 +4272,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="16" ht="26.4" spans="1:9">
+    <row r="16" ht="25.5" spans="1:9">
       <c r="A16" s="5">
         <v>11</v>
       </c>
@@ -4292,7 +4301,7 @@
         <v>201</v>
       </c>
     </row>
-    <row r="17" ht="26.4" spans="1:9">
+    <row r="17" ht="25.5" spans="1:9">
       <c r="A17" s="5">
         <v>12</v>
       </c>
@@ -4321,7 +4330,7 @@
         <v>202</v>
       </c>
     </row>
-    <row r="18" ht="26.4" spans="1:9">
+    <row r="18" ht="25.5" spans="1:9">
       <c r="A18" s="5">
         <v>13</v>
       </c>
@@ -4365,7 +4374,7 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
   <dimension ref="A1:I37"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.4"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="5" customWidth="1"/>
     <col min="2" max="2" width="25" customWidth="1"/>
@@ -5342,7 +5351,7 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
   <dimension ref="A1:I17"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.4"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="5" customWidth="1"/>
     <col min="2" max="2" width="25" customWidth="1"/>
@@ -5755,7 +5764,7 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
   <dimension ref="A1:F30"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.4" outlineLevelCol="5"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="15" outlineLevelCol="5"/>
   <cols>
     <col min="1" max="1" width="14" customWidth="1"/>
     <col min="2" max="2" width="42" customWidth="1"/>

</xml_diff>

<commit_message>
Xong chức năng phản hồi và gửi thông báo
</commit_message>
<xml_diff>
--- a/Project_Tracking.xlsx
+++ b/Project_Tracking.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="20760" windowHeight="12300"/>
+    <workbookView windowWidth="28800" windowHeight="12885"/>
   </bookViews>
   <sheets>
     <sheet name="Project Tracking" sheetId="1" r:id="rId1"/>
@@ -996,13 +996,13 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.4"/>
+        <fgColor rgb="FFFFFF00"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFFFFF00"/>
+        <fgColor theme="4" tint="0.4"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -1510,7 +1510,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="45">
+  <cellXfs count="46">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -1579,6 +1579,12 @@
     <xf numFmtId="0" fontId="3" fillId="9" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="10" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="8" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
@@ -1620,9 +1626,6 @@
     <xf numFmtId="0" fontId="9" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="10" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="8" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -2088,13 +2091,13 @@
     <col min="4" max="4" width="22" customWidth="1"/>
     <col min="5" max="5" width="60" customWidth="1"/>
     <col min="6" max="7" width="14" customWidth="1"/>
-    <col min="8" max="8" width="10" style="38" customWidth="1"/>
+    <col min="8" max="8" width="10" style="40" customWidth="1"/>
     <col min="9" max="9" width="14" customWidth="1"/>
     <col min="10" max="10" width="30" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" ht="40" customHeight="1" spans="1:10">
-      <c r="A1" s="39" t="s">
+      <c r="A1" s="41" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="8"/>
@@ -2103,7 +2106,7 @@
       <c r="E1" s="8"/>
       <c r="F1" s="8"/>
       <c r="G1" s="8"/>
-      <c r="H1" s="40"/>
+      <c r="H1" s="42"/>
       <c r="I1" s="8"/>
       <c r="J1" s="9"/>
     </row>
@@ -2117,7 +2120,7 @@
       <c r="E2" s="8"/>
       <c r="F2" s="8"/>
       <c r="G2" s="8"/>
-      <c r="H2" s="40"/>
+      <c r="H2" s="42"/>
       <c r="I2" s="8"/>
       <c r="J2" s="9"/>
     </row>
@@ -2153,26 +2156,26 @@
         <v>11</v>
       </c>
     </row>
-    <row r="4" s="37" customFormat="1" ht="28" customHeight="1" spans="1:8">
-      <c r="A4" s="29" t="s">
+    <row r="4" s="39" customFormat="1" ht="28" customHeight="1" spans="1:8">
+      <c r="A4" s="31" t="s">
         <v>12</v>
       </c>
-      <c r="H4" s="41"/>
+      <c r="H4" s="43"/>
     </row>
     <row r="5" ht="45" customHeight="1" spans="1:10">
-      <c r="A5" s="27">
+      <c r="A5" s="29">
         <v>1</v>
       </c>
-      <c r="B5" s="27" t="s">
+      <c r="B5" s="29" t="s">
         <v>13</v>
       </c>
-      <c r="C5" s="27" t="s">
+      <c r="C5" s="29" t="s">
         <v>14</v>
       </c>
-      <c r="D5" s="27" t="s">
+      <c r="D5" s="29" t="s">
         <v>15</v>
       </c>
-      <c r="E5" s="27" t="s">
+      <c r="E5" s="29" t="s">
         <v>16</v>
       </c>
       <c r="F5" s="5" t="s">
@@ -2181,28 +2184,28 @@
       <c r="G5" s="5" t="s">
         <v>18</v>
       </c>
-      <c r="H5" s="42" t="s">
+      <c r="H5" s="44" t="s">
         <v>19</v>
       </c>
-      <c r="I5" s="30"/>
+      <c r="I5" s="32"/>
       <c r="J5" s="5" t="s">
         <v>20</v>
       </c>
     </row>
     <row r="6" ht="45" customHeight="1" spans="1:10">
-      <c r="A6" s="27">
+      <c r="A6" s="29">
         <v>2</v>
       </c>
-      <c r="B6" s="27" t="s">
+      <c r="B6" s="29" t="s">
         <v>21</v>
       </c>
-      <c r="C6" s="27" t="s">
+      <c r="C6" s="29" t="s">
         <v>22</v>
       </c>
-      <c r="D6" s="27" t="s">
+      <c r="D6" s="29" t="s">
         <v>23</v>
       </c>
-      <c r="E6" s="27" t="s">
+      <c r="E6" s="29" t="s">
         <v>24</v>
       </c>
       <c r="F6" s="5" t="s">
@@ -2211,28 +2214,28 @@
       <c r="G6" s="5" t="s">
         <v>18</v>
       </c>
-      <c r="H6" s="42" t="s">
+      <c r="H6" s="44" t="s">
         <v>19</v>
       </c>
-      <c r="I6" s="30"/>
+      <c r="I6" s="32"/>
       <c r="J6" s="5" t="s">
         <v>20</v>
       </c>
     </row>
     <row r="7" ht="45" customHeight="1" spans="1:10">
-      <c r="A7" s="27">
+      <c r="A7" s="29">
         <v>3</v>
       </c>
-      <c r="B7" s="27" t="s">
+      <c r="B7" s="29" t="s">
         <v>25</v>
       </c>
-      <c r="C7" s="27" t="s">
+      <c r="C7" s="29" t="s">
         <v>26</v>
       </c>
-      <c r="D7" s="27" t="s">
+      <c r="D7" s="29" t="s">
         <v>15</v>
       </c>
-      <c r="E7" s="27" t="s">
+      <c r="E7" s="29" t="s">
         <v>27</v>
       </c>
       <c r="F7" s="5" t="s">
@@ -2241,28 +2244,28 @@
       <c r="G7" s="5" t="s">
         <v>18</v>
       </c>
-      <c r="H7" s="42" t="s">
+      <c r="H7" s="44" t="s">
         <v>19</v>
       </c>
-      <c r="I7" s="30"/>
+      <c r="I7" s="32"/>
       <c r="J7" s="5" t="s">
         <v>20</v>
       </c>
     </row>
     <row r="8" ht="45" customHeight="1" spans="1:10">
-      <c r="A8" s="27">
+      <c r="A8" s="29">
         <v>4</v>
       </c>
-      <c r="B8" s="27" t="s">
+      <c r="B8" s="29" t="s">
         <v>28</v>
       </c>
-      <c r="C8" s="27" t="s">
+      <c r="C8" s="29" t="s">
         <v>29</v>
       </c>
-      <c r="D8" s="27" t="s">
+      <c r="D8" s="29" t="s">
         <v>15</v>
       </c>
-      <c r="E8" s="27" t="s">
+      <c r="E8" s="29" t="s">
         <v>30</v>
       </c>
       <c r="F8" s="5" t="s">
@@ -2271,28 +2274,28 @@
       <c r="G8" s="5" t="s">
         <v>18</v>
       </c>
-      <c r="H8" s="42" t="s">
+      <c r="H8" s="44" t="s">
         <v>19</v>
       </c>
-      <c r="I8" s="30"/>
+      <c r="I8" s="32"/>
       <c r="J8" s="5" t="s">
         <v>20</v>
       </c>
     </row>
     <row r="9" ht="45" customHeight="1" spans="1:10">
-      <c r="A9" s="27">
+      <c r="A9" s="29">
         <v>5</v>
       </c>
-      <c r="B9" s="27" t="s">
+      <c r="B9" s="29" t="s">
         <v>31</v>
       </c>
-      <c r="C9" s="27" t="s">
+      <c r="C9" s="29" t="s">
         <v>32</v>
       </c>
-      <c r="D9" s="27" t="s">
+      <c r="D9" s="29" t="s">
         <v>15</v>
       </c>
-      <c r="E9" s="27" t="s">
+      <c r="E9" s="29" t="s">
         <v>33</v>
       </c>
       <c r="F9" s="5" t="s">
@@ -2301,10 +2304,10 @@
       <c r="G9" s="5" t="s">
         <v>18</v>
       </c>
-      <c r="H9" s="42" t="s">
+      <c r="H9" s="44" t="s">
         <v>19</v>
       </c>
-      <c r="I9" s="30"/>
+      <c r="I9" s="32"/>
       <c r="J9" s="5" t="s">
         <v>20</v>
       </c>
@@ -2313,15 +2316,15 @@
       <c r="A10" s="23" t="s">
         <v>34</v>
       </c>
-      <c r="B10" s="26"/>
-      <c r="C10" s="26"/>
-      <c r="D10" s="26"/>
-      <c r="E10" s="26"/>
-      <c r="F10" s="26"/>
-      <c r="G10" s="26"/>
-      <c r="H10" s="26"/>
-      <c r="I10" s="26"/>
-      <c r="J10" s="44"/>
+      <c r="B10" s="28"/>
+      <c r="C10" s="28"/>
+      <c r="D10" s="28"/>
+      <c r="E10" s="28"/>
+      <c r="F10" s="28"/>
+      <c r="G10" s="28"/>
+      <c r="H10" s="28"/>
+      <c r="I10" s="28"/>
+      <c r="J10" s="45"/>
     </row>
     <row r="11" ht="45" customHeight="1" spans="1:10">
       <c r="A11" s="5">
@@ -2345,7 +2348,7 @@
       <c r="G11" s="5" t="s">
         <v>18</v>
       </c>
-      <c r="H11" s="42" t="s">
+      <c r="H11" s="44" t="s">
         <v>19</v>
       </c>
       <c r="I11" s="5" t="s">
@@ -2377,7 +2380,7 @@
       <c r="G12" s="5" t="s">
         <v>18</v>
       </c>
-      <c r="H12" s="42" t="s">
+      <c r="H12" s="44" t="s">
         <v>19</v>
       </c>
       <c r="I12" s="5" t="s">
@@ -2409,7 +2412,7 @@
       <c r="G13" s="5" t="s">
         <v>18</v>
       </c>
-      <c r="H13" s="42" t="s">
+      <c r="H13" s="44" t="s">
         <v>19</v>
       </c>
       <c r="I13" s="5" t="s">
@@ -2441,7 +2444,7 @@
       <c r="G14" s="5" t="s">
         <v>18</v>
       </c>
-      <c r="H14" s="42" t="s">
+      <c r="H14" s="44" t="s">
         <v>19</v>
       </c>
       <c r="I14" s="5" t="s">
@@ -2473,7 +2476,7 @@
       <c r="G15" s="5" t="s">
         <v>18</v>
       </c>
-      <c r="H15" s="42" t="s">
+      <c r="H15" s="44" t="s">
         <v>19</v>
       </c>
       <c r="I15" s="5" t="s">
@@ -2505,7 +2508,7 @@
       <c r="G16" s="5" t="s">
         <v>18</v>
       </c>
-      <c r="H16" s="42" t="s">
+      <c r="H16" s="44" t="s">
         <v>19</v>
       </c>
       <c r="I16" s="5" t="s">
@@ -2537,7 +2540,7 @@
       <c r="G17" s="5" t="s">
         <v>18</v>
       </c>
-      <c r="H17" s="42" t="s">
+      <c r="H17" s="44" t="s">
         <v>19</v>
       </c>
       <c r="I17" s="5" t="s">
@@ -2569,7 +2572,7 @@
       <c r="G18" s="5" t="s">
         <v>18</v>
       </c>
-      <c r="H18" s="42" t="s">
+      <c r="H18" s="44" t="s">
         <v>19</v>
       </c>
       <c r="I18" s="5" t="s">
@@ -2601,7 +2604,7 @@
       <c r="G19" s="5" t="s">
         <v>63</v>
       </c>
-      <c r="H19" s="42" t="s">
+      <c r="H19" s="44" t="s">
         <v>64</v>
       </c>
       <c r="I19" s="5" t="s">
@@ -2633,7 +2636,7 @@
       <c r="G20" s="5" t="s">
         <v>63</v>
       </c>
-      <c r="H20" s="42" t="s">
+      <c r="H20" s="44" t="s">
         <v>64</v>
       </c>
       <c r="I20" s="5" t="s">
@@ -2665,7 +2668,7 @@
       <c r="G21" s="5" t="s">
         <v>63</v>
       </c>
-      <c r="H21" s="42" t="s">
+      <c r="H21" s="44" t="s">
         <v>64</v>
       </c>
       <c r="I21" s="5" t="s">
@@ -2675,7 +2678,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="22" s="37" customFormat="1" ht="28" customHeight="1" spans="1:10">
+    <row r="22" s="39" customFormat="1" ht="28" customHeight="1" spans="1:10">
       <c r="A22" s="6">
         <v>17</v>
       </c>
@@ -2697,7 +2700,7 @@
       <c r="G22" s="5" t="s">
         <v>63</v>
       </c>
-      <c r="H22" s="42" t="s">
+      <c r="H22" s="44" t="s">
         <v>64</v>
       </c>
       <c r="I22" s="5" t="s">
@@ -2729,7 +2732,7 @@
       <c r="G23" s="5" t="s">
         <v>63</v>
       </c>
-      <c r="H23" s="42" t="s">
+      <c r="H23" s="44" t="s">
         <v>64</v>
       </c>
       <c r="I23" s="5" t="s">
@@ -2761,7 +2764,7 @@
       <c r="G24" s="5" t="s">
         <v>63</v>
       </c>
-      <c r="H24" s="42" t="s">
+      <c r="H24" s="44" t="s">
         <v>64</v>
       </c>
       <c r="I24" s="5" t="s">
@@ -2793,7 +2796,7 @@
       <c r="G25" s="5" t="s">
         <v>63</v>
       </c>
-      <c r="H25" s="42" t="s">
+      <c r="H25" s="44" t="s">
         <v>64</v>
       </c>
       <c r="I25" s="5" t="s">
@@ -2825,7 +2828,7 @@
       <c r="G26" s="5" t="s">
         <v>63</v>
       </c>
-      <c r="H26" s="42" t="s">
+      <c r="H26" s="44" t="s">
         <v>84</v>
       </c>
       <c r="I26" s="5" t="s">
@@ -2857,7 +2860,7 @@
       <c r="G27" s="5" t="s">
         <v>63</v>
       </c>
-      <c r="H27" s="42" t="s">
+      <c r="H27" s="44" t="s">
         <v>84</v>
       </c>
       <c r="I27" s="5" t="s">
@@ -2871,15 +2874,15 @@
       <c r="A28" s="23" t="s">
         <v>88</v>
       </c>
-      <c r="B28" s="26"/>
-      <c r="C28" s="26"/>
-      <c r="D28" s="26"/>
-      <c r="E28" s="26"/>
-      <c r="F28" s="26"/>
-      <c r="G28" s="26"/>
-      <c r="H28" s="26"/>
-      <c r="I28" s="26"/>
-      <c r="J28" s="44"/>
+      <c r="B28" s="28"/>
+      <c r="C28" s="28"/>
+      <c r="D28" s="28"/>
+      <c r="E28" s="28"/>
+      <c r="F28" s="28"/>
+      <c r="G28" s="28"/>
+      <c r="H28" s="28"/>
+      <c r="I28" s="28"/>
+      <c r="J28" s="45"/>
     </row>
     <row r="29" ht="45" customHeight="1" spans="1:10">
       <c r="A29" s="5">
@@ -2903,7 +2906,7 @@
       <c r="G29" s="24" t="s">
         <v>18</v>
       </c>
-      <c r="H29" s="42" t="s">
+      <c r="H29" s="44" t="s">
         <v>64</v>
       </c>
       <c r="I29" s="5" t="s">
@@ -2935,7 +2938,7 @@
       <c r="G30" s="24" t="s">
         <v>18</v>
       </c>
-      <c r="H30" s="42" t="s">
+      <c r="H30" s="44" t="s">
         <v>64</v>
       </c>
       <c r="I30" s="5" t="s">
@@ -2967,7 +2970,7 @@
       <c r="G31" s="24" t="s">
         <v>18</v>
       </c>
-      <c r="H31" s="42" t="s">
+      <c r="H31" s="44" t="s">
         <v>64</v>
       </c>
       <c r="I31" s="5" t="s">
@@ -2999,7 +3002,7 @@
       <c r="G32" s="24" t="s">
         <v>18</v>
       </c>
-      <c r="H32" s="42" t="s">
+      <c r="H32" s="44" t="s">
         <v>64</v>
       </c>
       <c r="I32" s="5" t="s">
@@ -3028,10 +3031,10 @@
       <c r="F33" s="5" t="s">
         <v>93</v>
       </c>
-      <c r="G33" s="43" t="s">
+      <c r="G33" s="25" t="s">
         <v>63</v>
       </c>
-      <c r="H33" s="42" t="s">
+      <c r="H33" s="44" t="s">
         <v>64</v>
       </c>
       <c r="I33" s="5" t="s">
@@ -3041,29 +3044,29 @@
         <v>20</v>
       </c>
     </row>
-    <row r="34" s="37" customFormat="1" ht="38" customHeight="1" spans="1:10">
+    <row r="34" s="39" customFormat="1" ht="38" customHeight="1" spans="1:10">
       <c r="A34" s="5">
         <v>28</v>
       </c>
-      <c r="B34" s="5" t="s">
+      <c r="B34" s="29" t="s">
         <v>103</v>
       </c>
-      <c r="C34" s="27" t="s">
+      <c r="C34" s="29" t="s">
         <v>104</v>
       </c>
-      <c r="D34" s="27" t="s">
+      <c r="D34" s="29" t="s">
         <v>91</v>
       </c>
-      <c r="E34" s="27" t="s">
+      <c r="E34" s="29" t="s">
         <v>105</v>
       </c>
       <c r="F34" s="5" t="s">
         <v>93</v>
       </c>
-      <c r="G34" s="43" t="s">
+      <c r="G34" s="25" t="s">
         <v>63</v>
       </c>
-      <c r="H34" s="42" t="s">
+      <c r="H34" s="44" t="s">
         <v>64</v>
       </c>
       <c r="I34" s="5" t="s">
@@ -3095,7 +3098,7 @@
       <c r="G35" s="5" t="s">
         <v>18</v>
       </c>
-      <c r="H35" s="42" t="s">
+      <c r="H35" s="44" t="s">
         <v>64</v>
       </c>
       <c r="I35" s="5" t="s">
@@ -3127,7 +3130,7 @@
       <c r="G36" s="5" t="s">
         <v>18</v>
       </c>
-      <c r="H36" s="42" t="s">
+      <c r="H36" s="44" t="s">
         <v>64</v>
       </c>
       <c r="I36" s="5" t="s">
@@ -3159,7 +3162,7 @@
       <c r="G37" s="5" t="s">
         <v>18</v>
       </c>
-      <c r="H37" s="42" t="s">
+      <c r="H37" s="44" t="s">
         <v>64</v>
       </c>
       <c r="I37" s="5" t="s">
@@ -3191,7 +3194,7 @@
       <c r="G38" s="5" t="s">
         <v>18</v>
       </c>
-      <c r="H38" s="42" t="s">
+      <c r="H38" s="44" t="s">
         <v>64</v>
       </c>
       <c r="I38" s="5" t="s">
@@ -3223,7 +3226,7 @@
       <c r="G39" s="5" t="s">
         <v>18</v>
       </c>
-      <c r="H39" s="42" t="s">
+      <c r="H39" s="44" t="s">
         <v>64</v>
       </c>
       <c r="I39" s="5" t="s">
@@ -3237,17 +3240,17 @@
       <c r="A40" s="23" t="s">
         <v>118</v>
       </c>
-      <c r="B40" s="26"/>
-      <c r="C40" s="26"/>
-      <c r="D40" s="26"/>
-      <c r="E40" s="26"/>
-      <c r="F40" s="26"/>
-      <c r="G40" s="26"/>
-      <c r="H40" s="26"/>
-      <c r="I40" s="26"/>
-      <c r="J40" s="44"/>
-    </row>
-    <row r="41" s="37" customFormat="1" ht="46" customHeight="1" spans="1:10">
+      <c r="B40" s="28"/>
+      <c r="C40" s="28"/>
+      <c r="D40" s="28"/>
+      <c r="E40" s="28"/>
+      <c r="F40" s="28"/>
+      <c r="G40" s="28"/>
+      <c r="H40" s="28"/>
+      <c r="I40" s="28"/>
+      <c r="J40" s="45"/>
+    </row>
+    <row r="41" s="39" customFormat="1" ht="46" customHeight="1" spans="1:10">
       <c r="A41" s="6">
         <v>34</v>
       </c>
@@ -3269,7 +3272,7 @@
       <c r="G41" s="5" t="s">
         <v>63</v>
       </c>
-      <c r="H41" s="42" t="s">
+      <c r="H41" s="44" t="s">
         <v>64</v>
       </c>
       <c r="I41" s="5" t="s">
@@ -3301,7 +3304,7 @@
       <c r="G42" s="5" t="s">
         <v>63</v>
       </c>
-      <c r="H42" s="42" t="s">
+      <c r="H42" s="44" t="s">
         <v>64</v>
       </c>
       <c r="I42" s="5" t="s">
@@ -3333,7 +3336,7 @@
       <c r="G43" s="5" t="s">
         <v>63</v>
       </c>
-      <c r="H43" s="42" t="s">
+      <c r="H43" s="44" t="s">
         <v>64</v>
       </c>
       <c r="I43" s="5" t="s">
@@ -3365,7 +3368,7 @@
       <c r="G44" s="5" t="s">
         <v>63</v>
       </c>
-      <c r="H44" s="42" t="s">
+      <c r="H44" s="44" t="s">
         <v>64</v>
       </c>
       <c r="I44" s="5" t="s">
@@ -3397,7 +3400,7 @@
       <c r="G45" s="5" t="s">
         <v>63</v>
       </c>
-      <c r="H45" s="42" t="s">
+      <c r="H45" s="44" t="s">
         <v>64</v>
       </c>
       <c r="I45" s="5" t="s">
@@ -3411,15 +3414,15 @@
       <c r="A46" s="23" t="s">
         <v>136</v>
       </c>
-      <c r="B46" s="26"/>
-      <c r="C46" s="26"/>
-      <c r="D46" s="26"/>
-      <c r="E46" s="26"/>
-      <c r="F46" s="26"/>
-      <c r="G46" s="26"/>
-      <c r="H46" s="26"/>
-      <c r="I46" s="26"/>
-      <c r="J46" s="44"/>
+      <c r="B46" s="28"/>
+      <c r="C46" s="28"/>
+      <c r="D46" s="28"/>
+      <c r="E46" s="28"/>
+      <c r="F46" s="28"/>
+      <c r="G46" s="28"/>
+      <c r="H46" s="28"/>
+      <c r="I46" s="28"/>
+      <c r="J46" s="45"/>
     </row>
     <row r="47" ht="45" customHeight="1" spans="1:10">
       <c r="A47" s="5">
@@ -3443,7 +3446,7 @@
       <c r="G47" s="5" t="s">
         <v>63</v>
       </c>
-      <c r="H47" s="42" t="s">
+      <c r="H47" s="44" t="s">
         <v>64</v>
       </c>
       <c r="I47" s="5" t="s">
@@ -3475,7 +3478,7 @@
       <c r="G48" s="5" t="s">
         <v>63</v>
       </c>
-      <c r="H48" s="42" t="s">
+      <c r="H48" s="44" t="s">
         <v>64</v>
       </c>
       <c r="I48" s="5" t="s">
@@ -3507,7 +3510,7 @@
       <c r="G49" s="5" t="s">
         <v>63</v>
       </c>
-      <c r="H49" s="42" t="s">
+      <c r="H49" s="44" t="s">
         <v>64</v>
       </c>
       <c r="I49" s="5" t="s">
@@ -3517,20 +3520,20 @@
         <v>20</v>
       </c>
     </row>
-    <row r="50" s="37" customFormat="1" ht="28" customHeight="1" spans="1:10">
+    <row r="50" s="39" customFormat="1" ht="28" customHeight="1" spans="1:10">
       <c r="A50" s="5">
         <v>42</v>
       </c>
-      <c r="B50" s="27" t="s">
+      <c r="B50" s="29" t="s">
         <v>147</v>
       </c>
-      <c r="C50" s="27" t="s">
+      <c r="C50" s="29" t="s">
         <v>148</v>
       </c>
-      <c r="D50" s="27" t="s">
+      <c r="D50" s="29" t="s">
         <v>139</v>
       </c>
-      <c r="E50" s="27" t="s">
+      <c r="E50" s="29" t="s">
         <v>149</v>
       </c>
       <c r="F50" s="5" t="s">
@@ -3539,7 +3542,7 @@
       <c r="G50" s="5" t="s">
         <v>63</v>
       </c>
-      <c r="H50" s="42" t="s">
+      <c r="H50" s="44" t="s">
         <v>64</v>
       </c>
       <c r="I50" s="5" t="s">
@@ -3571,7 +3574,7 @@
       <c r="G51" s="5" t="s">
         <v>63</v>
       </c>
-      <c r="H51" s="42" t="s">
+      <c r="H51" s="44" t="s">
         <v>64</v>
       </c>
       <c r="I51" s="5" t="s">
@@ -3603,7 +3606,7 @@
       <c r="G52" s="5" t="s">
         <v>63</v>
       </c>
-      <c r="H52" s="42" t="s">
+      <c r="H52" s="44" t="s">
         <v>84</v>
       </c>
       <c r="I52" s="5" t="s">
@@ -3635,7 +3638,7 @@
       <c r="G53" s="5" t="s">
         <v>63</v>
       </c>
-      <c r="H53" s="42" t="s">
+      <c r="H53" s="44" t="s">
         <v>64</v>
       </c>
       <c r="I53" s="5" t="s">
@@ -3667,7 +3670,7 @@
       <c r="G54" s="5" t="s">
         <v>63</v>
       </c>
-      <c r="H54" s="42" t="s">
+      <c r="H54" s="44" t="s">
         <v>84</v>
       </c>
       <c r="I54" s="5" t="s">
@@ -3681,15 +3684,15 @@
       <c r="A55" s="23" t="s">
         <v>161</v>
       </c>
-      <c r="B55" s="26"/>
-      <c r="C55" s="26"/>
-      <c r="D55" s="26"/>
-      <c r="E55" s="26"/>
-      <c r="F55" s="26"/>
-      <c r="G55" s="26"/>
-      <c r="H55" s="26"/>
-      <c r="I55" s="26"/>
-      <c r="J55" s="44"/>
+      <c r="B55" s="28"/>
+      <c r="C55" s="28"/>
+      <c r="D55" s="28"/>
+      <c r="E55" s="28"/>
+      <c r="F55" s="28"/>
+      <c r="G55" s="28"/>
+      <c r="H55" s="28"/>
+      <c r="I55" s="28"/>
+      <c r="J55" s="45"/>
     </row>
     <row r="56" ht="45" customHeight="1" spans="1:10">
       <c r="A56" s="5">
@@ -3713,7 +3716,7 @@
       <c r="G56" s="5" t="s">
         <v>63</v>
       </c>
-      <c r="H56" s="42" t="s">
+      <c r="H56" s="44" t="s">
         <v>84</v>
       </c>
       <c r="I56" s="5" t="s">
@@ -3745,7 +3748,7 @@
       <c r="G57" s="5" t="s">
         <v>63</v>
       </c>
-      <c r="H57" s="42" t="s">
+      <c r="H57" s="44" t="s">
         <v>84</v>
       </c>
       <c r="I57" s="5" t="s">
@@ -3777,7 +3780,7 @@
       <c r="G58" s="5" t="s">
         <v>63</v>
       </c>
-      <c r="H58" s="42" t="s">
+      <c r="H58" s="44" t="s">
         <v>84</v>
       </c>
       <c r="I58" s="5" t="s">
@@ -3809,7 +3812,7 @@
       <c r="G59" s="5" t="s">
         <v>63</v>
       </c>
-      <c r="H59" s="42" t="s">
+      <c r="H59" s="44" t="s">
         <v>84</v>
       </c>
       <c r="I59" s="5" t="s">
@@ -3841,7 +3844,7 @@
       <c r="G60" s="5" t="s">
         <v>63</v>
       </c>
-      <c r="H60" s="42" t="s">
+      <c r="H60" s="44" t="s">
         <v>84</v>
       </c>
       <c r="I60" s="5" t="s">
@@ -3873,7 +3876,7 @@
       <c r="G61" s="5" t="s">
         <v>63</v>
       </c>
-      <c r="H61" s="42" t="s">
+      <c r="H61" s="44" t="s">
         <v>84</v>
       </c>
       <c r="I61" s="5" t="s">
@@ -3965,152 +3968,152 @@
       </c>
     </row>
     <row r="4" ht="28" customHeight="1" spans="1:1">
-      <c r="A4" s="29" t="s">
+      <c r="A4" s="31" t="s">
         <v>12</v>
       </c>
     </row>
     <row r="5" ht="45" customHeight="1" spans="1:9">
-      <c r="A5" s="30">
+      <c r="A5" s="32">
         <v>1</v>
       </c>
-      <c r="B5" s="30" t="s">
+      <c r="B5" s="32" t="s">
         <v>13</v>
       </c>
-      <c r="C5" s="30" t="s">
+      <c r="C5" s="32" t="s">
         <v>14</v>
       </c>
-      <c r="D5" s="30" t="s">
+      <c r="D5" s="32" t="s">
         <v>16</v>
       </c>
-      <c r="E5" s="30" t="s">
+      <c r="E5" s="32" t="s">
         <v>17</v>
       </c>
-      <c r="F5" s="31" t="s">
+      <c r="F5" s="33" t="s">
         <v>18</v>
       </c>
-      <c r="G5" s="32" t="s">
-        <v>20</v>
-      </c>
-      <c r="H5" s="32" t="s">
-        <v>20</v>
-      </c>
-      <c r="I5" s="34" t="s">
+      <c r="G5" s="34" t="s">
+        <v>20</v>
+      </c>
+      <c r="H5" s="34" t="s">
+        <v>20</v>
+      </c>
+      <c r="I5" s="36" t="s">
         <v>187</v>
       </c>
     </row>
     <row r="6" ht="45" customHeight="1" spans="1:9">
-      <c r="A6" s="30">
+      <c r="A6" s="32">
         <v>2</v>
       </c>
-      <c r="B6" s="30" t="s">
+      <c r="B6" s="32" t="s">
         <v>21</v>
       </c>
-      <c r="C6" s="30" t="s">
+      <c r="C6" s="32" t="s">
         <v>22</v>
       </c>
-      <c r="D6" s="30" t="s">
+      <c r="D6" s="32" t="s">
         <v>24</v>
       </c>
-      <c r="E6" s="30" t="s">
+      <c r="E6" s="32" t="s">
         <v>17</v>
       </c>
-      <c r="F6" s="31" t="s">
+      <c r="F6" s="33" t="s">
         <v>18</v>
       </c>
-      <c r="G6" s="32" t="s">
-        <v>20</v>
-      </c>
-      <c r="H6" s="32" t="s">
-        <v>20</v>
-      </c>
-      <c r="I6" s="34" t="s">
+      <c r="G6" s="34" t="s">
+        <v>20</v>
+      </c>
+      <c r="H6" s="34" t="s">
+        <v>20</v>
+      </c>
+      <c r="I6" s="36" t="s">
         <v>188</v>
       </c>
     </row>
     <row r="7" ht="45" customHeight="1" spans="1:9">
-      <c r="A7" s="30">
+      <c r="A7" s="32">
         <v>3</v>
       </c>
-      <c r="B7" s="30" t="s">
+      <c r="B7" s="32" t="s">
         <v>25</v>
       </c>
-      <c r="C7" s="30" t="s">
+      <c r="C7" s="32" t="s">
         <v>26</v>
       </c>
-      <c r="D7" s="30" t="s">
+      <c r="D7" s="32" t="s">
         <v>27</v>
       </c>
-      <c r="E7" s="30" t="s">
+      <c r="E7" s="32" t="s">
         <v>17</v>
       </c>
-      <c r="F7" s="31" t="s">
+      <c r="F7" s="33" t="s">
         <v>18</v>
       </c>
-      <c r="G7" s="32" t="s">
-        <v>20</v>
-      </c>
-      <c r="H7" s="32" t="s">
-        <v>20</v>
-      </c>
-      <c r="I7" s="34" t="s">
+      <c r="G7" s="34" t="s">
+        <v>20</v>
+      </c>
+      <c r="H7" s="34" t="s">
+        <v>20</v>
+      </c>
+      <c r="I7" s="36" t="s">
         <v>189</v>
       </c>
     </row>
     <row r="8" ht="45" customHeight="1" spans="1:9">
-      <c r="A8" s="30">
+      <c r="A8" s="32">
         <v>4</v>
       </c>
-      <c r="B8" s="30" t="s">
+      <c r="B8" s="32" t="s">
         <v>28</v>
       </c>
-      <c r="C8" s="30" t="s">
+      <c r="C8" s="32" t="s">
         <v>29</v>
       </c>
-      <c r="D8" s="30" t="s">
+      <c r="D8" s="32" t="s">
         <v>30</v>
       </c>
-      <c r="E8" s="30" t="s">
+      <c r="E8" s="32" t="s">
         <v>17</v>
       </c>
-      <c r="F8" s="31" t="s">
+      <c r="F8" s="33" t="s">
         <v>18</v>
       </c>
-      <c r="G8" s="32" t="s">
-        <v>20</v>
-      </c>
-      <c r="H8" s="32" t="s">
-        <v>20</v>
-      </c>
-      <c r="I8" s="34" t="s">
+      <c r="G8" s="34" t="s">
+        <v>20</v>
+      </c>
+      <c r="H8" s="34" t="s">
+        <v>20</v>
+      </c>
+      <c r="I8" s="36" t="s">
         <v>190</v>
       </c>
     </row>
     <row r="9" ht="45" customHeight="1" spans="1:9">
-      <c r="A9" s="30">
+      <c r="A9" s="32">
         <v>5</v>
       </c>
-      <c r="B9" s="30" t="s">
+      <c r="B9" s="32" t="s">
         <v>31</v>
       </c>
-      <c r="C9" s="30" t="s">
+      <c r="C9" s="32" t="s">
         <v>191</v>
       </c>
-      <c r="D9" s="30" t="s">
+      <c r="D9" s="32" t="s">
         <v>192</v>
       </c>
-      <c r="E9" s="30" t="s">
+      <c r="E9" s="32" t="s">
         <v>17</v>
       </c>
-      <c r="F9" s="31" t="s">
+      <c r="F9" s="33" t="s">
         <v>18</v>
       </c>
-      <c r="G9" s="32" t="s">
-        <v>20</v>
-      </c>
-      <c r="H9" s="32" t="s">
-        <v>20</v>
-      </c>
-      <c r="I9" s="34" t="s">
+      <c r="G9" s="34" t="s">
+        <v>20</v>
+      </c>
+      <c r="H9" s="34" t="s">
+        <v>20</v>
+      </c>
+      <c r="I9" s="36" t="s">
         <v>193</v>
       </c>
     </row>
@@ -4118,14 +4121,14 @@
       <c r="A10" s="23" t="s">
         <v>34</v>
       </c>
-      <c r="B10" s="26"/>
-      <c r="C10" s="26"/>
-      <c r="D10" s="26"/>
-      <c r="E10" s="26"/>
-      <c r="F10" s="33"/>
-      <c r="G10" s="26"/>
-      <c r="H10" s="26"/>
-      <c r="I10" s="35"/>
+      <c r="B10" s="28"/>
+      <c r="C10" s="28"/>
+      <c r="D10" s="28"/>
+      <c r="E10" s="28"/>
+      <c r="F10" s="35"/>
+      <c r="G10" s="28"/>
+      <c r="H10" s="28"/>
+      <c r="I10" s="37"/>
     </row>
     <row r="11" ht="45" customHeight="1" spans="1:9">
       <c r="A11" s="5">
@@ -4143,7 +4146,7 @@
       <c r="E11" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="F11" s="31" t="s">
+      <c r="F11" s="33" t="s">
         <v>194</v>
       </c>
       <c r="G11" s="5" t="s">
@@ -4152,7 +4155,7 @@
       <c r="H11" s="5" t="s">
         <v>20</v>
       </c>
-      <c r="I11" s="36" t="s">
+      <c r="I11" s="38" t="s">
         <v>195</v>
       </c>
     </row>
@@ -4166,13 +4169,13 @@
       <c r="C12" s="6" t="s">
         <v>39</v>
       </c>
-      <c r="D12" s="30" t="s">
+      <c r="D12" s="32" t="s">
         <v>40</v>
       </c>
       <c r="E12" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="F12" s="31" t="s">
+      <c r="F12" s="33" t="s">
         <v>18</v>
       </c>
       <c r="G12" s="5" t="s">
@@ -4181,7 +4184,7 @@
       <c r="H12" s="5" t="s">
         <v>20</v>
       </c>
-      <c r="I12" s="36" t="s">
+      <c r="I12" s="38" t="s">
         <v>196</v>
       </c>
     </row>
@@ -4201,7 +4204,7 @@
       <c r="E13" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="F13" s="31" t="s">
+      <c r="F13" s="33" t="s">
         <v>18</v>
       </c>
       <c r="G13" s="5" t="s">
@@ -4210,7 +4213,7 @@
       <c r="H13" s="5" t="s">
         <v>20</v>
       </c>
-      <c r="I13" s="36" t="s">
+      <c r="I13" s="38" t="s">
         <v>197</v>
       </c>
     </row>
@@ -4230,7 +4233,7 @@
       <c r="E14" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="F14" s="31" t="s">
+      <c r="F14" s="33" t="s">
         <v>18</v>
       </c>
       <c r="G14" s="5" t="s">
@@ -4239,7 +4242,7 @@
       <c r="H14" s="5" t="s">
         <v>20</v>
       </c>
-      <c r="I14" s="36" t="s">
+      <c r="I14" s="38" t="s">
         <v>198</v>
       </c>
     </row>
@@ -4259,7 +4262,7 @@
       <c r="E15" s="5" t="s">
         <v>50</v>
       </c>
-      <c r="F15" s="31" t="s">
+      <c r="F15" s="33" t="s">
         <v>199</v>
       </c>
       <c r="G15" s="5" t="s">
@@ -4268,7 +4271,7 @@
       <c r="H15" s="5" t="s">
         <v>20</v>
       </c>
-      <c r="I15" s="36" t="s">
+      <c r="I15" s="38" t="s">
         <v>200</v>
       </c>
     </row>
@@ -4288,7 +4291,7 @@
       <c r="E16" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="F16" s="31" t="s">
+      <c r="F16" s="33" t="s">
         <v>18</v>
       </c>
       <c r="G16" s="5" t="s">
@@ -4297,7 +4300,7 @@
       <c r="H16" s="5" t="s">
         <v>20</v>
       </c>
-      <c r="I16" s="36" t="s">
+      <c r="I16" s="38" t="s">
         <v>201</v>
       </c>
     </row>
@@ -4317,7 +4320,7 @@
       <c r="E17" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="F17" s="31" t="s">
+      <c r="F17" s="33" t="s">
         <v>194</v>
       </c>
       <c r="G17" s="5" t="s">
@@ -4326,7 +4329,7 @@
       <c r="H17" s="5" t="s">
         <v>20</v>
       </c>
-      <c r="I17" s="36" t="s">
+      <c r="I17" s="38" t="s">
         <v>202</v>
       </c>
     </row>
@@ -4346,7 +4349,7 @@
       <c r="E18" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="F18" s="31" t="s">
+      <c r="F18" s="33" t="s">
         <v>18</v>
       </c>
       <c r="G18" s="5" t="s">
@@ -4355,7 +4358,7 @@
       <c r="H18" s="5" t="s">
         <v>20</v>
       </c>
-      <c r="I18" s="36" t="s">
+      <c r="I18" s="38" t="s">
         <v>203</v>
       </c>
     </row>
@@ -4830,8 +4833,8 @@
       <c r="E18" s="5" t="s">
         <v>93</v>
       </c>
-      <c r="F18" s="25" t="s">
-        <v>63</v>
+      <c r="F18" s="26" t="s">
+        <v>194</v>
       </c>
       <c r="G18" s="5" t="s">
         <v>20</v>
@@ -4859,8 +4862,8 @@
       <c r="E19" s="5" t="s">
         <v>93</v>
       </c>
-      <c r="F19" s="25" t="s">
-        <v>63</v>
+      <c r="F19" s="27" t="s">
+        <v>18</v>
       </c>
       <c r="G19" s="5" t="s">
         <v>20</v>
@@ -5150,26 +5153,26 @@
       <c r="A30" s="23" t="s">
         <v>136</v>
       </c>
-      <c r="B30" s="26"/>
-      <c r="C30" s="26"/>
-      <c r="D30" s="26"/>
-      <c r="E30" s="26"/>
-      <c r="F30" s="26"/>
-      <c r="G30" s="26"/>
-      <c r="H30" s="26"/>
-      <c r="I30" s="28"/>
+      <c r="B30" s="28"/>
+      <c r="C30" s="28"/>
+      <c r="D30" s="28"/>
+      <c r="E30" s="28"/>
+      <c r="F30" s="28"/>
+      <c r="G30" s="28"/>
+      <c r="H30" s="28"/>
+      <c r="I30" s="30"/>
     </row>
     <row r="31" ht="28" customHeight="1" spans="1:9">
-      <c r="A31" s="27">
+      <c r="A31" s="29">
         <v>24</v>
       </c>
-      <c r="B31" s="27" t="s">
+      <c r="B31" s="29" t="s">
         <v>137</v>
       </c>
-      <c r="C31" s="27" t="s">
+      <c r="C31" s="29" t="s">
         <v>138</v>
       </c>
-      <c r="D31" s="27" t="s">
+      <c r="D31" s="29" t="s">
         <v>140</v>
       </c>
       <c r="E31" s="5" t="s">

</xml_diff>

<commit_message>
Revert "Xong chức năng phản hồi và gửi thông báo"
</commit_message>
<xml_diff>
--- a/Project_Tracking.xlsx
+++ b/Project_Tracking.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="28800" windowHeight="12885"/>
+    <workbookView windowWidth="20760" windowHeight="12300"/>
   </bookViews>
   <sheets>
     <sheet name="Project Tracking" sheetId="1" r:id="rId1"/>
@@ -996,13 +996,13 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFFFFF00"/>
+        <fgColor theme="4" tint="0.4"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.4"/>
+        <fgColor rgb="FFFFFF00"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -1510,7 +1510,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="46">
+  <cellXfs count="45">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -1579,12 +1579,6 @@
     <xf numFmtId="0" fontId="3" fillId="9" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="10" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="8" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
@@ -1626,6 +1620,9 @@
     <xf numFmtId="0" fontId="9" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="10" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="8" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -2091,13 +2088,13 @@
     <col min="4" max="4" width="22" customWidth="1"/>
     <col min="5" max="5" width="60" customWidth="1"/>
     <col min="6" max="7" width="14" customWidth="1"/>
-    <col min="8" max="8" width="10" style="40" customWidth="1"/>
+    <col min="8" max="8" width="10" style="38" customWidth="1"/>
     <col min="9" max="9" width="14" customWidth="1"/>
     <col min="10" max="10" width="30" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" ht="40" customHeight="1" spans="1:10">
-      <c r="A1" s="41" t="s">
+      <c r="A1" s="39" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="8"/>
@@ -2106,7 +2103,7 @@
       <c r="E1" s="8"/>
       <c r="F1" s="8"/>
       <c r="G1" s="8"/>
-      <c r="H1" s="42"/>
+      <c r="H1" s="40"/>
       <c r="I1" s="8"/>
       <c r="J1" s="9"/>
     </row>
@@ -2120,7 +2117,7 @@
       <c r="E2" s="8"/>
       <c r="F2" s="8"/>
       <c r="G2" s="8"/>
-      <c r="H2" s="42"/>
+      <c r="H2" s="40"/>
       <c r="I2" s="8"/>
       <c r="J2" s="9"/>
     </row>
@@ -2156,26 +2153,26 @@
         <v>11</v>
       </c>
     </row>
-    <row r="4" s="39" customFormat="1" ht="28" customHeight="1" spans="1:8">
-      <c r="A4" s="31" t="s">
+    <row r="4" s="37" customFormat="1" ht="28" customHeight="1" spans="1:8">
+      <c r="A4" s="29" t="s">
         <v>12</v>
       </c>
-      <c r="H4" s="43"/>
+      <c r="H4" s="41"/>
     </row>
     <row r="5" ht="45" customHeight="1" spans="1:10">
-      <c r="A5" s="29">
+      <c r="A5" s="27">
         <v>1</v>
       </c>
-      <c r="B5" s="29" t="s">
+      <c r="B5" s="27" t="s">
         <v>13</v>
       </c>
-      <c r="C5" s="29" t="s">
+      <c r="C5" s="27" t="s">
         <v>14</v>
       </c>
-      <c r="D5" s="29" t="s">
+      <c r="D5" s="27" t="s">
         <v>15</v>
       </c>
-      <c r="E5" s="29" t="s">
+      <c r="E5" s="27" t="s">
         <v>16</v>
       </c>
       <c r="F5" s="5" t="s">
@@ -2184,28 +2181,28 @@
       <c r="G5" s="5" t="s">
         <v>18</v>
       </c>
-      <c r="H5" s="44" t="s">
+      <c r="H5" s="42" t="s">
         <v>19</v>
       </c>
-      <c r="I5" s="32"/>
+      <c r="I5" s="30"/>
       <c r="J5" s="5" t="s">
         <v>20</v>
       </c>
     </row>
     <row r="6" ht="45" customHeight="1" spans="1:10">
-      <c r="A6" s="29">
+      <c r="A6" s="27">
         <v>2</v>
       </c>
-      <c r="B6" s="29" t="s">
+      <c r="B6" s="27" t="s">
         <v>21</v>
       </c>
-      <c r="C6" s="29" t="s">
+      <c r="C6" s="27" t="s">
         <v>22</v>
       </c>
-      <c r="D6" s="29" t="s">
+      <c r="D6" s="27" t="s">
         <v>23</v>
       </c>
-      <c r="E6" s="29" t="s">
+      <c r="E6" s="27" t="s">
         <v>24</v>
       </c>
       <c r="F6" s="5" t="s">
@@ -2214,28 +2211,28 @@
       <c r="G6" s="5" t="s">
         <v>18</v>
       </c>
-      <c r="H6" s="44" t="s">
+      <c r="H6" s="42" t="s">
         <v>19</v>
       </c>
-      <c r="I6" s="32"/>
+      <c r="I6" s="30"/>
       <c r="J6" s="5" t="s">
         <v>20</v>
       </c>
     </row>
     <row r="7" ht="45" customHeight="1" spans="1:10">
-      <c r="A7" s="29">
+      <c r="A7" s="27">
         <v>3</v>
       </c>
-      <c r="B7" s="29" t="s">
+      <c r="B7" s="27" t="s">
         <v>25</v>
       </c>
-      <c r="C7" s="29" t="s">
+      <c r="C7" s="27" t="s">
         <v>26</v>
       </c>
-      <c r="D7" s="29" t="s">
+      <c r="D7" s="27" t="s">
         <v>15</v>
       </c>
-      <c r="E7" s="29" t="s">
+      <c r="E7" s="27" t="s">
         <v>27</v>
       </c>
       <c r="F7" s="5" t="s">
@@ -2244,28 +2241,28 @@
       <c r="G7" s="5" t="s">
         <v>18</v>
       </c>
-      <c r="H7" s="44" t="s">
+      <c r="H7" s="42" t="s">
         <v>19</v>
       </c>
-      <c r="I7" s="32"/>
+      <c r="I7" s="30"/>
       <c r="J7" s="5" t="s">
         <v>20</v>
       </c>
     </row>
     <row r="8" ht="45" customHeight="1" spans="1:10">
-      <c r="A8" s="29">
+      <c r="A8" s="27">
         <v>4</v>
       </c>
-      <c r="B8" s="29" t="s">
+      <c r="B8" s="27" t="s">
         <v>28</v>
       </c>
-      <c r="C8" s="29" t="s">
+      <c r="C8" s="27" t="s">
         <v>29</v>
       </c>
-      <c r="D8" s="29" t="s">
+      <c r="D8" s="27" t="s">
         <v>15</v>
       </c>
-      <c r="E8" s="29" t="s">
+      <c r="E8" s="27" t="s">
         <v>30</v>
       </c>
       <c r="F8" s="5" t="s">
@@ -2274,28 +2271,28 @@
       <c r="G8" s="5" t="s">
         <v>18</v>
       </c>
-      <c r="H8" s="44" t="s">
+      <c r="H8" s="42" t="s">
         <v>19</v>
       </c>
-      <c r="I8" s="32"/>
+      <c r="I8" s="30"/>
       <c r="J8" s="5" t="s">
         <v>20</v>
       </c>
     </row>
     <row r="9" ht="45" customHeight="1" spans="1:10">
-      <c r="A9" s="29">
+      <c r="A9" s="27">
         <v>5</v>
       </c>
-      <c r="B9" s="29" t="s">
+      <c r="B9" s="27" t="s">
         <v>31</v>
       </c>
-      <c r="C9" s="29" t="s">
+      <c r="C9" s="27" t="s">
         <v>32</v>
       </c>
-      <c r="D9" s="29" t="s">
+      <c r="D9" s="27" t="s">
         <v>15</v>
       </c>
-      <c r="E9" s="29" t="s">
+      <c r="E9" s="27" t="s">
         <v>33</v>
       </c>
       <c r="F9" s="5" t="s">
@@ -2304,10 +2301,10 @@
       <c r="G9" s="5" t="s">
         <v>18</v>
       </c>
-      <c r="H9" s="44" t="s">
+      <c r="H9" s="42" t="s">
         <v>19</v>
       </c>
-      <c r="I9" s="32"/>
+      <c r="I9" s="30"/>
       <c r="J9" s="5" t="s">
         <v>20</v>
       </c>
@@ -2316,15 +2313,15 @@
       <c r="A10" s="23" t="s">
         <v>34</v>
       </c>
-      <c r="B10" s="28"/>
-      <c r="C10" s="28"/>
-      <c r="D10" s="28"/>
-      <c r="E10" s="28"/>
-      <c r="F10" s="28"/>
-      <c r="G10" s="28"/>
-      <c r="H10" s="28"/>
-      <c r="I10" s="28"/>
-      <c r="J10" s="45"/>
+      <c r="B10" s="26"/>
+      <c r="C10" s="26"/>
+      <c r="D10" s="26"/>
+      <c r="E10" s="26"/>
+      <c r="F10" s="26"/>
+      <c r="G10" s="26"/>
+      <c r="H10" s="26"/>
+      <c r="I10" s="26"/>
+      <c r="J10" s="44"/>
     </row>
     <row r="11" ht="45" customHeight="1" spans="1:10">
       <c r="A11" s="5">
@@ -2348,7 +2345,7 @@
       <c r="G11" s="5" t="s">
         <v>18</v>
       </c>
-      <c r="H11" s="44" t="s">
+      <c r="H11" s="42" t="s">
         <v>19</v>
       </c>
       <c r="I11" s="5" t="s">
@@ -2380,7 +2377,7 @@
       <c r="G12" s="5" t="s">
         <v>18</v>
       </c>
-      <c r="H12" s="44" t="s">
+      <c r="H12" s="42" t="s">
         <v>19</v>
       </c>
       <c r="I12" s="5" t="s">
@@ -2412,7 +2409,7 @@
       <c r="G13" s="5" t="s">
         <v>18</v>
       </c>
-      <c r="H13" s="44" t="s">
+      <c r="H13" s="42" t="s">
         <v>19</v>
       </c>
       <c r="I13" s="5" t="s">
@@ -2444,7 +2441,7 @@
       <c r="G14" s="5" t="s">
         <v>18</v>
       </c>
-      <c r="H14" s="44" t="s">
+      <c r="H14" s="42" t="s">
         <v>19</v>
       </c>
       <c r="I14" s="5" t="s">
@@ -2476,7 +2473,7 @@
       <c r="G15" s="5" t="s">
         <v>18</v>
       </c>
-      <c r="H15" s="44" t="s">
+      <c r="H15" s="42" t="s">
         <v>19</v>
       </c>
       <c r="I15" s="5" t="s">
@@ -2508,7 +2505,7 @@
       <c r="G16" s="5" t="s">
         <v>18</v>
       </c>
-      <c r="H16" s="44" t="s">
+      <c r="H16" s="42" t="s">
         <v>19</v>
       </c>
       <c r="I16" s="5" t="s">
@@ -2540,7 +2537,7 @@
       <c r="G17" s="5" t="s">
         <v>18</v>
       </c>
-      <c r="H17" s="44" t="s">
+      <c r="H17" s="42" t="s">
         <v>19</v>
       </c>
       <c r="I17" s="5" t="s">
@@ -2572,7 +2569,7 @@
       <c r="G18" s="5" t="s">
         <v>18</v>
       </c>
-      <c r="H18" s="44" t="s">
+      <c r="H18" s="42" t="s">
         <v>19</v>
       </c>
       <c r="I18" s="5" t="s">
@@ -2604,7 +2601,7 @@
       <c r="G19" s="5" t="s">
         <v>63</v>
       </c>
-      <c r="H19" s="44" t="s">
+      <c r="H19" s="42" t="s">
         <v>64</v>
       </c>
       <c r="I19" s="5" t="s">
@@ -2636,7 +2633,7 @@
       <c r="G20" s="5" t="s">
         <v>63</v>
       </c>
-      <c r="H20" s="44" t="s">
+      <c r="H20" s="42" t="s">
         <v>64</v>
       </c>
       <c r="I20" s="5" t="s">
@@ -2668,7 +2665,7 @@
       <c r="G21" s="5" t="s">
         <v>63</v>
       </c>
-      <c r="H21" s="44" t="s">
+      <c r="H21" s="42" t="s">
         <v>64</v>
       </c>
       <c r="I21" s="5" t="s">
@@ -2678,7 +2675,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="22" s="39" customFormat="1" ht="28" customHeight="1" spans="1:10">
+    <row r="22" s="37" customFormat="1" ht="28" customHeight="1" spans="1:10">
       <c r="A22" s="6">
         <v>17</v>
       </c>
@@ -2700,7 +2697,7 @@
       <c r="G22" s="5" t="s">
         <v>63</v>
       </c>
-      <c r="H22" s="44" t="s">
+      <c r="H22" s="42" t="s">
         <v>64</v>
       </c>
       <c r="I22" s="5" t="s">
@@ -2732,7 +2729,7 @@
       <c r="G23" s="5" t="s">
         <v>63</v>
       </c>
-      <c r="H23" s="44" t="s">
+      <c r="H23" s="42" t="s">
         <v>64</v>
       </c>
       <c r="I23" s="5" t="s">
@@ -2764,7 +2761,7 @@
       <c r="G24" s="5" t="s">
         <v>63</v>
       </c>
-      <c r="H24" s="44" t="s">
+      <c r="H24" s="42" t="s">
         <v>64</v>
       </c>
       <c r="I24" s="5" t="s">
@@ -2796,7 +2793,7 @@
       <c r="G25" s="5" t="s">
         <v>63</v>
       </c>
-      <c r="H25" s="44" t="s">
+      <c r="H25" s="42" t="s">
         <v>64</v>
       </c>
       <c r="I25" s="5" t="s">
@@ -2828,7 +2825,7 @@
       <c r="G26" s="5" t="s">
         <v>63</v>
       </c>
-      <c r="H26" s="44" t="s">
+      <c r="H26" s="42" t="s">
         <v>84</v>
       </c>
       <c r="I26" s="5" t="s">
@@ -2860,7 +2857,7 @@
       <c r="G27" s="5" t="s">
         <v>63</v>
       </c>
-      <c r="H27" s="44" t="s">
+      <c r="H27" s="42" t="s">
         <v>84</v>
       </c>
       <c r="I27" s="5" t="s">
@@ -2874,15 +2871,15 @@
       <c r="A28" s="23" t="s">
         <v>88</v>
       </c>
-      <c r="B28" s="28"/>
-      <c r="C28" s="28"/>
-      <c r="D28" s="28"/>
-      <c r="E28" s="28"/>
-      <c r="F28" s="28"/>
-      <c r="G28" s="28"/>
-      <c r="H28" s="28"/>
-      <c r="I28" s="28"/>
-      <c r="J28" s="45"/>
+      <c r="B28" s="26"/>
+      <c r="C28" s="26"/>
+      <c r="D28" s="26"/>
+      <c r="E28" s="26"/>
+      <c r="F28" s="26"/>
+      <c r="G28" s="26"/>
+      <c r="H28" s="26"/>
+      <c r="I28" s="26"/>
+      <c r="J28" s="44"/>
     </row>
     <row r="29" ht="45" customHeight="1" spans="1:10">
       <c r="A29" s="5">
@@ -2906,7 +2903,7 @@
       <c r="G29" s="24" t="s">
         <v>18</v>
       </c>
-      <c r="H29" s="44" t="s">
+      <c r="H29" s="42" t="s">
         <v>64</v>
       </c>
       <c r="I29" s="5" t="s">
@@ -2938,7 +2935,7 @@
       <c r="G30" s="24" t="s">
         <v>18</v>
       </c>
-      <c r="H30" s="44" t="s">
+      <c r="H30" s="42" t="s">
         <v>64</v>
       </c>
       <c r="I30" s="5" t="s">
@@ -2970,7 +2967,7 @@
       <c r="G31" s="24" t="s">
         <v>18</v>
       </c>
-      <c r="H31" s="44" t="s">
+      <c r="H31" s="42" t="s">
         <v>64</v>
       </c>
       <c r="I31" s="5" t="s">
@@ -3002,7 +2999,7 @@
       <c r="G32" s="24" t="s">
         <v>18</v>
       </c>
-      <c r="H32" s="44" t="s">
+      <c r="H32" s="42" t="s">
         <v>64</v>
       </c>
       <c r="I32" s="5" t="s">
@@ -3031,10 +3028,10 @@
       <c r="F33" s="5" t="s">
         <v>93</v>
       </c>
-      <c r="G33" s="25" t="s">
+      <c r="G33" s="43" t="s">
         <v>63</v>
       </c>
-      <c r="H33" s="44" t="s">
+      <c r="H33" s="42" t="s">
         <v>64</v>
       </c>
       <c r="I33" s="5" t="s">
@@ -3044,29 +3041,29 @@
         <v>20</v>
       </c>
     </row>
-    <row r="34" s="39" customFormat="1" ht="38" customHeight="1" spans="1:10">
+    <row r="34" s="37" customFormat="1" ht="38" customHeight="1" spans="1:10">
       <c r="A34" s="5">
         <v>28</v>
       </c>
-      <c r="B34" s="29" t="s">
+      <c r="B34" s="5" t="s">
         <v>103</v>
       </c>
-      <c r="C34" s="29" t="s">
+      <c r="C34" s="27" t="s">
         <v>104</v>
       </c>
-      <c r="D34" s="29" t="s">
+      <c r="D34" s="27" t="s">
         <v>91</v>
       </c>
-      <c r="E34" s="29" t="s">
+      <c r="E34" s="27" t="s">
         <v>105</v>
       </c>
       <c r="F34" s="5" t="s">
         <v>93</v>
       </c>
-      <c r="G34" s="25" t="s">
+      <c r="G34" s="43" t="s">
         <v>63</v>
       </c>
-      <c r="H34" s="44" t="s">
+      <c r="H34" s="42" t="s">
         <v>64</v>
       </c>
       <c r="I34" s="5" t="s">
@@ -3098,7 +3095,7 @@
       <c r="G35" s="5" t="s">
         <v>18</v>
       </c>
-      <c r="H35" s="44" t="s">
+      <c r="H35" s="42" t="s">
         <v>64</v>
       </c>
       <c r="I35" s="5" t="s">
@@ -3130,7 +3127,7 @@
       <c r="G36" s="5" t="s">
         <v>18</v>
       </c>
-      <c r="H36" s="44" t="s">
+      <c r="H36" s="42" t="s">
         <v>64</v>
       </c>
       <c r="I36" s="5" t="s">
@@ -3162,7 +3159,7 @@
       <c r="G37" s="5" t="s">
         <v>18</v>
       </c>
-      <c r="H37" s="44" t="s">
+      <c r="H37" s="42" t="s">
         <v>64</v>
       </c>
       <c r="I37" s="5" t="s">
@@ -3194,7 +3191,7 @@
       <c r="G38" s="5" t="s">
         <v>18</v>
       </c>
-      <c r="H38" s="44" t="s">
+      <c r="H38" s="42" t="s">
         <v>64</v>
       </c>
       <c r="I38" s="5" t="s">
@@ -3226,7 +3223,7 @@
       <c r="G39" s="5" t="s">
         <v>18</v>
       </c>
-      <c r="H39" s="44" t="s">
+      <c r="H39" s="42" t="s">
         <v>64</v>
       </c>
       <c r="I39" s="5" t="s">
@@ -3240,17 +3237,17 @@
       <c r="A40" s="23" t="s">
         <v>118</v>
       </c>
-      <c r="B40" s="28"/>
-      <c r="C40" s="28"/>
-      <c r="D40" s="28"/>
-      <c r="E40" s="28"/>
-      <c r="F40" s="28"/>
-      <c r="G40" s="28"/>
-      <c r="H40" s="28"/>
-      <c r="I40" s="28"/>
-      <c r="J40" s="45"/>
-    </row>
-    <row r="41" s="39" customFormat="1" ht="46" customHeight="1" spans="1:10">
+      <c r="B40" s="26"/>
+      <c r="C40" s="26"/>
+      <c r="D40" s="26"/>
+      <c r="E40" s="26"/>
+      <c r="F40" s="26"/>
+      <c r="G40" s="26"/>
+      <c r="H40" s="26"/>
+      <c r="I40" s="26"/>
+      <c r="J40" s="44"/>
+    </row>
+    <row r="41" s="37" customFormat="1" ht="46" customHeight="1" spans="1:10">
       <c r="A41" s="6">
         <v>34</v>
       </c>
@@ -3272,7 +3269,7 @@
       <c r="G41" s="5" t="s">
         <v>63</v>
       </c>
-      <c r="H41" s="44" t="s">
+      <c r="H41" s="42" t="s">
         <v>64</v>
       </c>
       <c r="I41" s="5" t="s">
@@ -3304,7 +3301,7 @@
       <c r="G42" s="5" t="s">
         <v>63</v>
       </c>
-      <c r="H42" s="44" t="s">
+      <c r="H42" s="42" t="s">
         <v>64</v>
       </c>
       <c r="I42" s="5" t="s">
@@ -3336,7 +3333,7 @@
       <c r="G43" s="5" t="s">
         <v>63</v>
       </c>
-      <c r="H43" s="44" t="s">
+      <c r="H43" s="42" t="s">
         <v>64</v>
       </c>
       <c r="I43" s="5" t="s">
@@ -3368,7 +3365,7 @@
       <c r="G44" s="5" t="s">
         <v>63</v>
       </c>
-      <c r="H44" s="44" t="s">
+      <c r="H44" s="42" t="s">
         <v>64</v>
       </c>
       <c r="I44" s="5" t="s">
@@ -3400,7 +3397,7 @@
       <c r="G45" s="5" t="s">
         <v>63</v>
       </c>
-      <c r="H45" s="44" t="s">
+      <c r="H45" s="42" t="s">
         <v>64</v>
       </c>
       <c r="I45" s="5" t="s">
@@ -3414,15 +3411,15 @@
       <c r="A46" s="23" t="s">
         <v>136</v>
       </c>
-      <c r="B46" s="28"/>
-      <c r="C46" s="28"/>
-      <c r="D46" s="28"/>
-      <c r="E46" s="28"/>
-      <c r="F46" s="28"/>
-      <c r="G46" s="28"/>
-      <c r="H46" s="28"/>
-      <c r="I46" s="28"/>
-      <c r="J46" s="45"/>
+      <c r="B46" s="26"/>
+      <c r="C46" s="26"/>
+      <c r="D46" s="26"/>
+      <c r="E46" s="26"/>
+      <c r="F46" s="26"/>
+      <c r="G46" s="26"/>
+      <c r="H46" s="26"/>
+      <c r="I46" s="26"/>
+      <c r="J46" s="44"/>
     </row>
     <row r="47" ht="45" customHeight="1" spans="1:10">
       <c r="A47" s="5">
@@ -3446,7 +3443,7 @@
       <c r="G47" s="5" t="s">
         <v>63</v>
       </c>
-      <c r="H47" s="44" t="s">
+      <c r="H47" s="42" t="s">
         <v>64</v>
       </c>
       <c r="I47" s="5" t="s">
@@ -3478,7 +3475,7 @@
       <c r="G48" s="5" t="s">
         <v>63</v>
       </c>
-      <c r="H48" s="44" t="s">
+      <c r="H48" s="42" t="s">
         <v>64</v>
       </c>
       <c r="I48" s="5" t="s">
@@ -3510,7 +3507,7 @@
       <c r="G49" s="5" t="s">
         <v>63</v>
       </c>
-      <c r="H49" s="44" t="s">
+      <c r="H49" s="42" t="s">
         <v>64</v>
       </c>
       <c r="I49" s="5" t="s">
@@ -3520,20 +3517,20 @@
         <v>20</v>
       </c>
     </row>
-    <row r="50" s="39" customFormat="1" ht="28" customHeight="1" spans="1:10">
+    <row r="50" s="37" customFormat="1" ht="28" customHeight="1" spans="1:10">
       <c r="A50" s="5">
         <v>42</v>
       </c>
-      <c r="B50" s="29" t="s">
+      <c r="B50" s="27" t="s">
         <v>147</v>
       </c>
-      <c r="C50" s="29" t="s">
+      <c r="C50" s="27" t="s">
         <v>148</v>
       </c>
-      <c r="D50" s="29" t="s">
+      <c r="D50" s="27" t="s">
         <v>139</v>
       </c>
-      <c r="E50" s="29" t="s">
+      <c r="E50" s="27" t="s">
         <v>149</v>
       </c>
       <c r="F50" s="5" t="s">
@@ -3542,7 +3539,7 @@
       <c r="G50" s="5" t="s">
         <v>63</v>
       </c>
-      <c r="H50" s="44" t="s">
+      <c r="H50" s="42" t="s">
         <v>64</v>
       </c>
       <c r="I50" s="5" t="s">
@@ -3574,7 +3571,7 @@
       <c r="G51" s="5" t="s">
         <v>63</v>
       </c>
-      <c r="H51" s="44" t="s">
+      <c r="H51" s="42" t="s">
         <v>64</v>
       </c>
       <c r="I51" s="5" t="s">
@@ -3606,7 +3603,7 @@
       <c r="G52" s="5" t="s">
         <v>63</v>
       </c>
-      <c r="H52" s="44" t="s">
+      <c r="H52" s="42" t="s">
         <v>84</v>
       </c>
       <c r="I52" s="5" t="s">
@@ -3638,7 +3635,7 @@
       <c r="G53" s="5" t="s">
         <v>63</v>
       </c>
-      <c r="H53" s="44" t="s">
+      <c r="H53" s="42" t="s">
         <v>64</v>
       </c>
       <c r="I53" s="5" t="s">
@@ -3670,7 +3667,7 @@
       <c r="G54" s="5" t="s">
         <v>63</v>
       </c>
-      <c r="H54" s="44" t="s">
+      <c r="H54" s="42" t="s">
         <v>84</v>
       </c>
       <c r="I54" s="5" t="s">
@@ -3684,15 +3681,15 @@
       <c r="A55" s="23" t="s">
         <v>161</v>
       </c>
-      <c r="B55" s="28"/>
-      <c r="C55" s="28"/>
-      <c r="D55" s="28"/>
-      <c r="E55" s="28"/>
-      <c r="F55" s="28"/>
-      <c r="G55" s="28"/>
-      <c r="H55" s="28"/>
-      <c r="I55" s="28"/>
-      <c r="J55" s="45"/>
+      <c r="B55" s="26"/>
+      <c r="C55" s="26"/>
+      <c r="D55" s="26"/>
+      <c r="E55" s="26"/>
+      <c r="F55" s="26"/>
+      <c r="G55" s="26"/>
+      <c r="H55" s="26"/>
+      <c r="I55" s="26"/>
+      <c r="J55" s="44"/>
     </row>
     <row r="56" ht="45" customHeight="1" spans="1:10">
       <c r="A56" s="5">
@@ -3716,7 +3713,7 @@
       <c r="G56" s="5" t="s">
         <v>63</v>
       </c>
-      <c r="H56" s="44" t="s">
+      <c r="H56" s="42" t="s">
         <v>84</v>
       </c>
       <c r="I56" s="5" t="s">
@@ -3748,7 +3745,7 @@
       <c r="G57" s="5" t="s">
         <v>63</v>
       </c>
-      <c r="H57" s="44" t="s">
+      <c r="H57" s="42" t="s">
         <v>84</v>
       </c>
       <c r="I57" s="5" t="s">
@@ -3780,7 +3777,7 @@
       <c r="G58" s="5" t="s">
         <v>63</v>
       </c>
-      <c r="H58" s="44" t="s">
+      <c r="H58" s="42" t="s">
         <v>84</v>
       </c>
       <c r="I58" s="5" t="s">
@@ -3812,7 +3809,7 @@
       <c r="G59" s="5" t="s">
         <v>63</v>
       </c>
-      <c r="H59" s="44" t="s">
+      <c r="H59" s="42" t="s">
         <v>84</v>
       </c>
       <c r="I59" s="5" t="s">
@@ -3844,7 +3841,7 @@
       <c r="G60" s="5" t="s">
         <v>63</v>
       </c>
-      <c r="H60" s="44" t="s">
+      <c r="H60" s="42" t="s">
         <v>84</v>
       </c>
       <c r="I60" s="5" t="s">
@@ -3876,7 +3873,7 @@
       <c r="G61" s="5" t="s">
         <v>63</v>
       </c>
-      <c r="H61" s="44" t="s">
+      <c r="H61" s="42" t="s">
         <v>84</v>
       </c>
       <c r="I61" s="5" t="s">
@@ -3968,152 +3965,152 @@
       </c>
     </row>
     <row r="4" ht="28" customHeight="1" spans="1:1">
-      <c r="A4" s="31" t="s">
+      <c r="A4" s="29" t="s">
         <v>12</v>
       </c>
     </row>
     <row r="5" ht="45" customHeight="1" spans="1:9">
-      <c r="A5" s="32">
+      <c r="A5" s="30">
         <v>1</v>
       </c>
-      <c r="B5" s="32" t="s">
+      <c r="B5" s="30" t="s">
         <v>13</v>
       </c>
-      <c r="C5" s="32" t="s">
+      <c r="C5" s="30" t="s">
         <v>14</v>
       </c>
-      <c r="D5" s="32" t="s">
+      <c r="D5" s="30" t="s">
         <v>16</v>
       </c>
-      <c r="E5" s="32" t="s">
+      <c r="E5" s="30" t="s">
         <v>17</v>
       </c>
-      <c r="F5" s="33" t="s">
+      <c r="F5" s="31" t="s">
         <v>18</v>
       </c>
-      <c r="G5" s="34" t="s">
-        <v>20</v>
-      </c>
-      <c r="H5" s="34" t="s">
-        <v>20</v>
-      </c>
-      <c r="I5" s="36" t="s">
+      <c r="G5" s="32" t="s">
+        <v>20</v>
+      </c>
+      <c r="H5" s="32" t="s">
+        <v>20</v>
+      </c>
+      <c r="I5" s="34" t="s">
         <v>187</v>
       </c>
     </row>
     <row r="6" ht="45" customHeight="1" spans="1:9">
-      <c r="A6" s="32">
+      <c r="A6" s="30">
         <v>2</v>
       </c>
-      <c r="B6" s="32" t="s">
+      <c r="B6" s="30" t="s">
         <v>21</v>
       </c>
-      <c r="C6" s="32" t="s">
+      <c r="C6" s="30" t="s">
         <v>22</v>
       </c>
-      <c r="D6" s="32" t="s">
+      <c r="D6" s="30" t="s">
         <v>24</v>
       </c>
-      <c r="E6" s="32" t="s">
+      <c r="E6" s="30" t="s">
         <v>17</v>
       </c>
-      <c r="F6" s="33" t="s">
+      <c r="F6" s="31" t="s">
         <v>18</v>
       </c>
-      <c r="G6" s="34" t="s">
-        <v>20</v>
-      </c>
-      <c r="H6" s="34" t="s">
-        <v>20</v>
-      </c>
-      <c r="I6" s="36" t="s">
+      <c r="G6" s="32" t="s">
+        <v>20</v>
+      </c>
+      <c r="H6" s="32" t="s">
+        <v>20</v>
+      </c>
+      <c r="I6" s="34" t="s">
         <v>188</v>
       </c>
     </row>
     <row r="7" ht="45" customHeight="1" spans="1:9">
-      <c r="A7" s="32">
+      <c r="A7" s="30">
         <v>3</v>
       </c>
-      <c r="B7" s="32" t="s">
+      <c r="B7" s="30" t="s">
         <v>25</v>
       </c>
-      <c r="C7" s="32" t="s">
+      <c r="C7" s="30" t="s">
         <v>26</v>
       </c>
-      <c r="D7" s="32" t="s">
+      <c r="D7" s="30" t="s">
         <v>27</v>
       </c>
-      <c r="E7" s="32" t="s">
+      <c r="E7" s="30" t="s">
         <v>17</v>
       </c>
-      <c r="F7" s="33" t="s">
+      <c r="F7" s="31" t="s">
         <v>18</v>
       </c>
-      <c r="G7" s="34" t="s">
-        <v>20</v>
-      </c>
-      <c r="H7" s="34" t="s">
-        <v>20</v>
-      </c>
-      <c r="I7" s="36" t="s">
+      <c r="G7" s="32" t="s">
+        <v>20</v>
+      </c>
+      <c r="H7" s="32" t="s">
+        <v>20</v>
+      </c>
+      <c r="I7" s="34" t="s">
         <v>189</v>
       </c>
     </row>
     <row r="8" ht="45" customHeight="1" spans="1:9">
-      <c r="A8" s="32">
+      <c r="A8" s="30">
         <v>4</v>
       </c>
-      <c r="B8" s="32" t="s">
+      <c r="B8" s="30" t="s">
         <v>28</v>
       </c>
-      <c r="C8" s="32" t="s">
+      <c r="C8" s="30" t="s">
         <v>29</v>
       </c>
-      <c r="D8" s="32" t="s">
+      <c r="D8" s="30" t="s">
         <v>30</v>
       </c>
-      <c r="E8" s="32" t="s">
+      <c r="E8" s="30" t="s">
         <v>17</v>
       </c>
-      <c r="F8" s="33" t="s">
+      <c r="F8" s="31" t="s">
         <v>18</v>
       </c>
-      <c r="G8" s="34" t="s">
-        <v>20</v>
-      </c>
-      <c r="H8" s="34" t="s">
-        <v>20</v>
-      </c>
-      <c r="I8" s="36" t="s">
+      <c r="G8" s="32" t="s">
+        <v>20</v>
+      </c>
+      <c r="H8" s="32" t="s">
+        <v>20</v>
+      </c>
+      <c r="I8" s="34" t="s">
         <v>190</v>
       </c>
     </row>
     <row r="9" ht="45" customHeight="1" spans="1:9">
-      <c r="A9" s="32">
+      <c r="A9" s="30">
         <v>5</v>
       </c>
-      <c r="B9" s="32" t="s">
+      <c r="B9" s="30" t="s">
         <v>31</v>
       </c>
-      <c r="C9" s="32" t="s">
+      <c r="C9" s="30" t="s">
         <v>191</v>
       </c>
-      <c r="D9" s="32" t="s">
+      <c r="D9" s="30" t="s">
         <v>192</v>
       </c>
-      <c r="E9" s="32" t="s">
+      <c r="E9" s="30" t="s">
         <v>17</v>
       </c>
-      <c r="F9" s="33" t="s">
+      <c r="F9" s="31" t="s">
         <v>18</v>
       </c>
-      <c r="G9" s="34" t="s">
-        <v>20</v>
-      </c>
-      <c r="H9" s="34" t="s">
-        <v>20</v>
-      </c>
-      <c r="I9" s="36" t="s">
+      <c r="G9" s="32" t="s">
+        <v>20</v>
+      </c>
+      <c r="H9" s="32" t="s">
+        <v>20</v>
+      </c>
+      <c r="I9" s="34" t="s">
         <v>193</v>
       </c>
     </row>
@@ -4121,14 +4118,14 @@
       <c r="A10" s="23" t="s">
         <v>34</v>
       </c>
-      <c r="B10" s="28"/>
-      <c r="C10" s="28"/>
-      <c r="D10" s="28"/>
-      <c r="E10" s="28"/>
-      <c r="F10" s="35"/>
-      <c r="G10" s="28"/>
-      <c r="H10" s="28"/>
-      <c r="I10" s="37"/>
+      <c r="B10" s="26"/>
+      <c r="C10" s="26"/>
+      <c r="D10" s="26"/>
+      <c r="E10" s="26"/>
+      <c r="F10" s="33"/>
+      <c r="G10" s="26"/>
+      <c r="H10" s="26"/>
+      <c r="I10" s="35"/>
     </row>
     <row r="11" ht="45" customHeight="1" spans="1:9">
       <c r="A11" s="5">
@@ -4146,7 +4143,7 @@
       <c r="E11" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="F11" s="33" t="s">
+      <c r="F11" s="31" t="s">
         <v>194</v>
       </c>
       <c r="G11" s="5" t="s">
@@ -4155,7 +4152,7 @@
       <c r="H11" s="5" t="s">
         <v>20</v>
       </c>
-      <c r="I11" s="38" t="s">
+      <c r="I11" s="36" t="s">
         <v>195</v>
       </c>
     </row>
@@ -4169,13 +4166,13 @@
       <c r="C12" s="6" t="s">
         <v>39</v>
       </c>
-      <c r="D12" s="32" t="s">
+      <c r="D12" s="30" t="s">
         <v>40</v>
       </c>
       <c r="E12" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="F12" s="33" t="s">
+      <c r="F12" s="31" t="s">
         <v>18</v>
       </c>
       <c r="G12" s="5" t="s">
@@ -4184,7 +4181,7 @@
       <c r="H12" s="5" t="s">
         <v>20</v>
       </c>
-      <c r="I12" s="38" t="s">
+      <c r="I12" s="36" t="s">
         <v>196</v>
       </c>
     </row>
@@ -4204,7 +4201,7 @@
       <c r="E13" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="F13" s="33" t="s">
+      <c r="F13" s="31" t="s">
         <v>18</v>
       </c>
       <c r="G13" s="5" t="s">
@@ -4213,7 +4210,7 @@
       <c r="H13" s="5" t="s">
         <v>20</v>
       </c>
-      <c r="I13" s="38" t="s">
+      <c r="I13" s="36" t="s">
         <v>197</v>
       </c>
     </row>
@@ -4233,7 +4230,7 @@
       <c r="E14" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="F14" s="33" t="s">
+      <c r="F14" s="31" t="s">
         <v>18</v>
       </c>
       <c r="G14" s="5" t="s">
@@ -4242,7 +4239,7 @@
       <c r="H14" s="5" t="s">
         <v>20</v>
       </c>
-      <c r="I14" s="38" t="s">
+      <c r="I14" s="36" t="s">
         <v>198</v>
       </c>
     </row>
@@ -4262,7 +4259,7 @@
       <c r="E15" s="5" t="s">
         <v>50</v>
       </c>
-      <c r="F15" s="33" t="s">
+      <c r="F15" s="31" t="s">
         <v>199</v>
       </c>
       <c r="G15" s="5" t="s">
@@ -4271,7 +4268,7 @@
       <c r="H15" s="5" t="s">
         <v>20</v>
       </c>
-      <c r="I15" s="38" t="s">
+      <c r="I15" s="36" t="s">
         <v>200</v>
       </c>
     </row>
@@ -4291,7 +4288,7 @@
       <c r="E16" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="F16" s="33" t="s">
+      <c r="F16" s="31" t="s">
         <v>18</v>
       </c>
       <c r="G16" s="5" t="s">
@@ -4300,7 +4297,7 @@
       <c r="H16" s="5" t="s">
         <v>20</v>
       </c>
-      <c r="I16" s="38" t="s">
+      <c r="I16" s="36" t="s">
         <v>201</v>
       </c>
     </row>
@@ -4320,7 +4317,7 @@
       <c r="E17" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="F17" s="33" t="s">
+      <c r="F17" s="31" t="s">
         <v>194</v>
       </c>
       <c r="G17" s="5" t="s">
@@ -4329,7 +4326,7 @@
       <c r="H17" s="5" t="s">
         <v>20</v>
       </c>
-      <c r="I17" s="38" t="s">
+      <c r="I17" s="36" t="s">
         <v>202</v>
       </c>
     </row>
@@ -4349,7 +4346,7 @@
       <c r="E18" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="F18" s="33" t="s">
+      <c r="F18" s="31" t="s">
         <v>18</v>
       </c>
       <c r="G18" s="5" t="s">
@@ -4358,7 +4355,7 @@
       <c r="H18" s="5" t="s">
         <v>20</v>
       </c>
-      <c r="I18" s="38" t="s">
+      <c r="I18" s="36" t="s">
         <v>203</v>
       </c>
     </row>
@@ -4833,8 +4830,8 @@
       <c r="E18" s="5" t="s">
         <v>93</v>
       </c>
-      <c r="F18" s="26" t="s">
-        <v>194</v>
+      <c r="F18" s="25" t="s">
+        <v>63</v>
       </c>
       <c r="G18" s="5" t="s">
         <v>20</v>
@@ -4862,8 +4859,8 @@
       <c r="E19" s="5" t="s">
         <v>93</v>
       </c>
-      <c r="F19" s="27" t="s">
-        <v>18</v>
+      <c r="F19" s="25" t="s">
+        <v>63</v>
       </c>
       <c r="G19" s="5" t="s">
         <v>20</v>
@@ -5153,26 +5150,26 @@
       <c r="A30" s="23" t="s">
         <v>136</v>
       </c>
-      <c r="B30" s="28"/>
-      <c r="C30" s="28"/>
-      <c r="D30" s="28"/>
-      <c r="E30" s="28"/>
-      <c r="F30" s="28"/>
-      <c r="G30" s="28"/>
-      <c r="H30" s="28"/>
-      <c r="I30" s="30"/>
+      <c r="B30" s="26"/>
+      <c r="C30" s="26"/>
+      <c r="D30" s="26"/>
+      <c r="E30" s="26"/>
+      <c r="F30" s="26"/>
+      <c r="G30" s="26"/>
+      <c r="H30" s="26"/>
+      <c r="I30" s="28"/>
     </row>
     <row r="31" ht="28" customHeight="1" spans="1:9">
-      <c r="A31" s="29">
+      <c r="A31" s="27">
         <v>24</v>
       </c>
-      <c r="B31" s="29" t="s">
+      <c r="B31" s="27" t="s">
         <v>137</v>
       </c>
-      <c r="C31" s="29" t="s">
+      <c r="C31" s="27" t="s">
         <v>138</v>
       </c>
-      <c r="D31" s="29" t="s">
+      <c r="D31" s="27" t="s">
         <v>140</v>
       </c>
       <c r="E31" s="5" t="s">

</xml_diff>

<commit_message>
Sửa lại lỗi ở phần quản lý tuyến
</commit_message>
<xml_diff>
--- a/Project_Tracking.xlsx
+++ b/Project_Tracking.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="28800" windowHeight="12885"/>
+    <workbookView windowWidth="23040" windowHeight="9707" activeTab="2"/>
   </bookViews>
   <sheets>
     <sheet name="Project Tracking" sheetId="1" r:id="rId1"/>
@@ -945,7 +945,7 @@
       <charset val="134"/>
     </font>
   </fonts>
-  <fills count="41">
+  <fills count="40">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -997,12 +997,6 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFFFFF00"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.4"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -1386,7 +1380,7 @@
     <xf numFmtId="0" fontId="13" fillId="0" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="11" borderId="6">
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="6">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="14" fillId="0" borderId="0">
@@ -1410,16 +1404,16 @@
     <xf numFmtId="0" fontId="19" fillId="0" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="12" borderId="9">
+    <xf numFmtId="0" fontId="20" fillId="11" borderId="9">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="13" borderId="10">
+    <xf numFmtId="0" fontId="21" fillId="12" borderId="10">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="13" borderId="9">
+    <xf numFmtId="0" fontId="22" fillId="12" borderId="9">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="23" fillId="14" borderId="11">
+    <xf numFmtId="0" fontId="23" fillId="13" borderId="11">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="24" fillId="0" borderId="12">
@@ -1431,86 +1425,86 @@
     <xf numFmtId="0" fontId="25" fillId="4" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="26" fillId="15" borderId="0">
+    <xf numFmtId="0" fontId="26" fillId="14" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="27" fillId="16" borderId="0">
+    <xf numFmtId="0" fontId="27" fillId="15" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="17" borderId="0">
+    <xf numFmtId="0" fontId="8" fillId="16" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="17" borderId="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="18" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="19" borderId="0">
+    <xf numFmtId="0" fontId="8" fillId="19" borderId="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="20" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="21" borderId="0">
+    <xf numFmtId="0" fontId="0" fillId="21" borderId="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="22" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="23" borderId="0">
+    <xf numFmtId="0" fontId="8" fillId="23" borderId="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="24" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="25" borderId="0">
+    <xf numFmtId="0" fontId="0" fillId="25" borderId="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="26" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="27" borderId="0">
+    <xf numFmtId="0" fontId="8" fillId="27" borderId="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="28" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="29" borderId="0">
+    <xf numFmtId="0" fontId="0" fillId="29" borderId="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="30" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="31" borderId="0">
+    <xf numFmtId="0" fontId="8" fillId="31" borderId="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="32" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="33" borderId="0">
+    <xf numFmtId="0" fontId="0" fillId="33" borderId="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="34" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0">
+    <xf numFmtId="0" fontId="8" fillId="35" borderId="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="36" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="37" borderId="0">
+    <xf numFmtId="0" fontId="0" fillId="37" borderId="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="38" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="39" borderId="0">
+    <xf numFmtId="0" fontId="8" fillId="39" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="40" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
   </cellStyleXfs>
-  <cellXfs count="46">
+  <cellXfs count="45">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -1577,9 +1571,6 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="9" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="10" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -2083,7 +2074,7 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
   <dimension ref="A1:J61"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="15"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.4"/>
   <cols>
     <col min="1" max="1" width="5" customWidth="1"/>
     <col min="2" max="2" width="25" customWidth="1"/>
@@ -2091,13 +2082,13 @@
     <col min="4" max="4" width="22" customWidth="1"/>
     <col min="5" max="5" width="60" customWidth="1"/>
     <col min="6" max="7" width="14" customWidth="1"/>
-    <col min="8" max="8" width="10" style="40" customWidth="1"/>
+    <col min="8" max="8" width="10" style="39" customWidth="1"/>
     <col min="9" max="9" width="14" customWidth="1"/>
     <col min="10" max="10" width="30" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" ht="40" customHeight="1" spans="1:10">
-      <c r="A1" s="41" t="s">
+      <c r="A1" s="40" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="8"/>
@@ -2106,7 +2097,7 @@
       <c r="E1" s="8"/>
       <c r="F1" s="8"/>
       <c r="G1" s="8"/>
-      <c r="H1" s="42"/>
+      <c r="H1" s="41"/>
       <c r="I1" s="8"/>
       <c r="J1" s="9"/>
     </row>
@@ -2120,7 +2111,7 @@
       <c r="E2" s="8"/>
       <c r="F2" s="8"/>
       <c r="G2" s="8"/>
-      <c r="H2" s="42"/>
+      <c r="H2" s="41"/>
       <c r="I2" s="8"/>
       <c r="J2" s="9"/>
     </row>
@@ -2156,26 +2147,26 @@
         <v>11</v>
       </c>
     </row>
-    <row r="4" s="39" customFormat="1" ht="28" customHeight="1" spans="1:8">
-      <c r="A4" s="31" t="s">
+    <row r="4" s="38" customFormat="1" ht="28" customHeight="1" spans="1:8">
+      <c r="A4" s="30" t="s">
         <v>12</v>
       </c>
-      <c r="H4" s="43"/>
+      <c r="H4" s="42"/>
     </row>
     <row r="5" ht="45" customHeight="1" spans="1:10">
-      <c r="A5" s="29">
+      <c r="A5" s="28">
         <v>1</v>
       </c>
-      <c r="B5" s="29" t="s">
+      <c r="B5" s="28" t="s">
         <v>13</v>
       </c>
-      <c r="C5" s="29" t="s">
+      <c r="C5" s="28" t="s">
         <v>14</v>
       </c>
-      <c r="D5" s="29" t="s">
+      <c r="D5" s="28" t="s">
         <v>15</v>
       </c>
-      <c r="E5" s="29" t="s">
+      <c r="E5" s="28" t="s">
         <v>16</v>
       </c>
       <c r="F5" s="5" t="s">
@@ -2184,28 +2175,28 @@
       <c r="G5" s="5" t="s">
         <v>18</v>
       </c>
-      <c r="H5" s="44" t="s">
+      <c r="H5" s="43" t="s">
         <v>19</v>
       </c>
-      <c r="I5" s="32"/>
+      <c r="I5" s="31"/>
       <c r="J5" s="5" t="s">
         <v>20</v>
       </c>
     </row>
     <row r="6" ht="45" customHeight="1" spans="1:10">
-      <c r="A6" s="29">
+      <c r="A6" s="28">
         <v>2</v>
       </c>
-      <c r="B6" s="29" t="s">
+      <c r="B6" s="28" t="s">
         <v>21</v>
       </c>
-      <c r="C6" s="29" t="s">
+      <c r="C6" s="28" t="s">
         <v>22</v>
       </c>
-      <c r="D6" s="29" t="s">
+      <c r="D6" s="28" t="s">
         <v>23</v>
       </c>
-      <c r="E6" s="29" t="s">
+      <c r="E6" s="28" t="s">
         <v>24</v>
       </c>
       <c r="F6" s="5" t="s">
@@ -2214,28 +2205,28 @@
       <c r="G6" s="5" t="s">
         <v>18</v>
       </c>
-      <c r="H6" s="44" t="s">
+      <c r="H6" s="43" t="s">
         <v>19</v>
       </c>
-      <c r="I6" s="32"/>
+      <c r="I6" s="31"/>
       <c r="J6" s="5" t="s">
         <v>20</v>
       </c>
     </row>
     <row r="7" ht="45" customHeight="1" spans="1:10">
-      <c r="A7" s="29">
+      <c r="A7" s="28">
         <v>3</v>
       </c>
-      <c r="B7" s="29" t="s">
+      <c r="B7" s="28" t="s">
         <v>25</v>
       </c>
-      <c r="C7" s="29" t="s">
+      <c r="C7" s="28" t="s">
         <v>26</v>
       </c>
-      <c r="D7" s="29" t="s">
+      <c r="D7" s="28" t="s">
         <v>15</v>
       </c>
-      <c r="E7" s="29" t="s">
+      <c r="E7" s="28" t="s">
         <v>27</v>
       </c>
       <c r="F7" s="5" t="s">
@@ -2244,28 +2235,28 @@
       <c r="G7" s="5" t="s">
         <v>18</v>
       </c>
-      <c r="H7" s="44" t="s">
+      <c r="H7" s="43" t="s">
         <v>19</v>
       </c>
-      <c r="I7" s="32"/>
+      <c r="I7" s="31"/>
       <c r="J7" s="5" t="s">
         <v>20</v>
       </c>
     </row>
     <row r="8" ht="45" customHeight="1" spans="1:10">
-      <c r="A8" s="29">
+      <c r="A8" s="28">
         <v>4</v>
       </c>
-      <c r="B8" s="29" t="s">
+      <c r="B8" s="28" t="s">
         <v>28</v>
       </c>
-      <c r="C8" s="29" t="s">
+      <c r="C8" s="28" t="s">
         <v>29</v>
       </c>
-      <c r="D8" s="29" t="s">
+      <c r="D8" s="28" t="s">
         <v>15</v>
       </c>
-      <c r="E8" s="29" t="s">
+      <c r="E8" s="28" t="s">
         <v>30</v>
       </c>
       <c r="F8" s="5" t="s">
@@ -2274,28 +2265,28 @@
       <c r="G8" s="5" t="s">
         <v>18</v>
       </c>
-      <c r="H8" s="44" t="s">
+      <c r="H8" s="43" t="s">
         <v>19</v>
       </c>
-      <c r="I8" s="32"/>
+      <c r="I8" s="31"/>
       <c r="J8" s="5" t="s">
         <v>20</v>
       </c>
     </row>
     <row r="9" ht="45" customHeight="1" spans="1:10">
-      <c r="A9" s="29">
+      <c r="A9" s="28">
         <v>5</v>
       </c>
-      <c r="B9" s="29" t="s">
+      <c r="B9" s="28" t="s">
         <v>31</v>
       </c>
-      <c r="C9" s="29" t="s">
+      <c r="C9" s="28" t="s">
         <v>32</v>
       </c>
-      <c r="D9" s="29" t="s">
+      <c r="D9" s="28" t="s">
         <v>15</v>
       </c>
-      <c r="E9" s="29" t="s">
+      <c r="E9" s="28" t="s">
         <v>33</v>
       </c>
       <c r="F9" s="5" t="s">
@@ -2304,10 +2295,10 @@
       <c r="G9" s="5" t="s">
         <v>18</v>
       </c>
-      <c r="H9" s="44" t="s">
+      <c r="H9" s="43" t="s">
         <v>19</v>
       </c>
-      <c r="I9" s="32"/>
+      <c r="I9" s="31"/>
       <c r="J9" s="5" t="s">
         <v>20</v>
       </c>
@@ -2316,15 +2307,15 @@
       <c r="A10" s="23" t="s">
         <v>34</v>
       </c>
-      <c r="B10" s="28"/>
-      <c r="C10" s="28"/>
-      <c r="D10" s="28"/>
-      <c r="E10" s="28"/>
-      <c r="F10" s="28"/>
-      <c r="G10" s="28"/>
-      <c r="H10" s="28"/>
-      <c r="I10" s="28"/>
-      <c r="J10" s="45"/>
+      <c r="B10" s="27"/>
+      <c r="C10" s="27"/>
+      <c r="D10" s="27"/>
+      <c r="E10" s="27"/>
+      <c r="F10" s="27"/>
+      <c r="G10" s="27"/>
+      <c r="H10" s="27"/>
+      <c r="I10" s="27"/>
+      <c r="J10" s="44"/>
     </row>
     <row r="11" ht="45" customHeight="1" spans="1:10">
       <c r="A11" s="5">
@@ -2348,7 +2339,7 @@
       <c r="G11" s="5" t="s">
         <v>18</v>
       </c>
-      <c r="H11" s="44" t="s">
+      <c r="H11" s="43" t="s">
         <v>19</v>
       </c>
       <c r="I11" s="5" t="s">
@@ -2380,7 +2371,7 @@
       <c r="G12" s="5" t="s">
         <v>18</v>
       </c>
-      <c r="H12" s="44" t="s">
+      <c r="H12" s="43" t="s">
         <v>19</v>
       </c>
       <c r="I12" s="5" t="s">
@@ -2412,7 +2403,7 @@
       <c r="G13" s="5" t="s">
         <v>18</v>
       </c>
-      <c r="H13" s="44" t="s">
+      <c r="H13" s="43" t="s">
         <v>19</v>
       </c>
       <c r="I13" s="5" t="s">
@@ -2444,7 +2435,7 @@
       <c r="G14" s="5" t="s">
         <v>18</v>
       </c>
-      <c r="H14" s="44" t="s">
+      <c r="H14" s="43" t="s">
         <v>19</v>
       </c>
       <c r="I14" s="5" t="s">
@@ -2476,7 +2467,7 @@
       <c r="G15" s="5" t="s">
         <v>18</v>
       </c>
-      <c r="H15" s="44" t="s">
+      <c r="H15" s="43" t="s">
         <v>19</v>
       </c>
       <c r="I15" s="5" t="s">
@@ -2508,7 +2499,7 @@
       <c r="G16" s="5" t="s">
         <v>18</v>
       </c>
-      <c r="H16" s="44" t="s">
+      <c r="H16" s="43" t="s">
         <v>19</v>
       </c>
       <c r="I16" s="5" t="s">
@@ -2540,7 +2531,7 @@
       <c r="G17" s="5" t="s">
         <v>18</v>
       </c>
-      <c r="H17" s="44" t="s">
+      <c r="H17" s="43" t="s">
         <v>19</v>
       </c>
       <c r="I17" s="5" t="s">
@@ -2572,7 +2563,7 @@
       <c r="G18" s="5" t="s">
         <v>18</v>
       </c>
-      <c r="H18" s="44" t="s">
+      <c r="H18" s="43" t="s">
         <v>19</v>
       </c>
       <c r="I18" s="5" t="s">
@@ -2604,7 +2595,7 @@
       <c r="G19" s="5" t="s">
         <v>63</v>
       </c>
-      <c r="H19" s="44" t="s">
+      <c r="H19" s="43" t="s">
         <v>64</v>
       </c>
       <c r="I19" s="5" t="s">
@@ -2636,7 +2627,7 @@
       <c r="G20" s="5" t="s">
         <v>63</v>
       </c>
-      <c r="H20" s="44" t="s">
+      <c r="H20" s="43" t="s">
         <v>64</v>
       </c>
       <c r="I20" s="5" t="s">
@@ -2668,7 +2659,7 @@
       <c r="G21" s="5" t="s">
         <v>63</v>
       </c>
-      <c r="H21" s="44" t="s">
+      <c r="H21" s="43" t="s">
         <v>64</v>
       </c>
       <c r="I21" s="5" t="s">
@@ -2678,7 +2669,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="22" s="39" customFormat="1" ht="28" customHeight="1" spans="1:10">
+    <row r="22" s="38" customFormat="1" ht="28" customHeight="1" spans="1:10">
       <c r="A22" s="6">
         <v>17</v>
       </c>
@@ -2700,7 +2691,7 @@
       <c r="G22" s="5" t="s">
         <v>63</v>
       </c>
-      <c r="H22" s="44" t="s">
+      <c r="H22" s="43" t="s">
         <v>64</v>
       </c>
       <c r="I22" s="5" t="s">
@@ -2732,7 +2723,7 @@
       <c r="G23" s="5" t="s">
         <v>63</v>
       </c>
-      <c r="H23" s="44" t="s">
+      <c r="H23" s="43" t="s">
         <v>64</v>
       </c>
       <c r="I23" s="5" t="s">
@@ -2764,7 +2755,7 @@
       <c r="G24" s="5" t="s">
         <v>63</v>
       </c>
-      <c r="H24" s="44" t="s">
+      <c r="H24" s="43" t="s">
         <v>64</v>
       </c>
       <c r="I24" s="5" t="s">
@@ -2796,7 +2787,7 @@
       <c r="G25" s="5" t="s">
         <v>63</v>
       </c>
-      <c r="H25" s="44" t="s">
+      <c r="H25" s="43" t="s">
         <v>64</v>
       </c>
       <c r="I25" s="5" t="s">
@@ -2828,7 +2819,7 @@
       <c r="G26" s="5" t="s">
         <v>63</v>
       </c>
-      <c r="H26" s="44" t="s">
+      <c r="H26" s="43" t="s">
         <v>84</v>
       </c>
       <c r="I26" s="5" t="s">
@@ -2860,7 +2851,7 @@
       <c r="G27" s="5" t="s">
         <v>63</v>
       </c>
-      <c r="H27" s="44" t="s">
+      <c r="H27" s="43" t="s">
         <v>84</v>
       </c>
       <c r="I27" s="5" t="s">
@@ -2874,15 +2865,15 @@
       <c r="A28" s="23" t="s">
         <v>88</v>
       </c>
-      <c r="B28" s="28"/>
-      <c r="C28" s="28"/>
-      <c r="D28" s="28"/>
-      <c r="E28" s="28"/>
-      <c r="F28" s="28"/>
-      <c r="G28" s="28"/>
-      <c r="H28" s="28"/>
-      <c r="I28" s="28"/>
-      <c r="J28" s="45"/>
+      <c r="B28" s="27"/>
+      <c r="C28" s="27"/>
+      <c r="D28" s="27"/>
+      <c r="E28" s="27"/>
+      <c r="F28" s="27"/>
+      <c r="G28" s="27"/>
+      <c r="H28" s="27"/>
+      <c r="I28" s="27"/>
+      <c r="J28" s="44"/>
     </row>
     <row r="29" ht="45" customHeight="1" spans="1:10">
       <c r="A29" s="5">
@@ -2906,7 +2897,7 @@
       <c r="G29" s="24" t="s">
         <v>18</v>
       </c>
-      <c r="H29" s="44" t="s">
+      <c r="H29" s="43" t="s">
         <v>64</v>
       </c>
       <c r="I29" s="5" t="s">
@@ -2938,7 +2929,7 @@
       <c r="G30" s="24" t="s">
         <v>18</v>
       </c>
-      <c r="H30" s="44" t="s">
+      <c r="H30" s="43" t="s">
         <v>64</v>
       </c>
       <c r="I30" s="5" t="s">
@@ -2970,7 +2961,7 @@
       <c r="G31" s="24" t="s">
         <v>18</v>
       </c>
-      <c r="H31" s="44" t="s">
+      <c r="H31" s="43" t="s">
         <v>64</v>
       </c>
       <c r="I31" s="5" t="s">
@@ -3002,7 +2993,7 @@
       <c r="G32" s="24" t="s">
         <v>18</v>
       </c>
-      <c r="H32" s="44" t="s">
+      <c r="H32" s="43" t="s">
         <v>64</v>
       </c>
       <c r="I32" s="5" t="s">
@@ -3034,7 +3025,7 @@
       <c r="G33" s="25" t="s">
         <v>63</v>
       </c>
-      <c r="H33" s="44" t="s">
+      <c r="H33" s="43" t="s">
         <v>64</v>
       </c>
       <c r="I33" s="5" t="s">
@@ -3044,29 +3035,29 @@
         <v>20</v>
       </c>
     </row>
-    <row r="34" s="39" customFormat="1" ht="38" customHeight="1" spans="1:10">
+    <row r="34" s="38" customFormat="1" ht="38" customHeight="1" spans="1:10">
       <c r="A34" s="5">
         <v>28</v>
       </c>
-      <c r="B34" s="29" t="s">
+      <c r="B34" s="28" t="s">
         <v>103</v>
       </c>
-      <c r="C34" s="29" t="s">
+      <c r="C34" s="28" t="s">
         <v>104</v>
       </c>
-      <c r="D34" s="29" t="s">
+      <c r="D34" s="28" t="s">
         <v>91</v>
       </c>
-      <c r="E34" s="29" t="s">
+      <c r="E34" s="28" t="s">
         <v>105</v>
       </c>
       <c r="F34" s="5" t="s">
         <v>93</v>
       </c>
-      <c r="G34" s="25" t="s">
-        <v>63</v>
-      </c>
-      <c r="H34" s="44" t="s">
+      <c r="G34" s="26" t="s">
+        <v>18</v>
+      </c>
+      <c r="H34" s="43" t="s">
         <v>64</v>
       </c>
       <c r="I34" s="5" t="s">
@@ -3098,7 +3089,7 @@
       <c r="G35" s="5" t="s">
         <v>18</v>
       </c>
-      <c r="H35" s="44" t="s">
+      <c r="H35" s="43" t="s">
         <v>64</v>
       </c>
       <c r="I35" s="5" t="s">
@@ -3130,7 +3121,7 @@
       <c r="G36" s="5" t="s">
         <v>18</v>
       </c>
-      <c r="H36" s="44" t="s">
+      <c r="H36" s="43" t="s">
         <v>64</v>
       </c>
       <c r="I36" s="5" t="s">
@@ -3162,7 +3153,7 @@
       <c r="G37" s="5" t="s">
         <v>18</v>
       </c>
-      <c r="H37" s="44" t="s">
+      <c r="H37" s="43" t="s">
         <v>64</v>
       </c>
       <c r="I37" s="5" t="s">
@@ -3194,7 +3185,7 @@
       <c r="G38" s="5" t="s">
         <v>18</v>
       </c>
-      <c r="H38" s="44" t="s">
+      <c r="H38" s="43" t="s">
         <v>64</v>
       </c>
       <c r="I38" s="5" t="s">
@@ -3226,7 +3217,7 @@
       <c r="G39" s="5" t="s">
         <v>18</v>
       </c>
-      <c r="H39" s="44" t="s">
+      <c r="H39" s="43" t="s">
         <v>64</v>
       </c>
       <c r="I39" s="5" t="s">
@@ -3240,17 +3231,17 @@
       <c r="A40" s="23" t="s">
         <v>118</v>
       </c>
-      <c r="B40" s="28"/>
-      <c r="C40" s="28"/>
-      <c r="D40" s="28"/>
-      <c r="E40" s="28"/>
-      <c r="F40" s="28"/>
-      <c r="G40" s="28"/>
-      <c r="H40" s="28"/>
-      <c r="I40" s="28"/>
-      <c r="J40" s="45"/>
-    </row>
-    <row r="41" s="39" customFormat="1" ht="46" customHeight="1" spans="1:10">
+      <c r="B40" s="27"/>
+      <c r="C40" s="27"/>
+      <c r="D40" s="27"/>
+      <c r="E40" s="27"/>
+      <c r="F40" s="27"/>
+      <c r="G40" s="27"/>
+      <c r="H40" s="27"/>
+      <c r="I40" s="27"/>
+      <c r="J40" s="44"/>
+    </row>
+    <row r="41" s="38" customFormat="1" ht="46" customHeight="1" spans="1:10">
       <c r="A41" s="6">
         <v>34</v>
       </c>
@@ -3272,7 +3263,7 @@
       <c r="G41" s="5" t="s">
         <v>63</v>
       </c>
-      <c r="H41" s="44" t="s">
+      <c r="H41" s="43" t="s">
         <v>64</v>
       </c>
       <c r="I41" s="5" t="s">
@@ -3304,7 +3295,7 @@
       <c r="G42" s="5" t="s">
         <v>63</v>
       </c>
-      <c r="H42" s="44" t="s">
+      <c r="H42" s="43" t="s">
         <v>64</v>
       </c>
       <c r="I42" s="5" t="s">
@@ -3336,7 +3327,7 @@
       <c r="G43" s="5" t="s">
         <v>63</v>
       </c>
-      <c r="H43" s="44" t="s">
+      <c r="H43" s="43" t="s">
         <v>64</v>
       </c>
       <c r="I43" s="5" t="s">
@@ -3368,7 +3359,7 @@
       <c r="G44" s="5" t="s">
         <v>63</v>
       </c>
-      <c r="H44" s="44" t="s">
+      <c r="H44" s="43" t="s">
         <v>64</v>
       </c>
       <c r="I44" s="5" t="s">
@@ -3400,7 +3391,7 @@
       <c r="G45" s="5" t="s">
         <v>63</v>
       </c>
-      <c r="H45" s="44" t="s">
+      <c r="H45" s="43" t="s">
         <v>64</v>
       </c>
       <c r="I45" s="5" t="s">
@@ -3414,15 +3405,15 @@
       <c r="A46" s="23" t="s">
         <v>136</v>
       </c>
-      <c r="B46" s="28"/>
-      <c r="C46" s="28"/>
-      <c r="D46" s="28"/>
-      <c r="E46" s="28"/>
-      <c r="F46" s="28"/>
-      <c r="G46" s="28"/>
-      <c r="H46" s="28"/>
-      <c r="I46" s="28"/>
-      <c r="J46" s="45"/>
+      <c r="B46" s="27"/>
+      <c r="C46" s="27"/>
+      <c r="D46" s="27"/>
+      <c r="E46" s="27"/>
+      <c r="F46" s="27"/>
+      <c r="G46" s="27"/>
+      <c r="H46" s="27"/>
+      <c r="I46" s="27"/>
+      <c r="J46" s="44"/>
     </row>
     <row r="47" ht="45" customHeight="1" spans="1:10">
       <c r="A47" s="5">
@@ -3446,7 +3437,7 @@
       <c r="G47" s="5" t="s">
         <v>63</v>
       </c>
-      <c r="H47" s="44" t="s">
+      <c r="H47" s="43" t="s">
         <v>64</v>
       </c>
       <c r="I47" s="5" t="s">
@@ -3478,7 +3469,7 @@
       <c r="G48" s="5" t="s">
         <v>63</v>
       </c>
-      <c r="H48" s="44" t="s">
+      <c r="H48" s="43" t="s">
         <v>64</v>
       </c>
       <c r="I48" s="5" t="s">
@@ -3510,7 +3501,7 @@
       <c r="G49" s="5" t="s">
         <v>63</v>
       </c>
-      <c r="H49" s="44" t="s">
+      <c r="H49" s="43" t="s">
         <v>64</v>
       </c>
       <c r="I49" s="5" t="s">
@@ -3520,20 +3511,20 @@
         <v>20</v>
       </c>
     </row>
-    <row r="50" s="39" customFormat="1" ht="28" customHeight="1" spans="1:10">
+    <row r="50" s="38" customFormat="1" ht="28" customHeight="1" spans="1:10">
       <c r="A50" s="5">
         <v>42</v>
       </c>
-      <c r="B50" s="29" t="s">
+      <c r="B50" s="28" t="s">
         <v>147</v>
       </c>
-      <c r="C50" s="29" t="s">
+      <c r="C50" s="28" t="s">
         <v>148</v>
       </c>
-      <c r="D50" s="29" t="s">
+      <c r="D50" s="28" t="s">
         <v>139</v>
       </c>
-      <c r="E50" s="29" t="s">
+      <c r="E50" s="28" t="s">
         <v>149</v>
       </c>
       <c r="F50" s="5" t="s">
@@ -3542,7 +3533,7 @@
       <c r="G50" s="5" t="s">
         <v>63</v>
       </c>
-      <c r="H50" s="44" t="s">
+      <c r="H50" s="43" t="s">
         <v>64</v>
       </c>
       <c r="I50" s="5" t="s">
@@ -3574,7 +3565,7 @@
       <c r="G51" s="5" t="s">
         <v>63</v>
       </c>
-      <c r="H51" s="44" t="s">
+      <c r="H51" s="43" t="s">
         <v>64</v>
       </c>
       <c r="I51" s="5" t="s">
@@ -3606,7 +3597,7 @@
       <c r="G52" s="5" t="s">
         <v>63</v>
       </c>
-      <c r="H52" s="44" t="s">
+      <c r="H52" s="43" t="s">
         <v>84</v>
       </c>
       <c r="I52" s="5" t="s">
@@ -3638,7 +3629,7 @@
       <c r="G53" s="5" t="s">
         <v>63</v>
       </c>
-      <c r="H53" s="44" t="s">
+      <c r="H53" s="43" t="s">
         <v>64</v>
       </c>
       <c r="I53" s="5" t="s">
@@ -3670,7 +3661,7 @@
       <c r="G54" s="5" t="s">
         <v>63</v>
       </c>
-      <c r="H54" s="44" t="s">
+      <c r="H54" s="43" t="s">
         <v>84</v>
       </c>
       <c r="I54" s="5" t="s">
@@ -3684,15 +3675,15 @@
       <c r="A55" s="23" t="s">
         <v>161</v>
       </c>
-      <c r="B55" s="28"/>
-      <c r="C55" s="28"/>
-      <c r="D55" s="28"/>
-      <c r="E55" s="28"/>
-      <c r="F55" s="28"/>
-      <c r="G55" s="28"/>
-      <c r="H55" s="28"/>
-      <c r="I55" s="28"/>
-      <c r="J55" s="45"/>
+      <c r="B55" s="27"/>
+      <c r="C55" s="27"/>
+      <c r="D55" s="27"/>
+      <c r="E55" s="27"/>
+      <c r="F55" s="27"/>
+      <c r="G55" s="27"/>
+      <c r="H55" s="27"/>
+      <c r="I55" s="27"/>
+      <c r="J55" s="44"/>
     </row>
     <row r="56" ht="45" customHeight="1" spans="1:10">
       <c r="A56" s="5">
@@ -3716,7 +3707,7 @@
       <c r="G56" s="5" t="s">
         <v>63</v>
       </c>
-      <c r="H56" s="44" t="s">
+      <c r="H56" s="43" t="s">
         <v>84</v>
       </c>
       <c r="I56" s="5" t="s">
@@ -3748,7 +3739,7 @@
       <c r="G57" s="5" t="s">
         <v>63</v>
       </c>
-      <c r="H57" s="44" t="s">
+      <c r="H57" s="43" t="s">
         <v>84</v>
       </c>
       <c r="I57" s="5" t="s">
@@ -3780,7 +3771,7 @@
       <c r="G58" s="5" t="s">
         <v>63</v>
       </c>
-      <c r="H58" s="44" t="s">
+      <c r="H58" s="43" t="s">
         <v>84</v>
       </c>
       <c r="I58" s="5" t="s">
@@ -3812,7 +3803,7 @@
       <c r="G59" s="5" t="s">
         <v>63</v>
       </c>
-      <c r="H59" s="44" t="s">
+      <c r="H59" s="43" t="s">
         <v>84</v>
       </c>
       <c r="I59" s="5" t="s">
@@ -3844,7 +3835,7 @@
       <c r="G60" s="5" t="s">
         <v>63</v>
       </c>
-      <c r="H60" s="44" t="s">
+      <c r="H60" s="43" t="s">
         <v>84</v>
       </c>
       <c r="I60" s="5" t="s">
@@ -3876,7 +3867,7 @@
       <c r="G61" s="5" t="s">
         <v>63</v>
       </c>
-      <c r="H61" s="44" t="s">
+      <c r="H61" s="43" t="s">
         <v>84</v>
       </c>
       <c r="I61" s="5" t="s">
@@ -3901,7 +3892,7 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
   <dimension ref="A1:I18"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="15"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.4"/>
   <cols>
     <col min="1" max="1" width="5" customWidth="1"/>
     <col min="2" max="2" width="25" customWidth="1"/>
@@ -3968,152 +3959,152 @@
       </c>
     </row>
     <row r="4" ht="28" customHeight="1" spans="1:1">
-      <c r="A4" s="31" t="s">
+      <c r="A4" s="30" t="s">
         <v>12</v>
       </c>
     </row>
     <row r="5" ht="45" customHeight="1" spans="1:9">
-      <c r="A5" s="32">
+      <c r="A5" s="31">
         <v>1</v>
       </c>
-      <c r="B5" s="32" t="s">
+      <c r="B5" s="31" t="s">
         <v>13</v>
       </c>
-      <c r="C5" s="32" t="s">
+      <c r="C5" s="31" t="s">
         <v>14</v>
       </c>
-      <c r="D5" s="32" t="s">
+      <c r="D5" s="31" t="s">
         <v>16</v>
       </c>
-      <c r="E5" s="32" t="s">
+      <c r="E5" s="31" t="s">
         <v>17</v>
       </c>
-      <c r="F5" s="33" t="s">
+      <c r="F5" s="32" t="s">
         <v>18</v>
       </c>
-      <c r="G5" s="34" t="s">
-        <v>20</v>
-      </c>
-      <c r="H5" s="34" t="s">
-        <v>20</v>
-      </c>
-      <c r="I5" s="36" t="s">
+      <c r="G5" s="33" t="s">
+        <v>20</v>
+      </c>
+      <c r="H5" s="33" t="s">
+        <v>20</v>
+      </c>
+      <c r="I5" s="35" t="s">
         <v>187</v>
       </c>
     </row>
     <row r="6" ht="45" customHeight="1" spans="1:9">
-      <c r="A6" s="32">
+      <c r="A6" s="31">
         <v>2</v>
       </c>
-      <c r="B6" s="32" t="s">
+      <c r="B6" s="31" t="s">
         <v>21</v>
       </c>
-      <c r="C6" s="32" t="s">
+      <c r="C6" s="31" t="s">
         <v>22</v>
       </c>
-      <c r="D6" s="32" t="s">
+      <c r="D6" s="31" t="s">
         <v>24</v>
       </c>
-      <c r="E6" s="32" t="s">
+      <c r="E6" s="31" t="s">
         <v>17</v>
       </c>
-      <c r="F6" s="33" t="s">
+      <c r="F6" s="32" t="s">
         <v>18</v>
       </c>
-      <c r="G6" s="34" t="s">
-        <v>20</v>
-      </c>
-      <c r="H6" s="34" t="s">
-        <v>20</v>
-      </c>
-      <c r="I6" s="36" t="s">
+      <c r="G6" s="33" t="s">
+        <v>20</v>
+      </c>
+      <c r="H6" s="33" t="s">
+        <v>20</v>
+      </c>
+      <c r="I6" s="35" t="s">
         <v>188</v>
       </c>
     </row>
     <row r="7" ht="45" customHeight="1" spans="1:9">
-      <c r="A7" s="32">
+      <c r="A7" s="31">
         <v>3</v>
       </c>
-      <c r="B7" s="32" t="s">
+      <c r="B7" s="31" t="s">
         <v>25</v>
       </c>
-      <c r="C7" s="32" t="s">
+      <c r="C7" s="31" t="s">
         <v>26</v>
       </c>
-      <c r="D7" s="32" t="s">
+      <c r="D7" s="31" t="s">
         <v>27</v>
       </c>
-      <c r="E7" s="32" t="s">
+      <c r="E7" s="31" t="s">
         <v>17</v>
       </c>
-      <c r="F7" s="33" t="s">
+      <c r="F7" s="32" t="s">
         <v>18</v>
       </c>
-      <c r="G7" s="34" t="s">
-        <v>20</v>
-      </c>
-      <c r="H7" s="34" t="s">
-        <v>20</v>
-      </c>
-      <c r="I7" s="36" t="s">
+      <c r="G7" s="33" t="s">
+        <v>20</v>
+      </c>
+      <c r="H7" s="33" t="s">
+        <v>20</v>
+      </c>
+      <c r="I7" s="35" t="s">
         <v>189</v>
       </c>
     </row>
     <row r="8" ht="45" customHeight="1" spans="1:9">
-      <c r="A8" s="32">
+      <c r="A8" s="31">
         <v>4</v>
       </c>
-      <c r="B8" s="32" t="s">
+      <c r="B8" s="31" t="s">
         <v>28</v>
       </c>
-      <c r="C8" s="32" t="s">
+      <c r="C8" s="31" t="s">
         <v>29</v>
       </c>
-      <c r="D8" s="32" t="s">
+      <c r="D8" s="31" t="s">
         <v>30</v>
       </c>
-      <c r="E8" s="32" t="s">
+      <c r="E8" s="31" t="s">
         <v>17</v>
       </c>
-      <c r="F8" s="33" t="s">
+      <c r="F8" s="32" t="s">
         <v>18</v>
       </c>
-      <c r="G8" s="34" t="s">
-        <v>20</v>
-      </c>
-      <c r="H8" s="34" t="s">
-        <v>20</v>
-      </c>
-      <c r="I8" s="36" t="s">
+      <c r="G8" s="33" t="s">
+        <v>20</v>
+      </c>
+      <c r="H8" s="33" t="s">
+        <v>20</v>
+      </c>
+      <c r="I8" s="35" t="s">
         <v>190</v>
       </c>
     </row>
     <row r="9" ht="45" customHeight="1" spans="1:9">
-      <c r="A9" s="32">
+      <c r="A9" s="31">
         <v>5</v>
       </c>
-      <c r="B9" s="32" t="s">
+      <c r="B9" s="31" t="s">
         <v>31</v>
       </c>
-      <c r="C9" s="32" t="s">
+      <c r="C9" s="31" t="s">
         <v>191</v>
       </c>
-      <c r="D9" s="32" t="s">
+      <c r="D9" s="31" t="s">
         <v>192</v>
       </c>
-      <c r="E9" s="32" t="s">
+      <c r="E9" s="31" t="s">
         <v>17</v>
       </c>
-      <c r="F9" s="33" t="s">
+      <c r="F9" s="32" t="s">
         <v>18</v>
       </c>
-      <c r="G9" s="34" t="s">
-        <v>20</v>
-      </c>
-      <c r="H9" s="34" t="s">
-        <v>20</v>
-      </c>
-      <c r="I9" s="36" t="s">
+      <c r="G9" s="33" t="s">
+        <v>20</v>
+      </c>
+      <c r="H9" s="33" t="s">
+        <v>20</v>
+      </c>
+      <c r="I9" s="35" t="s">
         <v>193</v>
       </c>
     </row>
@@ -4121,14 +4112,14 @@
       <c r="A10" s="23" t="s">
         <v>34</v>
       </c>
-      <c r="B10" s="28"/>
-      <c r="C10" s="28"/>
-      <c r="D10" s="28"/>
-      <c r="E10" s="28"/>
-      <c r="F10" s="35"/>
-      <c r="G10" s="28"/>
-      <c r="H10" s="28"/>
-      <c r="I10" s="37"/>
+      <c r="B10" s="27"/>
+      <c r="C10" s="27"/>
+      <c r="D10" s="27"/>
+      <c r="E10" s="27"/>
+      <c r="F10" s="34"/>
+      <c r="G10" s="27"/>
+      <c r="H10" s="27"/>
+      <c r="I10" s="36"/>
     </row>
     <row r="11" ht="45" customHeight="1" spans="1:9">
       <c r="A11" s="5">
@@ -4146,7 +4137,7 @@
       <c r="E11" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="F11" s="33" t="s">
+      <c r="F11" s="32" t="s">
         <v>194</v>
       </c>
       <c r="G11" s="5" t="s">
@@ -4155,7 +4146,7 @@
       <c r="H11" s="5" t="s">
         <v>20</v>
       </c>
-      <c r="I11" s="38" t="s">
+      <c r="I11" s="37" t="s">
         <v>195</v>
       </c>
     </row>
@@ -4169,13 +4160,13 @@
       <c r="C12" s="6" t="s">
         <v>39</v>
       </c>
-      <c r="D12" s="32" t="s">
+      <c r="D12" s="31" t="s">
         <v>40</v>
       </c>
       <c r="E12" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="F12" s="33" t="s">
+      <c r="F12" s="32" t="s">
         <v>18</v>
       </c>
       <c r="G12" s="5" t="s">
@@ -4184,11 +4175,11 @@
       <c r="H12" s="5" t="s">
         <v>20</v>
       </c>
-      <c r="I12" s="38" t="s">
+      <c r="I12" s="37" t="s">
         <v>196</v>
       </c>
     </row>
-    <row r="13" ht="25.5" spans="1:9">
+    <row r="13" ht="26.4" spans="1:9">
       <c r="A13" s="5">
         <v>8</v>
       </c>
@@ -4204,7 +4195,7 @@
       <c r="E13" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="F13" s="33" t="s">
+      <c r="F13" s="32" t="s">
         <v>18</v>
       </c>
       <c r="G13" s="5" t="s">
@@ -4213,11 +4204,11 @@
       <c r="H13" s="5" t="s">
         <v>20</v>
       </c>
-      <c r="I13" s="38" t="s">
+      <c r="I13" s="37" t="s">
         <v>197</v>
       </c>
     </row>
-    <row r="14" ht="25.5" spans="1:9">
+    <row r="14" ht="26.4" spans="1:9">
       <c r="A14" s="5">
         <v>9</v>
       </c>
@@ -4233,7 +4224,7 @@
       <c r="E14" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="F14" s="33" t="s">
+      <c r="F14" s="32" t="s">
         <v>18</v>
       </c>
       <c r="G14" s="5" t="s">
@@ -4242,11 +4233,11 @@
       <c r="H14" s="5" t="s">
         <v>20</v>
       </c>
-      <c r="I14" s="38" t="s">
+      <c r="I14" s="37" t="s">
         <v>198</v>
       </c>
     </row>
-    <row r="15" ht="25.5" spans="1:9">
+    <row r="15" ht="26.4" spans="1:9">
       <c r="A15" s="5">
         <v>10</v>
       </c>
@@ -4262,7 +4253,7 @@
       <c r="E15" s="5" t="s">
         <v>50</v>
       </c>
-      <c r="F15" s="33" t="s">
+      <c r="F15" s="32" t="s">
         <v>199</v>
       </c>
       <c r="G15" s="5" t="s">
@@ -4271,11 +4262,11 @@
       <c r="H15" s="5" t="s">
         <v>20</v>
       </c>
-      <c r="I15" s="38" t="s">
+      <c r="I15" s="37" t="s">
         <v>200</v>
       </c>
     </row>
-    <row r="16" ht="25.5" spans="1:9">
+    <row r="16" ht="26.4" spans="1:9">
       <c r="A16" s="5">
         <v>11</v>
       </c>
@@ -4291,7 +4282,7 @@
       <c r="E16" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="F16" s="33" t="s">
+      <c r="F16" s="32" t="s">
         <v>18</v>
       </c>
       <c r="G16" s="5" t="s">
@@ -4300,11 +4291,11 @@
       <c r="H16" s="5" t="s">
         <v>20</v>
       </c>
-      <c r="I16" s="38" t="s">
+      <c r="I16" s="37" t="s">
         <v>201</v>
       </c>
     </row>
-    <row r="17" ht="25.5" spans="1:9">
+    <row r="17" ht="26.4" spans="1:9">
       <c r="A17" s="5">
         <v>12</v>
       </c>
@@ -4320,7 +4311,7 @@
       <c r="E17" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="F17" s="33" t="s">
+      <c r="F17" s="32" t="s">
         <v>194</v>
       </c>
       <c r="G17" s="5" t="s">
@@ -4329,11 +4320,11 @@
       <c r="H17" s="5" t="s">
         <v>20</v>
       </c>
-      <c r="I17" s="38" t="s">
+      <c r="I17" s="37" t="s">
         <v>202</v>
       </c>
     </row>
-    <row r="18" ht="25.5" spans="1:9">
+    <row r="18" ht="26.4" spans="1:9">
       <c r="A18" s="5">
         <v>13</v>
       </c>
@@ -4349,7 +4340,7 @@
       <c r="E18" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="F18" s="33" t="s">
+      <c r="F18" s="32" t="s">
         <v>18</v>
       </c>
       <c r="G18" s="5" t="s">
@@ -4358,7 +4349,7 @@
       <c r="H18" s="5" t="s">
         <v>20</v>
       </c>
-      <c r="I18" s="38" t="s">
+      <c r="I18" s="37" t="s">
         <v>203</v>
       </c>
     </row>
@@ -4377,7 +4368,7 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
   <dimension ref="A1:I37"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="15"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.4"/>
   <cols>
     <col min="1" max="1" width="5" customWidth="1"/>
     <col min="2" max="2" width="25" customWidth="1"/>
@@ -4834,7 +4825,7 @@
         <v>93</v>
       </c>
       <c r="F18" s="26" t="s">
-        <v>194</v>
+        <v>18</v>
       </c>
       <c r="G18" s="5" t="s">
         <v>20</v>
@@ -4862,7 +4853,7 @@
       <c r="E19" s="5" t="s">
         <v>93</v>
       </c>
-      <c r="F19" s="27" t="s">
+      <c r="F19" s="24" t="s">
         <v>18</v>
       </c>
       <c r="G19" s="5" t="s">
@@ -5153,26 +5144,26 @@
       <c r="A30" s="23" t="s">
         <v>136</v>
       </c>
-      <c r="B30" s="28"/>
-      <c r="C30" s="28"/>
-      <c r="D30" s="28"/>
-      <c r="E30" s="28"/>
-      <c r="F30" s="28"/>
-      <c r="G30" s="28"/>
-      <c r="H30" s="28"/>
-      <c r="I30" s="30"/>
+      <c r="B30" s="27"/>
+      <c r="C30" s="27"/>
+      <c r="D30" s="27"/>
+      <c r="E30" s="27"/>
+      <c r="F30" s="27"/>
+      <c r="G30" s="27"/>
+      <c r="H30" s="27"/>
+      <c r="I30" s="29"/>
     </row>
     <row r="31" ht="28" customHeight="1" spans="1:9">
-      <c r="A31" s="29">
+      <c r="A31" s="28">
         <v>24</v>
       </c>
-      <c r="B31" s="29" t="s">
+      <c r="B31" s="28" t="s">
         <v>137</v>
       </c>
-      <c r="C31" s="29" t="s">
+      <c r="C31" s="28" t="s">
         <v>138</v>
       </c>
-      <c r="D31" s="29" t="s">
+      <c r="D31" s="28" t="s">
         <v>140</v>
       </c>
       <c r="E31" s="5" t="s">
@@ -5354,7 +5345,7 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
   <dimension ref="A1:I17"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="15"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.4"/>
   <cols>
     <col min="1" max="1" width="5" customWidth="1"/>
     <col min="2" max="2" width="25" customWidth="1"/>
@@ -5767,7 +5758,7 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
   <dimension ref="A1:F30"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="15" outlineLevelCol="5"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.4" outlineLevelCol="5"/>
   <cols>
     <col min="1" max="1" width="14" customWidth="1"/>
     <col min="2" max="2" width="42" customWidth="1"/>

</xml_diff>

<commit_message>
Cập nhật tiến trình trong file Tracking
</commit_message>
<xml_diff>
--- a/Project_Tracking.xlsx
+++ b/Project_Tracking.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="20760" windowHeight="12300"/>
+    <workbookView windowWidth="28800" windowHeight="12885" activeTab="2"/>
   </bookViews>
   <sheets>
     <sheet name="Project Tracking" sheetId="1" r:id="rId1"/>
@@ -1510,7 +1510,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="45">
+  <cellXfs count="46">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -1577,6 +1577,9 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="9" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="8" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -2088,13 +2091,13 @@
     <col min="4" max="4" width="22" customWidth="1"/>
     <col min="5" max="5" width="60" customWidth="1"/>
     <col min="6" max="7" width="14" customWidth="1"/>
-    <col min="8" max="8" width="10" style="38" customWidth="1"/>
+    <col min="8" max="8" width="10" style="39" customWidth="1"/>
     <col min="9" max="9" width="14" customWidth="1"/>
     <col min="10" max="10" width="30" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" ht="40" customHeight="1" spans="1:10">
-      <c r="A1" s="39" t="s">
+      <c r="A1" s="40" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="8"/>
@@ -2103,7 +2106,7 @@
       <c r="E1" s="8"/>
       <c r="F1" s="8"/>
       <c r="G1" s="8"/>
-      <c r="H1" s="40"/>
+      <c r="H1" s="41"/>
       <c r="I1" s="8"/>
       <c r="J1" s="9"/>
     </row>
@@ -2117,7 +2120,7 @@
       <c r="E2" s="8"/>
       <c r="F2" s="8"/>
       <c r="G2" s="8"/>
-      <c r="H2" s="40"/>
+      <c r="H2" s="41"/>
       <c r="I2" s="8"/>
       <c r="J2" s="9"/>
     </row>
@@ -2153,26 +2156,26 @@
         <v>11</v>
       </c>
     </row>
-    <row r="4" s="37" customFormat="1" ht="28" customHeight="1" spans="1:8">
-      <c r="A4" s="29" t="s">
+    <row r="4" s="38" customFormat="1" ht="28" customHeight="1" spans="1:8">
+      <c r="A4" s="30" t="s">
         <v>12</v>
       </c>
-      <c r="H4" s="41"/>
+      <c r="H4" s="42"/>
     </row>
     <row r="5" ht="45" customHeight="1" spans="1:10">
-      <c r="A5" s="27">
+      <c r="A5" s="28">
         <v>1</v>
       </c>
-      <c r="B5" s="27" t="s">
+      <c r="B5" s="28" t="s">
         <v>13</v>
       </c>
-      <c r="C5" s="27" t="s">
+      <c r="C5" s="28" t="s">
         <v>14</v>
       </c>
-      <c r="D5" s="27" t="s">
+      <c r="D5" s="28" t="s">
         <v>15</v>
       </c>
-      <c r="E5" s="27" t="s">
+      <c r="E5" s="28" t="s">
         <v>16</v>
       </c>
       <c r="F5" s="5" t="s">
@@ -2181,28 +2184,28 @@
       <c r="G5" s="5" t="s">
         <v>18</v>
       </c>
-      <c r="H5" s="42" t="s">
+      <c r="H5" s="43" t="s">
         <v>19</v>
       </c>
-      <c r="I5" s="30"/>
+      <c r="I5" s="31"/>
       <c r="J5" s="5" t="s">
         <v>20</v>
       </c>
     </row>
     <row r="6" ht="45" customHeight="1" spans="1:10">
-      <c r="A6" s="27">
+      <c r="A6" s="28">
         <v>2</v>
       </c>
-      <c r="B6" s="27" t="s">
+      <c r="B6" s="28" t="s">
         <v>21</v>
       </c>
-      <c r="C6" s="27" t="s">
+      <c r="C6" s="28" t="s">
         <v>22</v>
       </c>
-      <c r="D6" s="27" t="s">
+      <c r="D6" s="28" t="s">
         <v>23</v>
       </c>
-      <c r="E6" s="27" t="s">
+      <c r="E6" s="28" t="s">
         <v>24</v>
       </c>
       <c r="F6" s="5" t="s">
@@ -2211,28 +2214,28 @@
       <c r="G6" s="5" t="s">
         <v>18</v>
       </c>
-      <c r="H6" s="42" t="s">
+      <c r="H6" s="43" t="s">
         <v>19</v>
       </c>
-      <c r="I6" s="30"/>
+      <c r="I6" s="31"/>
       <c r="J6" s="5" t="s">
         <v>20</v>
       </c>
     </row>
     <row r="7" ht="45" customHeight="1" spans="1:10">
-      <c r="A7" s="27">
+      <c r="A7" s="28">
         <v>3</v>
       </c>
-      <c r="B7" s="27" t="s">
+      <c r="B7" s="28" t="s">
         <v>25</v>
       </c>
-      <c r="C7" s="27" t="s">
+      <c r="C7" s="28" t="s">
         <v>26</v>
       </c>
-      <c r="D7" s="27" t="s">
+      <c r="D7" s="28" t="s">
         <v>15</v>
       </c>
-      <c r="E7" s="27" t="s">
+      <c r="E7" s="28" t="s">
         <v>27</v>
       </c>
       <c r="F7" s="5" t="s">
@@ -2241,28 +2244,28 @@
       <c r="G7" s="5" t="s">
         <v>18</v>
       </c>
-      <c r="H7" s="42" t="s">
+      <c r="H7" s="43" t="s">
         <v>19</v>
       </c>
-      <c r="I7" s="30"/>
+      <c r="I7" s="31"/>
       <c r="J7" s="5" t="s">
         <v>20</v>
       </c>
     </row>
     <row r="8" ht="45" customHeight="1" spans="1:10">
-      <c r="A8" s="27">
+      <c r="A8" s="28">
         <v>4</v>
       </c>
-      <c r="B8" s="27" t="s">
+      <c r="B8" s="28" t="s">
         <v>28</v>
       </c>
-      <c r="C8" s="27" t="s">
+      <c r="C8" s="28" t="s">
         <v>29</v>
       </c>
-      <c r="D8" s="27" t="s">
+      <c r="D8" s="28" t="s">
         <v>15</v>
       </c>
-      <c r="E8" s="27" t="s">
+      <c r="E8" s="28" t="s">
         <v>30</v>
       </c>
       <c r="F8" s="5" t="s">
@@ -2271,28 +2274,28 @@
       <c r="G8" s="5" t="s">
         <v>18</v>
       </c>
-      <c r="H8" s="42" t="s">
+      <c r="H8" s="43" t="s">
         <v>19</v>
       </c>
-      <c r="I8" s="30"/>
+      <c r="I8" s="31"/>
       <c r="J8" s="5" t="s">
         <v>20</v>
       </c>
     </row>
     <row r="9" ht="45" customHeight="1" spans="1:10">
-      <c r="A9" s="27">
+      <c r="A9" s="28">
         <v>5</v>
       </c>
-      <c r="B9" s="27" t="s">
+      <c r="B9" s="28" t="s">
         <v>31</v>
       </c>
-      <c r="C9" s="27" t="s">
+      <c r="C9" s="28" t="s">
         <v>32</v>
       </c>
-      <c r="D9" s="27" t="s">
+      <c r="D9" s="28" t="s">
         <v>15</v>
       </c>
-      <c r="E9" s="27" t="s">
+      <c r="E9" s="28" t="s">
         <v>33</v>
       </c>
       <c r="F9" s="5" t="s">
@@ -2301,10 +2304,10 @@
       <c r="G9" s="5" t="s">
         <v>18</v>
       </c>
-      <c r="H9" s="42" t="s">
+      <c r="H9" s="43" t="s">
         <v>19</v>
       </c>
-      <c r="I9" s="30"/>
+      <c r="I9" s="31"/>
       <c r="J9" s="5" t="s">
         <v>20</v>
       </c>
@@ -2313,15 +2316,15 @@
       <c r="A10" s="23" t="s">
         <v>34</v>
       </c>
-      <c r="B10" s="26"/>
-      <c r="C10" s="26"/>
-      <c r="D10" s="26"/>
-      <c r="E10" s="26"/>
-      <c r="F10" s="26"/>
-      <c r="G10" s="26"/>
-      <c r="H10" s="26"/>
-      <c r="I10" s="26"/>
-      <c r="J10" s="44"/>
+      <c r="B10" s="27"/>
+      <c r="C10" s="27"/>
+      <c r="D10" s="27"/>
+      <c r="E10" s="27"/>
+      <c r="F10" s="27"/>
+      <c r="G10" s="27"/>
+      <c r="H10" s="27"/>
+      <c r="I10" s="27"/>
+      <c r="J10" s="45"/>
     </row>
     <row r="11" ht="45" customHeight="1" spans="1:10">
       <c r="A11" s="5">
@@ -2345,7 +2348,7 @@
       <c r="G11" s="5" t="s">
         <v>18</v>
       </c>
-      <c r="H11" s="42" t="s">
+      <c r="H11" s="43" t="s">
         <v>19</v>
       </c>
       <c r="I11" s="5" t="s">
@@ -2377,7 +2380,7 @@
       <c r="G12" s="5" t="s">
         <v>18</v>
       </c>
-      <c r="H12" s="42" t="s">
+      <c r="H12" s="43" t="s">
         <v>19</v>
       </c>
       <c r="I12" s="5" t="s">
@@ -2409,7 +2412,7 @@
       <c r="G13" s="5" t="s">
         <v>18</v>
       </c>
-      <c r="H13" s="42" t="s">
+      <c r="H13" s="43" t="s">
         <v>19</v>
       </c>
       <c r="I13" s="5" t="s">
@@ -2441,7 +2444,7 @@
       <c r="G14" s="5" t="s">
         <v>18</v>
       </c>
-      <c r="H14" s="42" t="s">
+      <c r="H14" s="43" t="s">
         <v>19</v>
       </c>
       <c r="I14" s="5" t="s">
@@ -2473,7 +2476,7 @@
       <c r="G15" s="5" t="s">
         <v>18</v>
       </c>
-      <c r="H15" s="42" t="s">
+      <c r="H15" s="43" t="s">
         <v>19</v>
       </c>
       <c r="I15" s="5" t="s">
@@ -2505,7 +2508,7 @@
       <c r="G16" s="5" t="s">
         <v>18</v>
       </c>
-      <c r="H16" s="42" t="s">
+      <c r="H16" s="43" t="s">
         <v>19</v>
       </c>
       <c r="I16" s="5" t="s">
@@ -2537,7 +2540,7 @@
       <c r="G17" s="5" t="s">
         <v>18</v>
       </c>
-      <c r="H17" s="42" t="s">
+      <c r="H17" s="43" t="s">
         <v>19</v>
       </c>
       <c r="I17" s="5" t="s">
@@ -2569,7 +2572,7 @@
       <c r="G18" s="5" t="s">
         <v>18</v>
       </c>
-      <c r="H18" s="42" t="s">
+      <c r="H18" s="43" t="s">
         <v>19</v>
       </c>
       <c r="I18" s="5" t="s">
@@ -2601,7 +2604,7 @@
       <c r="G19" s="5" t="s">
         <v>63</v>
       </c>
-      <c r="H19" s="42" t="s">
+      <c r="H19" s="43" t="s">
         <v>64</v>
       </c>
       <c r="I19" s="5" t="s">
@@ -2633,7 +2636,7 @@
       <c r="G20" s="5" t="s">
         <v>63</v>
       </c>
-      <c r="H20" s="42" t="s">
+      <c r="H20" s="43" t="s">
         <v>64</v>
       </c>
       <c r="I20" s="5" t="s">
@@ -2665,7 +2668,7 @@
       <c r="G21" s="5" t="s">
         <v>63</v>
       </c>
-      <c r="H21" s="42" t="s">
+      <c r="H21" s="43" t="s">
         <v>64</v>
       </c>
       <c r="I21" s="5" t="s">
@@ -2675,7 +2678,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="22" s="37" customFormat="1" ht="28" customHeight="1" spans="1:10">
+    <row r="22" s="38" customFormat="1" ht="28" customHeight="1" spans="1:10">
       <c r="A22" s="6">
         <v>17</v>
       </c>
@@ -2697,7 +2700,7 @@
       <c r="G22" s="5" t="s">
         <v>63</v>
       </c>
-      <c r="H22" s="42" t="s">
+      <c r="H22" s="43" t="s">
         <v>64</v>
       </c>
       <c r="I22" s="5" t="s">
@@ -2729,7 +2732,7 @@
       <c r="G23" s="5" t="s">
         <v>63</v>
       </c>
-      <c r="H23" s="42" t="s">
+      <c r="H23" s="43" t="s">
         <v>64</v>
       </c>
       <c r="I23" s="5" t="s">
@@ -2761,7 +2764,7 @@
       <c r="G24" s="5" t="s">
         <v>63</v>
       </c>
-      <c r="H24" s="42" t="s">
+      <c r="H24" s="43" t="s">
         <v>64</v>
       </c>
       <c r="I24" s="5" t="s">
@@ -2793,7 +2796,7 @@
       <c r="G25" s="5" t="s">
         <v>63</v>
       </c>
-      <c r="H25" s="42" t="s">
+      <c r="H25" s="43" t="s">
         <v>64</v>
       </c>
       <c r="I25" s="5" t="s">
@@ -2825,7 +2828,7 @@
       <c r="G26" s="5" t="s">
         <v>63</v>
       </c>
-      <c r="H26" s="42" t="s">
+      <c r="H26" s="43" t="s">
         <v>84</v>
       </c>
       <c r="I26" s="5" t="s">
@@ -2857,7 +2860,7 @@
       <c r="G27" s="5" t="s">
         <v>63</v>
       </c>
-      <c r="H27" s="42" t="s">
+      <c r="H27" s="43" t="s">
         <v>84</v>
       </c>
       <c r="I27" s="5" t="s">
@@ -2871,15 +2874,15 @@
       <c r="A28" s="23" t="s">
         <v>88</v>
       </c>
-      <c r="B28" s="26"/>
-      <c r="C28" s="26"/>
-      <c r="D28" s="26"/>
-      <c r="E28" s="26"/>
-      <c r="F28" s="26"/>
-      <c r="G28" s="26"/>
-      <c r="H28" s="26"/>
-      <c r="I28" s="26"/>
-      <c r="J28" s="44"/>
+      <c r="B28" s="27"/>
+      <c r="C28" s="27"/>
+      <c r="D28" s="27"/>
+      <c r="E28" s="27"/>
+      <c r="F28" s="27"/>
+      <c r="G28" s="27"/>
+      <c r="H28" s="27"/>
+      <c r="I28" s="27"/>
+      <c r="J28" s="45"/>
     </row>
     <row r="29" ht="45" customHeight="1" spans="1:10">
       <c r="A29" s="5">
@@ -2903,7 +2906,7 @@
       <c r="G29" s="24" t="s">
         <v>18</v>
       </c>
-      <c r="H29" s="42" t="s">
+      <c r="H29" s="43" t="s">
         <v>64</v>
       </c>
       <c r="I29" s="5" t="s">
@@ -2935,7 +2938,7 @@
       <c r="G30" s="24" t="s">
         <v>18</v>
       </c>
-      <c r="H30" s="42" t="s">
+      <c r="H30" s="43" t="s">
         <v>64</v>
       </c>
       <c r="I30" s="5" t="s">
@@ -2967,7 +2970,7 @@
       <c r="G31" s="24" t="s">
         <v>18</v>
       </c>
-      <c r="H31" s="42" t="s">
+      <c r="H31" s="43" t="s">
         <v>64</v>
       </c>
       <c r="I31" s="5" t="s">
@@ -2999,7 +3002,7 @@
       <c r="G32" s="24" t="s">
         <v>18</v>
       </c>
-      <c r="H32" s="42" t="s">
+      <c r="H32" s="43" t="s">
         <v>64</v>
       </c>
       <c r="I32" s="5" t="s">
@@ -3028,10 +3031,10 @@
       <c r="F33" s="5" t="s">
         <v>93</v>
       </c>
-      <c r="G33" s="43" t="s">
+      <c r="G33" s="44" t="s">
         <v>63</v>
       </c>
-      <c r="H33" s="42" t="s">
+      <c r="H33" s="43" t="s">
         <v>64</v>
       </c>
       <c r="I33" s="5" t="s">
@@ -3041,29 +3044,29 @@
         <v>20</v>
       </c>
     </row>
-    <row r="34" s="37" customFormat="1" ht="38" customHeight="1" spans="1:10">
+    <row r="34" s="38" customFormat="1" ht="38" customHeight="1" spans="1:10">
       <c r="A34" s="5">
         <v>28</v>
       </c>
       <c r="B34" s="5" t="s">
         <v>103</v>
       </c>
-      <c r="C34" s="27" t="s">
+      <c r="C34" s="28" t="s">
         <v>104</v>
       </c>
-      <c r="D34" s="27" t="s">
+      <c r="D34" s="28" t="s">
         <v>91</v>
       </c>
-      <c r="E34" s="27" t="s">
+      <c r="E34" s="28" t="s">
         <v>105</v>
       </c>
       <c r="F34" s="5" t="s">
         <v>93</v>
       </c>
-      <c r="G34" s="43" t="s">
-        <v>63</v>
-      </c>
-      <c r="H34" s="42" t="s">
+      <c r="G34" s="26" t="s">
+        <v>18</v>
+      </c>
+      <c r="H34" s="43" t="s">
         <v>64</v>
       </c>
       <c r="I34" s="5" t="s">
@@ -3095,7 +3098,7 @@
       <c r="G35" s="5" t="s">
         <v>18</v>
       </c>
-      <c r="H35" s="42" t="s">
+      <c r="H35" s="43" t="s">
         <v>64</v>
       </c>
       <c r="I35" s="5" t="s">
@@ -3127,7 +3130,7 @@
       <c r="G36" s="5" t="s">
         <v>18</v>
       </c>
-      <c r="H36" s="42" t="s">
+      <c r="H36" s="43" t="s">
         <v>64</v>
       </c>
       <c r="I36" s="5" t="s">
@@ -3159,7 +3162,7 @@
       <c r="G37" s="5" t="s">
         <v>18</v>
       </c>
-      <c r="H37" s="42" t="s">
+      <c r="H37" s="43" t="s">
         <v>64</v>
       </c>
       <c r="I37" s="5" t="s">
@@ -3191,7 +3194,7 @@
       <c r="G38" s="5" t="s">
         <v>18</v>
       </c>
-      <c r="H38" s="42" t="s">
+      <c r="H38" s="43" t="s">
         <v>64</v>
       </c>
       <c r="I38" s="5" t="s">
@@ -3223,7 +3226,7 @@
       <c r="G39" s="5" t="s">
         <v>18</v>
       </c>
-      <c r="H39" s="42" t="s">
+      <c r="H39" s="43" t="s">
         <v>64</v>
       </c>
       <c r="I39" s="5" t="s">
@@ -3237,17 +3240,17 @@
       <c r="A40" s="23" t="s">
         <v>118</v>
       </c>
-      <c r="B40" s="26"/>
-      <c r="C40" s="26"/>
-      <c r="D40" s="26"/>
-      <c r="E40" s="26"/>
-      <c r="F40" s="26"/>
-      <c r="G40" s="26"/>
-      <c r="H40" s="26"/>
-      <c r="I40" s="26"/>
-      <c r="J40" s="44"/>
-    </row>
-    <row r="41" s="37" customFormat="1" ht="46" customHeight="1" spans="1:10">
+      <c r="B40" s="27"/>
+      <c r="C40" s="27"/>
+      <c r="D40" s="27"/>
+      <c r="E40" s="27"/>
+      <c r="F40" s="27"/>
+      <c r="G40" s="27"/>
+      <c r="H40" s="27"/>
+      <c r="I40" s="27"/>
+      <c r="J40" s="45"/>
+    </row>
+    <row r="41" s="38" customFormat="1" ht="46" customHeight="1" spans="1:10">
       <c r="A41" s="6">
         <v>34</v>
       </c>
@@ -3269,7 +3272,7 @@
       <c r="G41" s="5" t="s">
         <v>63</v>
       </c>
-      <c r="H41" s="42" t="s">
+      <c r="H41" s="43" t="s">
         <v>64</v>
       </c>
       <c r="I41" s="5" t="s">
@@ -3301,7 +3304,7 @@
       <c r="G42" s="5" t="s">
         <v>63</v>
       </c>
-      <c r="H42" s="42" t="s">
+      <c r="H42" s="43" t="s">
         <v>64</v>
       </c>
       <c r="I42" s="5" t="s">
@@ -3333,7 +3336,7 @@
       <c r="G43" s="5" t="s">
         <v>63</v>
       </c>
-      <c r="H43" s="42" t="s">
+      <c r="H43" s="43" t="s">
         <v>64</v>
       </c>
       <c r="I43" s="5" t="s">
@@ -3365,7 +3368,7 @@
       <c r="G44" s="5" t="s">
         <v>63</v>
       </c>
-      <c r="H44" s="42" t="s">
+      <c r="H44" s="43" t="s">
         <v>64</v>
       </c>
       <c r="I44" s="5" t="s">
@@ -3397,7 +3400,7 @@
       <c r="G45" s="5" t="s">
         <v>63</v>
       </c>
-      <c r="H45" s="42" t="s">
+      <c r="H45" s="43" t="s">
         <v>64</v>
       </c>
       <c r="I45" s="5" t="s">
@@ -3411,15 +3414,15 @@
       <c r="A46" s="23" t="s">
         <v>136</v>
       </c>
-      <c r="B46" s="26"/>
-      <c r="C46" s="26"/>
-      <c r="D46" s="26"/>
-      <c r="E46" s="26"/>
-      <c r="F46" s="26"/>
-      <c r="G46" s="26"/>
-      <c r="H46" s="26"/>
-      <c r="I46" s="26"/>
-      <c r="J46" s="44"/>
+      <c r="B46" s="27"/>
+      <c r="C46" s="27"/>
+      <c r="D46" s="27"/>
+      <c r="E46" s="27"/>
+      <c r="F46" s="27"/>
+      <c r="G46" s="27"/>
+      <c r="H46" s="27"/>
+      <c r="I46" s="27"/>
+      <c r="J46" s="45"/>
     </row>
     <row r="47" ht="45" customHeight="1" spans="1:10">
       <c r="A47" s="5">
@@ -3443,7 +3446,7 @@
       <c r="G47" s="5" t="s">
         <v>63</v>
       </c>
-      <c r="H47" s="42" t="s">
+      <c r="H47" s="43" t="s">
         <v>64</v>
       </c>
       <c r="I47" s="5" t="s">
@@ -3475,7 +3478,7 @@
       <c r="G48" s="5" t="s">
         <v>63</v>
       </c>
-      <c r="H48" s="42" t="s">
+      <c r="H48" s="43" t="s">
         <v>64</v>
       </c>
       <c r="I48" s="5" t="s">
@@ -3507,7 +3510,7 @@
       <c r="G49" s="5" t="s">
         <v>63</v>
       </c>
-      <c r="H49" s="42" t="s">
+      <c r="H49" s="43" t="s">
         <v>64</v>
       </c>
       <c r="I49" s="5" t="s">
@@ -3517,20 +3520,20 @@
         <v>20</v>
       </c>
     </row>
-    <row r="50" s="37" customFormat="1" ht="28" customHeight="1" spans="1:10">
+    <row r="50" s="38" customFormat="1" ht="28" customHeight="1" spans="1:10">
       <c r="A50" s="5">
         <v>42</v>
       </c>
-      <c r="B50" s="27" t="s">
+      <c r="B50" s="28" t="s">
         <v>147</v>
       </c>
-      <c r="C50" s="27" t="s">
+      <c r="C50" s="28" t="s">
         <v>148</v>
       </c>
-      <c r="D50" s="27" t="s">
+      <c r="D50" s="28" t="s">
         <v>139</v>
       </c>
-      <c r="E50" s="27" t="s">
+      <c r="E50" s="28" t="s">
         <v>149</v>
       </c>
       <c r="F50" s="5" t="s">
@@ -3539,7 +3542,7 @@
       <c r="G50" s="5" t="s">
         <v>63</v>
       </c>
-      <c r="H50" s="42" t="s">
+      <c r="H50" s="43" t="s">
         <v>64</v>
       </c>
       <c r="I50" s="5" t="s">
@@ -3571,7 +3574,7 @@
       <c r="G51" s="5" t="s">
         <v>63</v>
       </c>
-      <c r="H51" s="42" t="s">
+      <c r="H51" s="43" t="s">
         <v>64</v>
       </c>
       <c r="I51" s="5" t="s">
@@ -3603,7 +3606,7 @@
       <c r="G52" s="5" t="s">
         <v>63</v>
       </c>
-      <c r="H52" s="42" t="s">
+      <c r="H52" s="43" t="s">
         <v>84</v>
       </c>
       <c r="I52" s="5" t="s">
@@ -3635,7 +3638,7 @@
       <c r="G53" s="5" t="s">
         <v>63</v>
       </c>
-      <c r="H53" s="42" t="s">
+      <c r="H53" s="43" t="s">
         <v>64</v>
       </c>
       <c r="I53" s="5" t="s">
@@ -3667,7 +3670,7 @@
       <c r="G54" s="5" t="s">
         <v>63</v>
       </c>
-      <c r="H54" s="42" t="s">
+      <c r="H54" s="43" t="s">
         <v>84</v>
       </c>
       <c r="I54" s="5" t="s">
@@ -3681,15 +3684,15 @@
       <c r="A55" s="23" t="s">
         <v>161</v>
       </c>
-      <c r="B55" s="26"/>
-      <c r="C55" s="26"/>
-      <c r="D55" s="26"/>
-      <c r="E55" s="26"/>
-      <c r="F55" s="26"/>
-      <c r="G55" s="26"/>
-      <c r="H55" s="26"/>
-      <c r="I55" s="26"/>
-      <c r="J55" s="44"/>
+      <c r="B55" s="27"/>
+      <c r="C55" s="27"/>
+      <c r="D55" s="27"/>
+      <c r="E55" s="27"/>
+      <c r="F55" s="27"/>
+      <c r="G55" s="27"/>
+      <c r="H55" s="27"/>
+      <c r="I55" s="27"/>
+      <c r="J55" s="45"/>
     </row>
     <row r="56" ht="45" customHeight="1" spans="1:10">
       <c r="A56" s="5">
@@ -3713,7 +3716,7 @@
       <c r="G56" s="5" t="s">
         <v>63</v>
       </c>
-      <c r="H56" s="42" t="s">
+      <c r="H56" s="43" t="s">
         <v>84</v>
       </c>
       <c r="I56" s="5" t="s">
@@ -3745,7 +3748,7 @@
       <c r="G57" s="5" t="s">
         <v>63</v>
       </c>
-      <c r="H57" s="42" t="s">
+      <c r="H57" s="43" t="s">
         <v>84</v>
       </c>
       <c r="I57" s="5" t="s">
@@ -3777,7 +3780,7 @@
       <c r="G58" s="5" t="s">
         <v>63</v>
       </c>
-      <c r="H58" s="42" t="s">
+      <c r="H58" s="43" t="s">
         <v>84</v>
       </c>
       <c r="I58" s="5" t="s">
@@ -3809,7 +3812,7 @@
       <c r="G59" s="5" t="s">
         <v>63</v>
       </c>
-      <c r="H59" s="42" t="s">
+      <c r="H59" s="43" t="s">
         <v>84</v>
       </c>
       <c r="I59" s="5" t="s">
@@ -3841,7 +3844,7 @@
       <c r="G60" s="5" t="s">
         <v>63</v>
       </c>
-      <c r="H60" s="42" t="s">
+      <c r="H60" s="43" t="s">
         <v>84</v>
       </c>
       <c r="I60" s="5" t="s">
@@ -3873,7 +3876,7 @@
       <c r="G61" s="5" t="s">
         <v>63</v>
       </c>
-      <c r="H61" s="42" t="s">
+      <c r="H61" s="43" t="s">
         <v>84</v>
       </c>
       <c r="I61" s="5" t="s">
@@ -3965,152 +3968,152 @@
       </c>
     </row>
     <row r="4" ht="28" customHeight="1" spans="1:1">
-      <c r="A4" s="29" t="s">
+      <c r="A4" s="30" t="s">
         <v>12</v>
       </c>
     </row>
     <row r="5" ht="45" customHeight="1" spans="1:9">
-      <c r="A5" s="30">
+      <c r="A5" s="31">
         <v>1</v>
       </c>
-      <c r="B5" s="30" t="s">
+      <c r="B5" s="31" t="s">
         <v>13</v>
       </c>
-      <c r="C5" s="30" t="s">
+      <c r="C5" s="31" t="s">
         <v>14</v>
       </c>
-      <c r="D5" s="30" t="s">
+      <c r="D5" s="31" t="s">
         <v>16</v>
       </c>
-      <c r="E5" s="30" t="s">
+      <c r="E5" s="31" t="s">
         <v>17</v>
       </c>
-      <c r="F5" s="31" t="s">
+      <c r="F5" s="32" t="s">
         <v>18</v>
       </c>
-      <c r="G5" s="32" t="s">
-        <v>20</v>
-      </c>
-      <c r="H5" s="32" t="s">
-        <v>20</v>
-      </c>
-      <c r="I5" s="34" t="s">
+      <c r="G5" s="33" t="s">
+        <v>20</v>
+      </c>
+      <c r="H5" s="33" t="s">
+        <v>20</v>
+      </c>
+      <c r="I5" s="35" t="s">
         <v>187</v>
       </c>
     </row>
     <row r="6" ht="45" customHeight="1" spans="1:9">
-      <c r="A6" s="30">
+      <c r="A6" s="31">
         <v>2</v>
       </c>
-      <c r="B6" s="30" t="s">
+      <c r="B6" s="31" t="s">
         <v>21</v>
       </c>
-      <c r="C6" s="30" t="s">
+      <c r="C6" s="31" t="s">
         <v>22</v>
       </c>
-      <c r="D6" s="30" t="s">
+      <c r="D6" s="31" t="s">
         <v>24</v>
       </c>
-      <c r="E6" s="30" t="s">
+      <c r="E6" s="31" t="s">
         <v>17</v>
       </c>
-      <c r="F6" s="31" t="s">
+      <c r="F6" s="32" t="s">
         <v>18</v>
       </c>
-      <c r="G6" s="32" t="s">
-        <v>20</v>
-      </c>
-      <c r="H6" s="32" t="s">
-        <v>20</v>
-      </c>
-      <c r="I6" s="34" t="s">
+      <c r="G6" s="33" t="s">
+        <v>20</v>
+      </c>
+      <c r="H6" s="33" t="s">
+        <v>20</v>
+      </c>
+      <c r="I6" s="35" t="s">
         <v>188</v>
       </c>
     </row>
     <row r="7" ht="45" customHeight="1" spans="1:9">
-      <c r="A7" s="30">
+      <c r="A7" s="31">
         <v>3</v>
       </c>
-      <c r="B7" s="30" t="s">
+      <c r="B7" s="31" t="s">
         <v>25</v>
       </c>
-      <c r="C7" s="30" t="s">
+      <c r="C7" s="31" t="s">
         <v>26</v>
       </c>
-      <c r="D7" s="30" t="s">
+      <c r="D7" s="31" t="s">
         <v>27</v>
       </c>
-      <c r="E7" s="30" t="s">
+      <c r="E7" s="31" t="s">
         <v>17</v>
       </c>
-      <c r="F7" s="31" t="s">
+      <c r="F7" s="32" t="s">
         <v>18</v>
       </c>
-      <c r="G7" s="32" t="s">
-        <v>20</v>
-      </c>
-      <c r="H7" s="32" t="s">
-        <v>20</v>
-      </c>
-      <c r="I7" s="34" t="s">
+      <c r="G7" s="33" t="s">
+        <v>20</v>
+      </c>
+      <c r="H7" s="33" t="s">
+        <v>20</v>
+      </c>
+      <c r="I7" s="35" t="s">
         <v>189</v>
       </c>
     </row>
     <row r="8" ht="45" customHeight="1" spans="1:9">
-      <c r="A8" s="30">
+      <c r="A8" s="31">
         <v>4</v>
       </c>
-      <c r="B8" s="30" t="s">
+      <c r="B8" s="31" t="s">
         <v>28</v>
       </c>
-      <c r="C8" s="30" t="s">
+      <c r="C8" s="31" t="s">
         <v>29</v>
       </c>
-      <c r="D8" s="30" t="s">
+      <c r="D8" s="31" t="s">
         <v>30</v>
       </c>
-      <c r="E8" s="30" t="s">
+      <c r="E8" s="31" t="s">
         <v>17</v>
       </c>
-      <c r="F8" s="31" t="s">
+      <c r="F8" s="32" t="s">
         <v>18</v>
       </c>
-      <c r="G8" s="32" t="s">
-        <v>20</v>
-      </c>
-      <c r="H8" s="32" t="s">
-        <v>20</v>
-      </c>
-      <c r="I8" s="34" t="s">
+      <c r="G8" s="33" t="s">
+        <v>20</v>
+      </c>
+      <c r="H8" s="33" t="s">
+        <v>20</v>
+      </c>
+      <c r="I8" s="35" t="s">
         <v>190</v>
       </c>
     </row>
     <row r="9" ht="45" customHeight="1" spans="1:9">
-      <c r="A9" s="30">
+      <c r="A9" s="31">
         <v>5</v>
       </c>
-      <c r="B9" s="30" t="s">
+      <c r="B9" s="31" t="s">
         <v>31</v>
       </c>
-      <c r="C9" s="30" t="s">
+      <c r="C9" s="31" t="s">
         <v>191</v>
       </c>
-      <c r="D9" s="30" t="s">
+      <c r="D9" s="31" t="s">
         <v>192</v>
       </c>
-      <c r="E9" s="30" t="s">
+      <c r="E9" s="31" t="s">
         <v>17</v>
       </c>
-      <c r="F9" s="31" t="s">
+      <c r="F9" s="32" t="s">
         <v>18</v>
       </c>
-      <c r="G9" s="32" t="s">
-        <v>20</v>
-      </c>
-      <c r="H9" s="32" t="s">
-        <v>20</v>
-      </c>
-      <c r="I9" s="34" t="s">
+      <c r="G9" s="33" t="s">
+        <v>20</v>
+      </c>
+      <c r="H9" s="33" t="s">
+        <v>20</v>
+      </c>
+      <c r="I9" s="35" t="s">
         <v>193</v>
       </c>
     </row>
@@ -4118,14 +4121,14 @@
       <c r="A10" s="23" t="s">
         <v>34</v>
       </c>
-      <c r="B10" s="26"/>
-      <c r="C10" s="26"/>
-      <c r="D10" s="26"/>
-      <c r="E10" s="26"/>
-      <c r="F10" s="33"/>
-      <c r="G10" s="26"/>
-      <c r="H10" s="26"/>
-      <c r="I10" s="35"/>
+      <c r="B10" s="27"/>
+      <c r="C10" s="27"/>
+      <c r="D10" s="27"/>
+      <c r="E10" s="27"/>
+      <c r="F10" s="34"/>
+      <c r="G10" s="27"/>
+      <c r="H10" s="27"/>
+      <c r="I10" s="36"/>
     </row>
     <row r="11" ht="45" customHeight="1" spans="1:9">
       <c r="A11" s="5">
@@ -4143,7 +4146,7 @@
       <c r="E11" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="F11" s="31" t="s">
+      <c r="F11" s="32" t="s">
         <v>194</v>
       </c>
       <c r="G11" s="5" t="s">
@@ -4152,7 +4155,7 @@
       <c r="H11" s="5" t="s">
         <v>20</v>
       </c>
-      <c r="I11" s="36" t="s">
+      <c r="I11" s="37" t="s">
         <v>195</v>
       </c>
     </row>
@@ -4166,13 +4169,13 @@
       <c r="C12" s="6" t="s">
         <v>39</v>
       </c>
-      <c r="D12" s="30" t="s">
+      <c r="D12" s="31" t="s">
         <v>40</v>
       </c>
       <c r="E12" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="F12" s="31" t="s">
+      <c r="F12" s="32" t="s">
         <v>18</v>
       </c>
       <c r="G12" s="5" t="s">
@@ -4181,7 +4184,7 @@
       <c r="H12" s="5" t="s">
         <v>20</v>
       </c>
-      <c r="I12" s="36" t="s">
+      <c r="I12" s="37" t="s">
         <v>196</v>
       </c>
     </row>
@@ -4201,7 +4204,7 @@
       <c r="E13" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="F13" s="31" t="s">
+      <c r="F13" s="32" t="s">
         <v>18</v>
       </c>
       <c r="G13" s="5" t="s">
@@ -4210,7 +4213,7 @@
       <c r="H13" s="5" t="s">
         <v>20</v>
       </c>
-      <c r="I13" s="36" t="s">
+      <c r="I13" s="37" t="s">
         <v>197</v>
       </c>
     </row>
@@ -4230,7 +4233,7 @@
       <c r="E14" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="F14" s="31" t="s">
+      <c r="F14" s="32" t="s">
         <v>18</v>
       </c>
       <c r="G14" s="5" t="s">
@@ -4239,7 +4242,7 @@
       <c r="H14" s="5" t="s">
         <v>20</v>
       </c>
-      <c r="I14" s="36" t="s">
+      <c r="I14" s="37" t="s">
         <v>198</v>
       </c>
     </row>
@@ -4259,7 +4262,7 @@
       <c r="E15" s="5" t="s">
         <v>50</v>
       </c>
-      <c r="F15" s="31" t="s">
+      <c r="F15" s="32" t="s">
         <v>199</v>
       </c>
       <c r="G15" s="5" t="s">
@@ -4268,7 +4271,7 @@
       <c r="H15" s="5" t="s">
         <v>20</v>
       </c>
-      <c r="I15" s="36" t="s">
+      <c r="I15" s="37" t="s">
         <v>200</v>
       </c>
     </row>
@@ -4288,7 +4291,7 @@
       <c r="E16" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="F16" s="31" t="s">
+      <c r="F16" s="32" t="s">
         <v>18</v>
       </c>
       <c r="G16" s="5" t="s">
@@ -4297,7 +4300,7 @@
       <c r="H16" s="5" t="s">
         <v>20</v>
       </c>
-      <c r="I16" s="36" t="s">
+      <c r="I16" s="37" t="s">
         <v>201</v>
       </c>
     </row>
@@ -4317,7 +4320,7 @@
       <c r="E17" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="F17" s="31" t="s">
+      <c r="F17" s="32" t="s">
         <v>194</v>
       </c>
       <c r="G17" s="5" t="s">
@@ -4326,7 +4329,7 @@
       <c r="H17" s="5" t="s">
         <v>20</v>
       </c>
-      <c r="I17" s="36" t="s">
+      <c r="I17" s="37" t="s">
         <v>202</v>
       </c>
     </row>
@@ -4346,7 +4349,7 @@
       <c r="E18" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="F18" s="31" t="s">
+      <c r="F18" s="32" t="s">
         <v>18</v>
       </c>
       <c r="G18" s="5" t="s">
@@ -4355,7 +4358,7 @@
       <c r="H18" s="5" t="s">
         <v>20</v>
       </c>
-      <c r="I18" s="36" t="s">
+      <c r="I18" s="37" t="s">
         <v>203</v>
       </c>
     </row>
@@ -4830,8 +4833,8 @@
       <c r="E18" s="5" t="s">
         <v>93</v>
       </c>
-      <c r="F18" s="25" t="s">
-        <v>63</v>
+      <c r="F18" s="26" t="s">
+        <v>18</v>
       </c>
       <c r="G18" s="5" t="s">
         <v>20</v>
@@ -4859,8 +4862,8 @@
       <c r="E19" s="5" t="s">
         <v>93</v>
       </c>
-      <c r="F19" s="25" t="s">
-        <v>63</v>
+      <c r="F19" s="26" t="s">
+        <v>18</v>
       </c>
       <c r="G19" s="5" t="s">
         <v>20</v>
@@ -5150,26 +5153,26 @@
       <c r="A30" s="23" t="s">
         <v>136</v>
       </c>
-      <c r="B30" s="26"/>
-      <c r="C30" s="26"/>
-      <c r="D30" s="26"/>
-      <c r="E30" s="26"/>
-      <c r="F30" s="26"/>
-      <c r="G30" s="26"/>
-      <c r="H30" s="26"/>
-      <c r="I30" s="28"/>
+      <c r="B30" s="27"/>
+      <c r="C30" s="27"/>
+      <c r="D30" s="27"/>
+      <c r="E30" s="27"/>
+      <c r="F30" s="27"/>
+      <c r="G30" s="27"/>
+      <c r="H30" s="27"/>
+      <c r="I30" s="29"/>
     </row>
     <row r="31" ht="28" customHeight="1" spans="1:9">
-      <c r="A31" s="27">
+      <c r="A31" s="28">
         <v>24</v>
       </c>
-      <c r="B31" s="27" t="s">
+      <c r="B31" s="28" t="s">
         <v>137</v>
       </c>
-      <c r="C31" s="27" t="s">
+      <c r="C31" s="28" t="s">
         <v>138</v>
       </c>
-      <c r="D31" s="27" t="s">
+      <c r="D31" s="28" t="s">
         <v>140</v>
       </c>
       <c r="E31" s="5" t="s">

</xml_diff>